<commit_message>
Datos Varin 2026-10-23 13:18
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -18749,7 +18749,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H117"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -18788,7 +18788,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>23-10-2026, 9:50:04 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B2" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18809,38 +18809,38 @@
         <v>48</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-23T12:50:04.195Z</v>
+        <v>2026-10-23T13:17:56.047Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B3" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C3" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-10-23T12:37:54.995Z</v>
+        <v>2026-10-23T13:17:56.044Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:52:55 a. m.</v>
       </c>
       <c r="B4" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18861,64 +18861,64 @@
         <v>48</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-10-23T12:37:54.994Z</v>
+        <v>2026-10-23T12:52:55.551Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:50:04 a. m.</v>
       </c>
       <c r="B5" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C5" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D5">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-10-23T12:37:54.992Z</v>
+        <v>2026-10-23T12:50:04.195Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>23-10-2026, 9:37:27 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B6" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C6" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D6">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-10-23T12:37:27.533Z</v>
+        <v>2026-10-23T12:37:54.995Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>23-10-2026, 9:34:31 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B7" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18939,64 +18939,64 @@
         <v>48</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-10-23T12:34:31.611Z</v>
+        <v>2026-10-23T12:37:54.994Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>23-10-2026, 9:19:14 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B8" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C8" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D8">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G8">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-10-23T12:19:14.833Z</v>
+        <v>2026-10-23T12:37:54.992Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:37:27 a. m.</v>
       </c>
       <c r="B9" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C9" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D9">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-10-22T11:51:13.535Z</v>
+        <v>2026-10-23T12:37:27.533Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:34:31 a. m.</v>
       </c>
       <c r="B10" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19017,38 +19017,38 @@
         <v>48</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-10-22T11:51:13.534Z</v>
+        <v>2026-10-23T12:34:31.611Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:19:14 a. m.</v>
       </c>
       <c r="B11" t="str">
-        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C11" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D11">
-        <v>134</v>
+        <v>48</v>
       </c>
       <c r="E11">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-10-22T11:51:13.529Z</v>
+        <v>2026-10-23T12:19:14.833Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B12" t="str">
         <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
@@ -19057,10 +19057,10 @@
         <v>Full ML · generado</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -19069,12 +19069,12 @@
         <v>2</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-10-21T11:58:09.619Z</v>
+        <v>2026-10-22T11:51:13.535Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B13" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19086,42 +19086,42 @@
         <v>48</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
       <c r="G13">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-10-21T11:58:09.618Z</v>
+        <v>2026-10-22T11:51:13.534Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B14" t="str">
-        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
+        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
       </c>
       <c r="C14" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D14">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F14">
         <v>5</v>
       </c>
       <c r="G14">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-10-21T11:58:09.614Z</v>
+        <v>2026-10-22T11:51:13.529Z</v>
       </c>
     </row>
     <row r="15">
@@ -19129,25 +19129,25 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B15" t="str">
-        <v>ventas-report (11).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C15" t="str">
-        <v>DropGO · ventas</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D15">
+        <v>4</v>
+      </c>
+      <c r="E15">
         <v>2</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-10-21T11:58:09.533Z</v>
+        <v>2026-10-21T11:58:09.619Z</v>
       </c>
     </row>
     <row r="16">
@@ -19155,13 +19155,13 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B16" t="str">
-        <v>picking-report (11).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C16" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -19170,50 +19170,50 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-10-21T11:58:09.530Z</v>
+        <v>2026-10-21T11:58:09.618Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B17" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
       </c>
       <c r="C17" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D17">
+        <v>128</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
         <v>5</v>
       </c>
-      <c r="E17">
-        <v>3</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
       <c r="G17">
-        <v>2</v>
+        <v>121</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.614Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B18" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (11).xlsx</v>
       </c>
       <c r="C18" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D18">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -19222,36 +19222,36 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.533Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B19" t="str">
-        <v>ventas-report (10).xlsx</v>
+        <v>picking-report (11).xlsx</v>
       </c>
       <c r="C19" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D19">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-10-20T12:36:20.899Z</v>
+        <v>2026-10-21T11:58:09.530Z</v>
       </c>
     </row>
     <row r="20">
@@ -19259,25 +19259,25 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B20" t="str">
-        <v>picking-report (10).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C20" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D20">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-10-20T12:36:20.895Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="21">
@@ -19285,212 +19285,212 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B21" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C21" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D21">
-        <v>126</v>
+        <v>47</v>
       </c>
       <c r="E21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>119</v>
+        <v>46</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-10-20T12:36:20.890Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>20-10-2026, 9:34:26 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B22" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (10).xlsx</v>
       </c>
       <c r="C22" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D22">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G22">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-20T12:34:26.210Z</v>
+        <v>2026-10-20T12:36:20.899Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B23" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (10).xlsx</v>
       </c>
       <c r="C23" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D23">
+        <v>11</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
+      </c>
+      <c r="G23">
         <v>7</v>
       </c>
-      <c r="E23">
-        <v>5</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>2</v>
-      </c>
       <c r="H23" t="str">
-        <v>2026-10-19T12:21:51.769Z</v>
+        <v>2026-10-20T12:36:20.895Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B24" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C24" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D24">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G24">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="H24" t="str">
-        <v>2026-10-19T12:21:51.768Z</v>
+        <v>2026-10-20T12:36:20.890Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:34:26 a. m.</v>
       </c>
       <c r="B25" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C25" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D25">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E25">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-10-19T12:21:51.766Z</v>
+        <v>2026-10-20T12:34:26.210Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B26" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C26" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D26">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E26">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H26" t="str">
-        <v>2026-10-19T12:20:51.921Z</v>
+        <v>2026-10-19T12:21:51.769Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B27" t="str">
-        <v>picking-report (9).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C27" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D27">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E27">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-10-19T12:20:51.919Z</v>
+        <v>2026-10-19T12:21:51.768Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B28" t="str">
-        <v>ventas-report (9).xlsx</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
       </c>
       <c r="C28" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D28">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="E28">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-10-19T12:20:51.913Z</v>
+        <v>2026-10-19T12:21:51.766Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>19-10-2026, 9:12:06 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B29" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19499,10 +19499,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D29">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F29">
         <v>0</v>
@@ -19511,229 +19511,229 @@
         <v>37</v>
       </c>
       <c r="H29" t="str">
-        <v>2026-10-19T12:12:06.575Z</v>
+        <v>2026-10-19T12:20:51.921Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B30" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (9).xlsx</v>
       </c>
       <c r="C30" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D30">
+        <v>14</v>
+      </c>
+      <c r="E30">
+        <v>7</v>
+      </c>
+      <c r="F30">
         <v>5</v>
-      </c>
-      <c r="E30">
-        <v>3</v>
-      </c>
-      <c r="F30">
-        <v>0</v>
       </c>
       <c r="G30">
         <v>2</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-10-16T12:37:12.832Z</v>
+        <v>2026-10-19T12:20:51.919Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B31" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (9).xlsx</v>
       </c>
       <c r="C31" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D31">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G31">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-10-16T12:37:12.831Z</v>
+        <v>2026-10-19T12:20:51.913Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:12:06 a. m.</v>
       </c>
       <c r="B32" t="str">
-        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C32" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D32">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E32">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G32">
         <v>37</v>
       </c>
       <c r="H32" t="str">
-        <v>2026-10-16T12:37:12.827Z</v>
+        <v>2026-10-19T12:12:06.575Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B33" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C33" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D33">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-10-16T11:52:26.043Z</v>
+        <v>2026-10-16T12:37:12.832Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B34" t="str">
-        <v>picking-report (8).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C34" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D34">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E34">
         <v>0</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H34" t="str">
-        <v>2026-10-16T11:52:26.040Z</v>
+        <v>2026-10-16T12:37:12.831Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B35" t="str">
-        <v>ventas-report (8).xlsx</v>
+        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
       </c>
       <c r="C35" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G35">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H35" t="str">
-        <v>2026-10-16T11:52:26.034Z</v>
+        <v>2026-10-16T12:37:12.827Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B36" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C36" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D36">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-10-15T12:11:36.404Z</v>
+        <v>2026-10-16T11:52:26.043Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B37" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (8).xlsx</v>
       </c>
       <c r="C37" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D37">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E37">
         <v>0</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H37" t="str">
-        <v>2026-10-15T12:11:36.403Z</v>
+        <v>2026-10-16T11:52:26.040Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B38" t="str">
-        <v>ventas-report (7).xlsx</v>
+        <v>ventas-report (8).xlsx</v>
       </c>
       <c r="C38" t="str">
         <v>DropGO · ventas</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E38">
         <v>0</v>
@@ -19742,10 +19742,10 @@
         <v>1</v>
       </c>
       <c r="G38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H38" t="str">
-        <v>2026-10-15T12:11:36.401Z</v>
+        <v>2026-10-16T11:52:26.034Z</v>
       </c>
     </row>
     <row r="39">
@@ -19753,25 +19753,25 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B39" t="str">
-        <v>picking-report (7).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C39" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39">
+        <v>2</v>
+      </c>
+      <c r="F39">
         <v>0</v>
-      </c>
-      <c r="F39">
-        <v>1</v>
       </c>
       <c r="G39">
         <v>2</v>
       </c>
       <c r="H39" t="str">
-        <v>2026-10-15T12:11:36.397Z</v>
+        <v>2026-10-15T12:11:36.404Z</v>
       </c>
     </row>
     <row r="40">
@@ -19779,143 +19779,143 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B40" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C40" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D40">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F40">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G40">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="H40" t="str">
-        <v>2026-10-15T12:11:36.389Z</v>
+        <v>2026-10-15T12:11:36.403Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>14-10-2026, 10:42:32 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B41" t="str">
-        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
+        <v>ventas-report (7).xlsx</v>
       </c>
       <c r="C41" t="str">
-        <v>Manual</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E41">
         <v>0</v>
       </c>
       <c r="F41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H41" t="str">
-        <v>2026-10-14T13:42:32.444Z</v>
+        <v>2026-10-15T12:11:36.401Z</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B42" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (7).xlsx</v>
       </c>
       <c r="C42" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D42">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
         <v>2</v>
       </c>
-      <c r="F42">
-        <v>0</v>
-      </c>
-      <c r="G42">
-        <v>35</v>
-      </c>
       <c r="H42" t="str">
-        <v>2026-10-14T13:41:21.926Z</v>
+        <v>2026-10-15T12:11:36.397Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B43" t="str">
-        <v>picking-report (6).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
       </c>
       <c r="C43" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D43">
-        <v>7</v>
+        <v>114</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G43">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="H43" t="str">
-        <v>2026-10-14T13:41:21.925Z</v>
+        <v>2026-10-15T12:11:36.389Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>14-10-2026, 10:42:32 a. m.</v>
       </c>
       <c r="B44" t="str">
-        <v>ventas-report (6).xlsx</v>
+        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
       </c>
       <c r="C44" t="str">
-        <v>DropGO · ventas</v>
+        <v>Manual</v>
       </c>
       <c r="D44">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F44">
         <v>0</v>
       </c>
       <c r="G44">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H44" t="str">
-        <v>2026-10-14T13:41:21.921Z</v>
+        <v>2026-10-14T13:42:32.444Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B45" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C45" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D45">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E45">
         <v>2</v>
@@ -19924,93 +19924,93 @@
         <v>0</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="H45" t="str">
-        <v>2026-10-14T13:40:03.191Z</v>
+        <v>2026-10-14T13:41:21.926Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B46" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (6).xlsx</v>
       </c>
       <c r="C46" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D46">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F46">
         <v>0</v>
       </c>
       <c r="G46">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H46" t="str">
-        <v>2026-10-14T13:40:03.190Z</v>
+        <v>2026-10-14T13:41:21.925Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B47" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
+        <v>ventas-report (6).xlsx</v>
       </c>
       <c r="C47" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D47">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="E47">
         <v>3</v>
       </c>
       <c r="F47">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G47">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-10-14T13:40:03.188Z</v>
+        <v>2026-10-14T13:41:21.921Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>14-10-2026, 10:39:50 a. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B48" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C48" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D48">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F48">
         <v>0</v>
       </c>
       <c r="G48">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H48" t="str">
-        <v>2026-10-14T13:39:50.407Z</v>
+        <v>2026-10-14T13:40:03.191Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B49" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20031,38 +20031,38 @@
         <v>35</v>
       </c>
       <c r="H49" t="str">
-        <v>2026-10-13T16:19:36.490Z</v>
+        <v>2026-10-14T13:40:03.190Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B50" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
       </c>
       <c r="C50" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D50">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G50">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H50" t="str">
-        <v>2026-10-13T16:19:36.488Z</v>
+        <v>2026-10-14T13:40:03.188Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>13-10-2026, 11:56:40 a. m.</v>
+        <v>14-10-2026, 10:39:50 a. m.</v>
       </c>
       <c r="B51" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20083,12 +20083,12 @@
         <v>35</v>
       </c>
       <c r="H51" t="str">
-        <v>2026-10-13T14:56:40.589Z</v>
+        <v>2026-10-14T13:39:50.407Z</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B52" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20100,177 +20100,177 @@
         <v>35</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G52">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H52" t="str">
-        <v>2026-10-13T14:44:42.285Z</v>
+        <v>2026-10-13T16:19:36.490Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B53" t="str">
-        <v>picking-report (5).xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C53" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D53">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G53">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="H53" t="str">
-        <v>2026-10-13T14:44:42.284Z</v>
+        <v>2026-10-13T16:19:36.488Z</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 11:56:40 a. m.</v>
       </c>
       <c r="B54" t="str">
-        <v>ventas-report (5).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C54" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D54">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F54">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H54" t="str">
-        <v>2026-10-13T14:44:42.280Z</v>
+        <v>2026-10-13T14:56:40.589Z</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B55" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C55" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D55">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="E55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G55">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H55" t="str">
-        <v>2026-10-13T12:49:30.632Z</v>
+        <v>2026-10-13T14:44:42.285Z</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B56" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (5).xlsx</v>
       </c>
       <c r="C56" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D56">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E56">
+        <v>2</v>
+      </c>
+      <c r="F56">
+        <v>6</v>
+      </c>
+      <c r="G56">
         <v>0</v>
       </c>
-      <c r="F56">
-        <v>0</v>
-      </c>
-      <c r="G56">
-        <v>34</v>
-      </c>
       <c r="H56" t="str">
-        <v>2026-10-13T12:49:30.631Z</v>
+        <v>2026-10-13T14:44:42.284Z</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B57" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>ventas-report (5).xlsx</v>
       </c>
       <c r="C57" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D57">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="E57">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F57">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G57">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H57" t="str">
-        <v>2026-10-13T12:49:30.629Z</v>
+        <v>2026-10-13T14:44:42.280Z</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>13-10-2026, 9:08:58 a. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B58" t="str">
-        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C58" t="str">
-        <v>Manual</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E58">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F58">
         <v>0</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-13T12:08:58.547Z</v>
+        <v>2026-10-13T12:49:30.632Z</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B59" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20291,116 +20291,116 @@
         <v>34</v>
       </c>
       <c r="H59" t="str">
-        <v>2026-10-12T18:40:27.007Z</v>
+        <v>2026-10-13T12:49:30.631Z</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B60" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C60" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D60">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E60">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F60">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G60">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H60" t="str">
-        <v>2026-10-12T18:40:27.006Z</v>
+        <v>2026-10-13T12:49:30.629Z</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>13-10-2026, 9:08:58 a. m.</v>
       </c>
       <c r="B61" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
       </c>
       <c r="C61" t="str">
-        <v>DropGO · generado</v>
+        <v>Manual</v>
       </c>
       <c r="D61">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E61">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F61">
         <v>0</v>
       </c>
       <c r="G61">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H61" t="str">
-        <v>2026-10-12T18:39:34.326Z</v>
+        <v>2026-10-13T12:08:58.547Z</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B62" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C62" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D62">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E62">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F62">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G62">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H62" t="str">
-        <v>2026-10-12T18:39:34.325Z</v>
+        <v>2026-10-12T18:40:27.007Z</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B63" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C63" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D63">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E63">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F63">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G63">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H63" t="str">
-        <v>2026-10-12T18:39:34.319Z</v>
+        <v>2026-10-12T18:40:27.006Z</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>12-10-2026, 3:39:18 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B64" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20409,10 +20409,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D64">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F64">
         <v>0</v>
@@ -20421,116 +20421,116 @@
         <v>25</v>
       </c>
       <c r="H64" t="str">
-        <v>2026-10-12T18:39:18.385Z</v>
+        <v>2026-10-12T18:39:34.326Z</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>12-10-2026, 12:05:40 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B65" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C65" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D65">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F65">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G65">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H65" t="str">
-        <v>2026-10-12T15:05:40.188Z</v>
+        <v>2026-10-12T18:39:34.325Z</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B66" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C66" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D66">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F66">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G66">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H66" t="str">
-        <v>2026-10-12T14:26:19.514Z</v>
+        <v>2026-10-12T18:39:34.319Z</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:18 p. m.</v>
       </c>
       <c r="B67" t="str">
-        <v>orders_export (6).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C67" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D67">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E67">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F67">
         <v>0</v>
       </c>
       <c r="G67">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H67" t="str">
-        <v>2026-10-12T14:26:19.513Z</v>
+        <v>2026-10-12T18:39:18.385Z</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 12:05:40 p. m.</v>
       </c>
       <c r="B68" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C68" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F68">
         <v>0</v>
       </c>
       <c r="G68">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H68" t="str">
-        <v>2026-10-12T14:24:55.059Z</v>
+        <v>2026-10-12T15:05:40.188Z</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B69" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20551,64 +20551,64 @@
         <v>25</v>
       </c>
       <c r="H69" t="str">
-        <v>2026-10-12T14:24:55.058Z</v>
+        <v>2026-10-12T14:26:19.514Z</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B70" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>orders_export (6).csv</v>
       </c>
       <c r="C70" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D70">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E70">
         <v>4</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G70">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H70" t="str">
-        <v>2026-10-12T14:24:55.057Z</v>
+        <v>2026-10-12T14:26:19.513Z</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>12-10-2026, 11:24:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B71" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C71" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D71">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F71">
         <v>0</v>
       </c>
       <c r="G71">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-10-12T14:24:00.106Z</v>
+        <v>2026-10-12T14:24:55.059Z</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B72" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20620,73 +20620,73 @@
         <v>25</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H72" t="str">
-        <v>2026-10-09T14:54:00.353Z</v>
+        <v>2026-10-12T14:24:55.058Z</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B73" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C73" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D73">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E73">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H73" t="str">
-        <v>2026-10-09T14:54:00.352Z</v>
+        <v>2026-10-12T14:24:55.057Z</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:00 a. m.</v>
       </c>
       <c r="B74" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C74" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D74">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E74">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F74">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H74" t="str">
-        <v>2026-10-09T14:54:00.347Z</v>
+        <v>2026-10-12T14:24:00.106Z</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>09-10-2026, 11:50:59 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B75" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20695,10 +20695,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D75">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E75">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -20707,64 +20707,64 @@
         <v>21</v>
       </c>
       <c r="H75" t="str">
-        <v>2026-10-09T14:50:59.695Z</v>
+        <v>2026-10-09T14:54:00.353Z</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B76" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C76" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D76">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E76">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G76">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H76" t="str">
-        <v>2026-10-09T14:28:16.404Z</v>
+        <v>2026-10-09T14:54:00.352Z</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B77" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C77" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D77">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E77">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H77" t="str">
-        <v>2026-10-09T14:28:16.403Z</v>
+        <v>2026-10-09T14:54:00.347Z</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>09-10-2026, 11:28:07 a. m.</v>
+        <v>09-10-2026, 11:50:59 a. m.</v>
       </c>
       <c r="B78" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20785,12 +20785,12 @@
         <v>21</v>
       </c>
       <c r="H78" t="str">
-        <v>2026-10-09T14:28:07.531Z</v>
+        <v>2026-10-09T14:50:59.695Z</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B79" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20811,12 +20811,12 @@
         <v>21</v>
       </c>
       <c r="H79" t="str">
-        <v>2026-10-09T14:26:45.497Z</v>
+        <v>2026-10-09T14:28:16.404Z</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B80" t="str">
         <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
@@ -20837,21 +20837,21 @@
         <v>19</v>
       </c>
       <c r="H80" t="str">
-        <v>2026-10-09T14:26:45.495Z</v>
+        <v>2026-10-09T14:28:16.403Z</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:07 a. m.</v>
       </c>
       <c r="B81" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C81" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D81">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E81">
         <v>0</v>
@@ -20860,50 +20860,50 @@
         <v>0</v>
       </c>
       <c r="G81">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H81" t="str">
-        <v>2026-10-09T14:26:45.477Z</v>
+        <v>2026-10-09T14:28:07.531Z</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B82" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C82" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D82">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F82">
         <v>0</v>
       </c>
       <c r="G82">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H82" t="str">
-        <v>2026-10-09T14:25:43.607Z</v>
+        <v>2026-10-09T14:26:45.497Z</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B83" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C83" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D83">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E83">
         <v>0</v>
@@ -20912,36 +20912,36 @@
         <v>0</v>
       </c>
       <c r="G83">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H83" t="str">
-        <v>2026-10-09T14:25:43.606Z</v>
+        <v>2026-10-09T14:26:45.495Z</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B84" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C84" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D84">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E84">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F84">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G84">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H84" t="str">
-        <v>2026-10-09T14:25:43.605Z</v>
+        <v>2026-10-09T14:26:45.477Z</v>
       </c>
     </row>
     <row r="85">
@@ -20949,30 +20949,30 @@
         <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B85" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C85" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D85">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E85">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F85">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G85">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H85" t="str">
-        <v>2026-10-09T14:25:43.580Z</v>
+        <v>2026-10-09T14:25:43.607Z</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>09-10-2026, 11:23:53 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B86" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20993,111 +20993,111 @@
         <v>21</v>
       </c>
       <c r="H86" t="str">
-        <v>2026-10-09T14:23:53.263Z</v>
+        <v>2026-10-09T14:25:43.606Z</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>08-10-2026, 9:14:25 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B87" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C87" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D87">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E87">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F87">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G87">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H87" t="str">
-        <v>2026-10-08T12:14:25.917Z</v>
+        <v>2026-10-09T14:25:43.605Z</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B88" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C88" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D88">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F88">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H88" t="str">
-        <v>2026-10-08T11:22:18.060Z</v>
+        <v>2026-10-09T14:25:43.580Z</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:23:53 a. m.</v>
       </c>
       <c r="B89" t="str">
-        <v>orders_export (4).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C89" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D89">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E89">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F89">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G89">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H89" t="str">
-        <v>2026-10-08T11:22:18.059Z</v>
+        <v>2026-10-09T14:23:53.263Z</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>08-10-2026, 9:14:25 a. m.</v>
       </c>
       <c r="B90" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C90" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D90">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E90">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F90">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G90">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H90" t="str">
-        <v>2026-10-08T11:22:18.042Z</v>
+        <v>2026-10-08T12:14:25.917Z</v>
       </c>
     </row>
     <row r="91">
@@ -21105,108 +21105,108 @@
         <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B91" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C91" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D91">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E91">
         <v>2</v>
       </c>
       <c r="F91">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G91">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H91" t="str">
-        <v>2026-10-08T11:22:18.032Z</v>
+        <v>2026-10-08T11:22:18.060Z</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>08-10-2026, 8:18:16 a. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B92" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (4).csv</v>
       </c>
       <c r="C92" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D92">
         <v>19</v>
       </c>
       <c r="E92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F92">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G92">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H92" t="str">
-        <v>2026-10-08T11:18:16.488Z</v>
+        <v>2026-10-08T11:22:18.059Z</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B93" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C93" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D93">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E93">
+        <v>2</v>
+      </c>
+      <c r="F93">
+        <v>1</v>
+      </c>
+      <c r="G93">
         <v>0</v>
       </c>
-      <c r="F93">
-        <v>0</v>
-      </c>
-      <c r="G93">
-        <v>19</v>
-      </c>
       <c r="H93" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.042Z</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B94" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C94" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D94">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E94">
         <v>2</v>
       </c>
       <c r="F94">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G94">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H94" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.032Z</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>07-10-2026, 8:20:41 p. m.</v>
+        <v>08-10-2026, 8:18:16 a. m.</v>
       </c>
       <c r="B95" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21227,12 +21227,12 @@
         <v>19</v>
       </c>
       <c r="H95" t="str">
-        <v>2026-10-07T23:20:41.390Z</v>
+        <v>2026-10-08T11:18:16.488Z</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B96" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21253,38 +21253,38 @@
         <v>19</v>
       </c>
       <c r="H96" t="str">
-        <v>2026-10-07T17:47:17.199Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B97" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
       </c>
       <c r="C97" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D97">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F97">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G97">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H97" t="str">
-        <v>2026-10-07T17:47:17.198Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>07-10-2026, 2:46:47 p. m.</v>
+        <v>07-10-2026, 8:20:41 p. m.</v>
       </c>
       <c r="B98" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21305,12 +21305,12 @@
         <v>19</v>
       </c>
       <c r="H98" t="str">
-        <v>2026-10-07T17:46:47.954Z</v>
+        <v>2026-10-07T23:20:41.390Z</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>07-10-2026, 2:44:00 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B99" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21331,64 +21331,64 @@
         <v>19</v>
       </c>
       <c r="H99" t="str">
-        <v>2026-10-07T17:44:00.660Z</v>
+        <v>2026-10-07T17:47:17.199Z</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>07-10-2026, 2:27:43 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B100" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
       </c>
       <c r="C100" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D100">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E100">
         <v>0</v>
       </c>
       <c r="F100">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G100">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="H100" t="str">
-        <v>2026-10-07T17:27:43.517Z</v>
+        <v>2026-10-07T17:47:17.198Z</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:46:47 p. m.</v>
       </c>
       <c r="B101" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C101" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D101">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E101">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F101">
         <v>0</v>
       </c>
       <c r="G101">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H101" t="str">
-        <v>2026-10-07T17:26:50.382Z</v>
+        <v>2026-10-07T17:46:47.954Z</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:44:00 p. m.</v>
       </c>
       <c r="B102" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21400,21 +21400,21 @@
         <v>19</v>
       </c>
       <c r="E102">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F102">
         <v>0</v>
       </c>
       <c r="G102">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H102" t="str">
-        <v>2026-10-07T17:26:50.380Z</v>
+        <v>2026-10-07T17:44:00.660Z</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:27:43 p. m.</v>
       </c>
       <c r="B103" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21423,7 +21423,7 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D103">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E103">
         <v>0</v>
@@ -21432,41 +21432,41 @@
         <v>0</v>
       </c>
       <c r="G103">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H103" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:27:43.517Z</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B104" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C104" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D104">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="E104">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F104">
         <v>0</v>
       </c>
       <c r="G104">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:26:50.382Z</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B105" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21475,71 +21475,71 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D105">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E105">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F105">
         <v>0</v>
       </c>
       <c r="G105">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H105" t="str">
-        <v>2026-10-07T16:25:12.953Z</v>
+        <v>2026-10-07T17:26:50.380Z</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B106" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C106" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D106">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E106">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F106">
         <v>0</v>
       </c>
       <c r="G106">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H106" t="str">
-        <v>2026-10-07T16:25:12.950Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B107" t="str">
-        <v>orders_export (3).csv</v>
+        <v>ventas_por_canal_y_mes.xlsx</v>
       </c>
       <c r="C107" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Ventas por canal y mes</v>
       </c>
       <c r="D107">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="E107">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F107">
         <v>0</v>
       </c>
       <c r="G107">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="H107" t="str">
-        <v>2026-10-07T16:25:12.939Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="108">
@@ -21547,25 +21547,25 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B108" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C108" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D108">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-10-07T16:25:12.924Z</v>
+        <v>2026-10-07T16:25:12.953Z</v>
       </c>
     </row>
     <row r="109">
@@ -21573,10 +21573,10 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B109" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C109" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D109">
         <v>19</v>
@@ -21591,142 +21591,220 @@
         <v>0</v>
       </c>
       <c r="H109" t="str">
-        <v>2026-10-07T16:25:12.851Z</v>
+        <v>2026-10-07T16:25:12.950Z</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>07-10-2026, 1:10:27 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B110" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>orders_export (3).csv</v>
       </c>
       <c r="C110" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D110">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F110">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G110">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="H110" t="str">
-        <v>2026-10-07T16:10:27.561Z</v>
+        <v>2026-10-07T16:25:12.939Z</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>07-10-2026, 12:20:36 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B111" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C111" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D111">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F111">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G111">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H111" t="str">
-        <v>2026-10-07T15:20:36.001Z</v>
+        <v>2026-10-07T16:25:12.924Z</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>07-10-2026, 12:20:35 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B112" t="str">
-        <v>varin_respaldo_2026-10-07.xlsx</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C112" t="str">
-        <v>Respaldo</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D112">
-        <v>322</v>
+        <v>19</v>
       </c>
       <c r="E112">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F112">
         <v>0</v>
       </c>
       <c r="G112">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H112" t="str">
-        <v>2026-10-07T15:20:35.967Z</v>
+        <v>2026-10-07T16:25:12.851Z</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>07-10-2026, 12:20:08 p. m.</v>
+        <v>07-10-2026, 1:10:27 p. m.</v>
       </c>
       <c r="B113" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C113" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D113">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E113">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="F113">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G113">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="H113" t="str">
-        <v>2026-10-07T15:20:08.547Z</v>
+        <v>2026-10-07T16:10:27.561Z</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
+        <v>07-10-2026, 12:20:36 p. m.</v>
+      </c>
+      <c r="B114" t="str">
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Ventas Mercado Libre</v>
+      </c>
+      <c r="D114">
+        <v>92</v>
+      </c>
+      <c r="E114">
+        <v>1</v>
+      </c>
+      <c r="F114">
+        <v>5</v>
+      </c>
+      <c r="G114">
+        <v>86</v>
+      </c>
+      <c r="H114" t="str">
+        <v>2026-10-07T15:20:36.001Z</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>07-10-2026, 12:20:35 p. m.</v>
+      </c>
+      <c r="B115" t="str">
+        <v>varin_respaldo_2026-10-07.xlsx</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Respaldo</v>
+      </c>
+      <c r="D115">
+        <v>322</v>
+      </c>
+      <c r="E115">
+        <v>190</v>
+      </c>
+      <c r="F115">
+        <v>0</v>
+      </c>
+      <c r="G115">
+        <v>132</v>
+      </c>
+      <c r="H115" t="str">
+        <v>2026-10-07T15:20:35.967Z</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
         <v>07-10-2026, 12:20:08 p. m.</v>
       </c>
-      <c r="B114" t="str">
+      <c r="B116" t="str">
+        <v>ventas_por_canal_y_mes.xlsx</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Ventas por canal y mes</v>
+      </c>
+      <c r="D116">
+        <v>118</v>
+      </c>
+      <c r="E116">
+        <v>118</v>
+      </c>
+      <c r="F116">
+        <v>0</v>
+      </c>
+      <c r="G116">
+        <v>0</v>
+      </c>
+      <c r="H116" t="str">
+        <v>2026-10-07T15:20:08.547Z</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>07-10-2026, 12:20:08 p. m.</v>
+      </c>
+      <c r="B117" t="str">
         <v>Varin_Movimientos_DropGO_2026-10-01_al_2026-10-06.xlsx</v>
       </c>
-      <c r="C114" t="str">
+      <c r="C117" t="str">
         <v>Movimientos DropGO</v>
       </c>
-      <c r="D114">
+      <c r="D117">
         <v>14</v>
       </c>
-      <c r="E114">
+      <c r="E117">
         <v>14</v>
       </c>
-      <c r="F114">
+      <c r="F117">
         <v>0</v>
       </c>
-      <c r="G114">
+      <c r="G117">
         <v>0</v>
       </c>
-      <c r="H114" t="str">
+      <c r="H117" t="str">
         <v>2026-10-07T15:20:08.525Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H114"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H117"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -25054,7 +25132,7 @@
         <v>Generado</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-23T12:52:00.578Z</v>
+        <v>2026-10-23T13:18:00.704Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Datos Varin 2026-10-23 22:12
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -18749,7 +18749,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H120"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -18788,7 +18788,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B2" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18809,15 +18809,15 @@
         <v>48</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-23T13:17:56.047Z</v>
+        <v>2026-10-23T22:12:12.477Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B3" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C3" t="str">
         <v>Ventas Mercado Libre</v>
@@ -18835,12 +18835,12 @@
         <v>135</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-10-23T13:17:56.044Z</v>
+        <v>2026-10-23T22:12:12.476Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>23-10-2026, 9:52:55 a. m.</v>
+        <v>23-10-2026, 7:11:53 p. m.</v>
       </c>
       <c r="B4" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18861,12 +18861,12 @@
         <v>48</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-10-23T12:52:55.551Z</v>
+        <v>2026-10-23T22:11:53.140Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>23-10-2026, 9:50:04 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B5" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18887,38 +18887,38 @@
         <v>48</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-10-23T12:50:04.195Z</v>
+        <v>2026-10-23T13:17:56.047Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B6" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C6" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-10-23T12:37:54.995Z</v>
+        <v>2026-10-23T13:17:56.044Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:52:55 a. m.</v>
       </c>
       <c r="B7" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -18939,64 +18939,64 @@
         <v>48</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-10-23T12:37:54.994Z</v>
+        <v>2026-10-23T12:52:55.551Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:50:04 a. m.</v>
       </c>
       <c r="B8" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C8" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D8">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-10-23T12:37:54.992Z</v>
+        <v>2026-10-23T12:50:04.195Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>23-10-2026, 9:37:27 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B9" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C9" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D9">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-10-23T12:37:27.533Z</v>
+        <v>2026-10-23T12:37:54.995Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>23-10-2026, 9:34:31 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B10" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19017,64 +19017,64 @@
         <v>48</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-10-23T12:34:31.611Z</v>
+        <v>2026-10-23T12:37:54.994Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>23-10-2026, 9:19:14 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B11" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C11" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D11">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G11">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-10-23T12:19:14.833Z</v>
+        <v>2026-10-23T12:37:54.992Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:37:27 a. m.</v>
       </c>
       <c r="B12" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C12" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E12">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-10-22T11:51:13.535Z</v>
+        <v>2026-10-23T12:37:27.533Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:34:31 a. m.</v>
       </c>
       <c r="B13" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19095,38 +19095,38 @@
         <v>48</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-10-22T11:51:13.534Z</v>
+        <v>2026-10-23T12:34:31.611Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:19:14 a. m.</v>
       </c>
       <c r="B14" t="str">
-        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C14" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D14">
-        <v>134</v>
+        <v>48</v>
       </c>
       <c r="E14">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-10-22T11:51:13.529Z</v>
+        <v>2026-10-23T12:19:14.833Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B15" t="str">
         <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
@@ -19135,10 +19135,10 @@
         <v>Full ML · generado</v>
       </c>
       <c r="D15">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -19147,12 +19147,12 @@
         <v>2</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-10-21T11:58:09.619Z</v>
+        <v>2026-10-22T11:51:13.535Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B16" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19164,42 +19164,42 @@
         <v>48</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
       </c>
       <c r="G16">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-10-21T11:58:09.618Z</v>
+        <v>2026-10-22T11:51:13.534Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B17" t="str">
-        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
+        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
       </c>
       <c r="C17" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D17">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F17">
         <v>5</v>
       </c>
       <c r="G17">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-10-21T11:58:09.614Z</v>
+        <v>2026-10-22T11:51:13.529Z</v>
       </c>
     </row>
     <row r="18">
@@ -19207,25 +19207,25 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B18" t="str">
-        <v>ventas-report (11).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C18" t="str">
-        <v>DropGO · ventas</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D18">
+        <v>4</v>
+      </c>
+      <c r="E18">
         <v>2</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-10-21T11:58:09.533Z</v>
+        <v>2026-10-21T11:58:09.619Z</v>
       </c>
     </row>
     <row r="19">
@@ -19233,13 +19233,13 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B19" t="str">
-        <v>picking-report (11).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C19" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -19248,50 +19248,50 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-10-21T11:58:09.530Z</v>
+        <v>2026-10-21T11:58:09.618Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B20" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
       </c>
       <c r="C20" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D20">
+        <v>128</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
         <v>5</v>
       </c>
-      <c r="E20">
-        <v>3</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
       <c r="G20">
-        <v>2</v>
+        <v>121</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.614Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B21" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (11).xlsx</v>
       </c>
       <c r="C21" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D21">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -19300,36 +19300,36 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.533Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B22" t="str">
-        <v>ventas-report (10).xlsx</v>
+        <v>picking-report (11).xlsx</v>
       </c>
       <c r="C22" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D22">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-20T12:36:20.899Z</v>
+        <v>2026-10-21T11:58:09.530Z</v>
       </c>
     </row>
     <row r="23">
@@ -19337,25 +19337,25 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B23" t="str">
-        <v>picking-report (10).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C23" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D23">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H23" t="str">
-        <v>2026-10-20T12:36:20.895Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="24">
@@ -19363,212 +19363,212 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B24" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C24" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D24">
-        <v>126</v>
+        <v>47</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F24">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>119</v>
+        <v>46</v>
       </c>
       <c r="H24" t="str">
-        <v>2026-10-20T12:36:20.890Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>20-10-2026, 9:34:26 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B25" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (10).xlsx</v>
       </c>
       <c r="C25" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D25">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G25">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-10-20T12:34:26.210Z</v>
+        <v>2026-10-20T12:36:20.899Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B26" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (10).xlsx</v>
       </c>
       <c r="C26" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D26">
+        <v>11</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>3</v>
+      </c>
+      <c r="G26">
         <v>7</v>
       </c>
-      <c r="E26">
-        <v>5</v>
-      </c>
-      <c r="F26">
-        <v>1</v>
-      </c>
-      <c r="G26">
-        <v>2</v>
-      </c>
       <c r="H26" t="str">
-        <v>2026-10-19T12:21:51.769Z</v>
+        <v>2026-10-20T12:36:20.895Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B27" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C27" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D27">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G27">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-10-19T12:21:51.768Z</v>
+        <v>2026-10-20T12:36:20.890Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:34:26 a. m.</v>
       </c>
       <c r="B28" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C28" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D28">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E28">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F28">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-10-19T12:21:51.766Z</v>
+        <v>2026-10-20T12:34:26.210Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B29" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C29" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D29">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E29">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H29" t="str">
-        <v>2026-10-19T12:20:51.921Z</v>
+        <v>2026-10-19T12:21:51.769Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B30" t="str">
-        <v>picking-report (9).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C30" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D30">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E30">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-10-19T12:20:51.919Z</v>
+        <v>2026-10-19T12:21:51.768Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B31" t="str">
-        <v>ventas-report (9).xlsx</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
       </c>
       <c r="C31" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D31">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="E31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-10-19T12:20:51.913Z</v>
+        <v>2026-10-19T12:21:51.766Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>19-10-2026, 9:12:06 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B32" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19577,10 +19577,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D32">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -19589,229 +19589,229 @@
         <v>37</v>
       </c>
       <c r="H32" t="str">
-        <v>2026-10-19T12:12:06.575Z</v>
+        <v>2026-10-19T12:20:51.921Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B33" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (9).xlsx</v>
       </c>
       <c r="C33" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D33">
+        <v>14</v>
+      </c>
+      <c r="E33">
+        <v>7</v>
+      </c>
+      <c r="F33">
         <v>5</v>
-      </c>
-      <c r="E33">
-        <v>3</v>
-      </c>
-      <c r="F33">
-        <v>0</v>
       </c>
       <c r="G33">
         <v>2</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-10-16T12:37:12.832Z</v>
+        <v>2026-10-19T12:20:51.919Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B34" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (9).xlsx</v>
       </c>
       <c r="C34" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D34">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H34" t="str">
-        <v>2026-10-16T12:37:12.831Z</v>
+        <v>2026-10-19T12:20:51.913Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:12:06 a. m.</v>
       </c>
       <c r="B35" t="str">
-        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C35" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D35">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E35">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F35">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G35">
         <v>37</v>
       </c>
       <c r="H35" t="str">
-        <v>2026-10-16T12:37:12.827Z</v>
+        <v>2026-10-19T12:12:06.575Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B36" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C36" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D36">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-10-16T11:52:26.043Z</v>
+        <v>2026-10-16T12:37:12.832Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B37" t="str">
-        <v>picking-report (8).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C37" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E37">
         <v>0</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H37" t="str">
-        <v>2026-10-16T11:52:26.040Z</v>
+        <v>2026-10-16T12:37:12.831Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B38" t="str">
-        <v>ventas-report (8).xlsx</v>
+        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
       </c>
       <c r="C38" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D38">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F38">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H38" t="str">
-        <v>2026-10-16T11:52:26.034Z</v>
+        <v>2026-10-16T12:37:12.827Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B39" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C39" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D39">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H39" t="str">
-        <v>2026-10-15T12:11:36.404Z</v>
+        <v>2026-10-16T11:52:26.043Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B40" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (8).xlsx</v>
       </c>
       <c r="C40" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D40">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E40">
         <v>0</v>
       </c>
       <c r="F40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H40" t="str">
-        <v>2026-10-15T12:11:36.403Z</v>
+        <v>2026-10-16T11:52:26.040Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B41" t="str">
-        <v>ventas-report (7).xlsx</v>
+        <v>ventas-report (8).xlsx</v>
       </c>
       <c r="C41" t="str">
         <v>DropGO · ventas</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -19820,10 +19820,10 @@
         <v>1</v>
       </c>
       <c r="G41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H41" t="str">
-        <v>2026-10-15T12:11:36.401Z</v>
+        <v>2026-10-16T11:52:26.034Z</v>
       </c>
     </row>
     <row r="42">
@@ -19831,25 +19831,25 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B42" t="str">
-        <v>picking-report (7).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C42" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D42">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
         <v>0</v>
-      </c>
-      <c r="F42">
-        <v>1</v>
       </c>
       <c r="G42">
         <v>2</v>
       </c>
       <c r="H42" t="str">
-        <v>2026-10-15T12:11:36.397Z</v>
+        <v>2026-10-15T12:11:36.404Z</v>
       </c>
     </row>
     <row r="43">
@@ -19857,143 +19857,143 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B43" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C43" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D43">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F43">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G43">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="H43" t="str">
-        <v>2026-10-15T12:11:36.389Z</v>
+        <v>2026-10-15T12:11:36.403Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>14-10-2026, 10:42:32 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B44" t="str">
-        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
+        <v>ventas-report (7).xlsx</v>
       </c>
       <c r="C44" t="str">
-        <v>Manual</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44">
         <v>0</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H44" t="str">
-        <v>2026-10-14T13:42:32.444Z</v>
+        <v>2026-10-15T12:11:36.401Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B45" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (7).xlsx</v>
       </c>
       <c r="C45" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D45">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45">
         <v>2</v>
       </c>
-      <c r="F45">
-        <v>0</v>
-      </c>
-      <c r="G45">
-        <v>35</v>
-      </c>
       <c r="H45" t="str">
-        <v>2026-10-14T13:41:21.926Z</v>
+        <v>2026-10-15T12:11:36.397Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B46" t="str">
-        <v>picking-report (6).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
       </c>
       <c r="C46" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D46">
-        <v>7</v>
+        <v>114</v>
       </c>
       <c r="E46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G46">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="H46" t="str">
-        <v>2026-10-14T13:41:21.925Z</v>
+        <v>2026-10-15T12:11:36.389Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>14-10-2026, 10:42:32 a. m.</v>
       </c>
       <c r="B47" t="str">
-        <v>ventas-report (6).xlsx</v>
+        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
       </c>
       <c r="C47" t="str">
-        <v>DropGO · ventas</v>
+        <v>Manual</v>
       </c>
       <c r="D47">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F47">
         <v>0</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-10-14T13:41:21.921Z</v>
+        <v>2026-10-14T13:42:32.444Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B48" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C48" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -20002,93 +20002,93 @@
         <v>0</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="H48" t="str">
-        <v>2026-10-14T13:40:03.191Z</v>
+        <v>2026-10-14T13:41:21.926Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B49" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (6).xlsx</v>
       </c>
       <c r="C49" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D49">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F49">
         <v>0</v>
       </c>
       <c r="G49">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H49" t="str">
-        <v>2026-10-14T13:40:03.190Z</v>
+        <v>2026-10-14T13:41:21.925Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B50" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
+        <v>ventas-report (6).xlsx</v>
       </c>
       <c r="C50" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D50">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="E50">
         <v>3</v>
       </c>
       <c r="F50">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G50">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="H50" t="str">
-        <v>2026-10-14T13:40:03.188Z</v>
+        <v>2026-10-14T13:41:21.921Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>14-10-2026, 10:39:50 a. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B51" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C51" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D51">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F51">
         <v>0</v>
       </c>
       <c r="G51">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H51" t="str">
-        <v>2026-10-14T13:39:50.407Z</v>
+        <v>2026-10-14T13:40:03.191Z</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B52" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20109,38 +20109,38 @@
         <v>35</v>
       </c>
       <c r="H52" t="str">
-        <v>2026-10-13T16:19:36.490Z</v>
+        <v>2026-10-14T13:40:03.190Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B53" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
       </c>
       <c r="C53" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D53">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F53">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G53">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H53" t="str">
-        <v>2026-10-13T16:19:36.488Z</v>
+        <v>2026-10-14T13:40:03.188Z</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>13-10-2026, 11:56:40 a. m.</v>
+        <v>14-10-2026, 10:39:50 a. m.</v>
       </c>
       <c r="B54" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20161,12 +20161,12 @@
         <v>35</v>
       </c>
       <c r="H54" t="str">
-        <v>2026-10-13T14:56:40.589Z</v>
+        <v>2026-10-14T13:39:50.407Z</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B55" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20178,177 +20178,177 @@
         <v>35</v>
       </c>
       <c r="E55">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G55">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H55" t="str">
-        <v>2026-10-13T14:44:42.285Z</v>
+        <v>2026-10-13T16:19:36.490Z</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B56" t="str">
-        <v>picking-report (5).xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C56" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D56">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F56">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G56">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="H56" t="str">
-        <v>2026-10-13T14:44:42.284Z</v>
+        <v>2026-10-13T16:19:36.488Z</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 11:56:40 a. m.</v>
       </c>
       <c r="B57" t="str">
-        <v>ventas-report (5).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C57" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D57">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F57">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G57">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H57" t="str">
-        <v>2026-10-13T14:44:42.280Z</v>
+        <v>2026-10-13T14:56:40.589Z</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B58" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C58" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D58">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="E58">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-13T12:49:30.632Z</v>
+        <v>2026-10-13T14:44:42.285Z</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B59" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (5).xlsx</v>
       </c>
       <c r="C59" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D59">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E59">
+        <v>2</v>
+      </c>
+      <c r="F59">
+        <v>6</v>
+      </c>
+      <c r="G59">
         <v>0</v>
       </c>
-      <c r="F59">
-        <v>0</v>
-      </c>
-      <c r="G59">
-        <v>34</v>
-      </c>
       <c r="H59" t="str">
-        <v>2026-10-13T12:49:30.631Z</v>
+        <v>2026-10-13T14:44:42.284Z</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B60" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>ventas-report (5).xlsx</v>
       </c>
       <c r="C60" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D60">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="E60">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F60">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G60">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H60" t="str">
-        <v>2026-10-13T12:49:30.629Z</v>
+        <v>2026-10-13T14:44:42.280Z</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>13-10-2026, 9:08:58 a. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B61" t="str">
-        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C61" t="str">
-        <v>Manual</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D61">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E61">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F61">
         <v>0</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H61" t="str">
-        <v>2026-10-13T12:08:58.547Z</v>
+        <v>2026-10-13T12:49:30.632Z</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B62" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20369,116 +20369,116 @@
         <v>34</v>
       </c>
       <c r="H62" t="str">
-        <v>2026-10-12T18:40:27.007Z</v>
+        <v>2026-10-13T12:49:30.631Z</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B63" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C63" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D63">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E63">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F63">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G63">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H63" t="str">
-        <v>2026-10-12T18:40:27.006Z</v>
+        <v>2026-10-13T12:49:30.629Z</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>13-10-2026, 9:08:58 a. m.</v>
       </c>
       <c r="B64" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
       </c>
       <c r="C64" t="str">
-        <v>DropGO · generado</v>
+        <v>Manual</v>
       </c>
       <c r="D64">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E64">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F64">
         <v>0</v>
       </c>
       <c r="G64">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H64" t="str">
-        <v>2026-10-12T18:39:34.326Z</v>
+        <v>2026-10-13T12:08:58.547Z</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B65" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C65" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D65">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E65">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F65">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H65" t="str">
-        <v>2026-10-12T18:39:34.325Z</v>
+        <v>2026-10-12T18:40:27.007Z</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B66" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C66" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D66">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E66">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H66" t="str">
-        <v>2026-10-12T18:39:34.319Z</v>
+        <v>2026-10-12T18:40:27.006Z</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>12-10-2026, 3:39:18 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B67" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20487,10 +20487,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D67">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F67">
         <v>0</v>
@@ -20499,116 +20499,116 @@
         <v>25</v>
       </c>
       <c r="H67" t="str">
-        <v>2026-10-12T18:39:18.385Z</v>
+        <v>2026-10-12T18:39:34.326Z</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>12-10-2026, 12:05:40 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B68" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C68" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D68">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F68">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G68">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H68" t="str">
-        <v>2026-10-12T15:05:40.188Z</v>
+        <v>2026-10-12T18:39:34.325Z</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B69" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C69" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D69">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G69">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H69" t="str">
-        <v>2026-10-12T14:26:19.514Z</v>
+        <v>2026-10-12T18:39:34.319Z</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:18 p. m.</v>
       </c>
       <c r="B70" t="str">
-        <v>orders_export (6).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C70" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D70">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E70">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F70">
         <v>0</v>
       </c>
       <c r="G70">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H70" t="str">
-        <v>2026-10-12T14:26:19.513Z</v>
+        <v>2026-10-12T18:39:18.385Z</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 12:05:40 p. m.</v>
       </c>
       <c r="B71" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C71" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D71">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E71">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F71">
         <v>0</v>
       </c>
       <c r="G71">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-10-12T14:24:55.059Z</v>
+        <v>2026-10-12T15:05:40.188Z</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B72" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20629,64 +20629,64 @@
         <v>25</v>
       </c>
       <c r="H72" t="str">
-        <v>2026-10-12T14:24:55.058Z</v>
+        <v>2026-10-12T14:26:19.514Z</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B73" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>orders_export (6).csv</v>
       </c>
       <c r="C73" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D73">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E73">
         <v>4</v>
       </c>
       <c r="F73">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G73">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H73" t="str">
-        <v>2026-10-12T14:24:55.057Z</v>
+        <v>2026-10-12T14:26:19.513Z</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>12-10-2026, 11:24:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B74" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C74" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D74">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F74">
         <v>0</v>
       </c>
       <c r="G74">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H74" t="str">
-        <v>2026-10-12T14:24:00.106Z</v>
+        <v>2026-10-12T14:24:55.059Z</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B75" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20698,73 +20698,73 @@
         <v>25</v>
       </c>
       <c r="E75">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F75">
         <v>0</v>
       </c>
       <c r="G75">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H75" t="str">
-        <v>2026-10-09T14:54:00.353Z</v>
+        <v>2026-10-12T14:24:55.058Z</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B76" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C76" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D76">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G76">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H76" t="str">
-        <v>2026-10-09T14:54:00.352Z</v>
+        <v>2026-10-12T14:24:55.057Z</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:00 a. m.</v>
       </c>
       <c r="B77" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C77" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D77">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E77">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F77">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G77">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H77" t="str">
-        <v>2026-10-09T14:54:00.347Z</v>
+        <v>2026-10-12T14:24:00.106Z</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>09-10-2026, 11:50:59 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B78" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20773,10 +20773,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D78">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F78">
         <v>0</v>
@@ -20785,64 +20785,64 @@
         <v>21</v>
       </c>
       <c r="H78" t="str">
-        <v>2026-10-09T14:50:59.695Z</v>
+        <v>2026-10-09T14:54:00.353Z</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B79" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C79" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D79">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G79">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H79" t="str">
-        <v>2026-10-09T14:28:16.404Z</v>
+        <v>2026-10-09T14:54:00.352Z</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B80" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C80" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D80">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E80">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G80">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H80" t="str">
-        <v>2026-10-09T14:28:16.403Z</v>
+        <v>2026-10-09T14:54:00.347Z</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>09-10-2026, 11:28:07 a. m.</v>
+        <v>09-10-2026, 11:50:59 a. m.</v>
       </c>
       <c r="B81" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20863,12 +20863,12 @@
         <v>21</v>
       </c>
       <c r="H81" t="str">
-        <v>2026-10-09T14:28:07.531Z</v>
+        <v>2026-10-09T14:50:59.695Z</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B82" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20889,12 +20889,12 @@
         <v>21</v>
       </c>
       <c r="H82" t="str">
-        <v>2026-10-09T14:26:45.497Z</v>
+        <v>2026-10-09T14:28:16.404Z</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B83" t="str">
         <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
@@ -20915,21 +20915,21 @@
         <v>19</v>
       </c>
       <c r="H83" t="str">
-        <v>2026-10-09T14:26:45.495Z</v>
+        <v>2026-10-09T14:28:16.403Z</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:07 a. m.</v>
       </c>
       <c r="B84" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C84" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D84">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -20938,50 +20938,50 @@
         <v>0</v>
       </c>
       <c r="G84">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H84" t="str">
-        <v>2026-10-09T14:26:45.477Z</v>
+        <v>2026-10-09T14:28:07.531Z</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B85" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C85" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D85">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E85">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F85">
         <v>0</v>
       </c>
       <c r="G85">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H85" t="str">
-        <v>2026-10-09T14:25:43.607Z</v>
+        <v>2026-10-09T14:26:45.497Z</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B86" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C86" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D86">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E86">
         <v>0</v>
@@ -20990,36 +20990,36 @@
         <v>0</v>
       </c>
       <c r="G86">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H86" t="str">
-        <v>2026-10-09T14:25:43.606Z</v>
+        <v>2026-10-09T14:26:45.495Z</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B87" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C87" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D87">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F87">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G87">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H87" t="str">
-        <v>2026-10-09T14:25:43.605Z</v>
+        <v>2026-10-09T14:26:45.477Z</v>
       </c>
     </row>
     <row r="88">
@@ -21027,30 +21027,30 @@
         <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B88" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C88" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D88">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E88">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F88">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G88">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H88" t="str">
-        <v>2026-10-09T14:25:43.580Z</v>
+        <v>2026-10-09T14:25:43.607Z</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>09-10-2026, 11:23:53 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B89" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21071,111 +21071,111 @@
         <v>21</v>
       </c>
       <c r="H89" t="str">
-        <v>2026-10-09T14:23:53.263Z</v>
+        <v>2026-10-09T14:25:43.606Z</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>08-10-2026, 9:14:25 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B90" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C90" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D90">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E90">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F90">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G90">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H90" t="str">
-        <v>2026-10-08T12:14:25.917Z</v>
+        <v>2026-10-09T14:25:43.605Z</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B91" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C91" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D91">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E91">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H91" t="str">
-        <v>2026-10-08T11:22:18.060Z</v>
+        <v>2026-10-09T14:25:43.580Z</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:23:53 a. m.</v>
       </c>
       <c r="B92" t="str">
-        <v>orders_export (4).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C92" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D92">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F92">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G92">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H92" t="str">
-        <v>2026-10-08T11:22:18.059Z</v>
+        <v>2026-10-09T14:23:53.263Z</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>08-10-2026, 9:14:25 a. m.</v>
       </c>
       <c r="B93" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C93" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D93">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E93">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F93">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H93" t="str">
-        <v>2026-10-08T11:22:18.042Z</v>
+        <v>2026-10-08T12:14:25.917Z</v>
       </c>
     </row>
     <row r="94">
@@ -21183,108 +21183,108 @@
         <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B94" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C94" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D94">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E94">
         <v>2</v>
       </c>
       <c r="F94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G94">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H94" t="str">
-        <v>2026-10-08T11:22:18.032Z</v>
+        <v>2026-10-08T11:22:18.060Z</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>08-10-2026, 8:18:16 a. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B95" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (4).csv</v>
       </c>
       <c r="C95" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D95">
         <v>19</v>
       </c>
       <c r="E95">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G95">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H95" t="str">
-        <v>2026-10-08T11:18:16.488Z</v>
+        <v>2026-10-08T11:22:18.059Z</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B96" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C96" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D96">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E96">
+        <v>2</v>
+      </c>
+      <c r="F96">
+        <v>1</v>
+      </c>
+      <c r="G96">
         <v>0</v>
       </c>
-      <c r="F96">
-        <v>0</v>
-      </c>
-      <c r="G96">
-        <v>19</v>
-      </c>
       <c r="H96" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.042Z</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B97" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C97" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D97">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E97">
         <v>2</v>
       </c>
       <c r="F97">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G97">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H97" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.032Z</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>07-10-2026, 8:20:41 p. m.</v>
+        <v>08-10-2026, 8:18:16 a. m.</v>
       </c>
       <c r="B98" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21305,12 +21305,12 @@
         <v>19</v>
       </c>
       <c r="H98" t="str">
-        <v>2026-10-07T23:20:41.390Z</v>
+        <v>2026-10-08T11:18:16.488Z</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B99" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21331,38 +21331,38 @@
         <v>19</v>
       </c>
       <c r="H99" t="str">
-        <v>2026-10-07T17:47:17.199Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B100" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
       </c>
       <c r="C100" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D100">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E100">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F100">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G100">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H100" t="str">
-        <v>2026-10-07T17:47:17.198Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>07-10-2026, 2:46:47 p. m.</v>
+        <v>07-10-2026, 8:20:41 p. m.</v>
       </c>
       <c r="B101" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21383,12 +21383,12 @@
         <v>19</v>
       </c>
       <c r="H101" t="str">
-        <v>2026-10-07T17:46:47.954Z</v>
+        <v>2026-10-07T23:20:41.390Z</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>07-10-2026, 2:44:00 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B102" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21409,64 +21409,64 @@
         <v>19</v>
       </c>
       <c r="H102" t="str">
-        <v>2026-10-07T17:44:00.660Z</v>
+        <v>2026-10-07T17:47:17.199Z</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>07-10-2026, 2:27:43 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B103" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
       </c>
       <c r="C103" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D103">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E103">
         <v>0</v>
       </c>
       <c r="F103">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G103">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="H103" t="str">
-        <v>2026-10-07T17:27:43.517Z</v>
+        <v>2026-10-07T17:47:17.198Z</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:46:47 p. m.</v>
       </c>
       <c r="B104" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C104" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D104">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E104">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F104">
         <v>0</v>
       </c>
       <c r="G104">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-10-07T17:26:50.382Z</v>
+        <v>2026-10-07T17:46:47.954Z</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:44:00 p. m.</v>
       </c>
       <c r="B105" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21478,21 +21478,21 @@
         <v>19</v>
       </c>
       <c r="E105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F105">
         <v>0</v>
       </c>
       <c r="G105">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H105" t="str">
-        <v>2026-10-07T17:26:50.380Z</v>
+        <v>2026-10-07T17:44:00.660Z</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:27:43 p. m.</v>
       </c>
       <c r="B106" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21501,7 +21501,7 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D106">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E106">
         <v>0</v>
@@ -21510,41 +21510,41 @@
         <v>0</v>
       </c>
       <c r="G106">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H106" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:27:43.517Z</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B107" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C107" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D107">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="E107">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F107">
         <v>0</v>
       </c>
       <c r="G107">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H107" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:26:50.382Z</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B108" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21553,71 +21553,71 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D108">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E108">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-10-07T16:25:12.953Z</v>
+        <v>2026-10-07T17:26:50.380Z</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B109" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C109" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D109">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E109">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F109">
         <v>0</v>
       </c>
       <c r="G109">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H109" t="str">
-        <v>2026-10-07T16:25:12.950Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B110" t="str">
-        <v>orders_export (3).csv</v>
+        <v>ventas_por_canal_y_mes.xlsx</v>
       </c>
       <c r="C110" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Ventas por canal y mes</v>
       </c>
       <c r="D110">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="E110">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F110">
         <v>0</v>
       </c>
       <c r="G110">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="H110" t="str">
-        <v>2026-10-07T16:25:12.939Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="111">
@@ -21625,25 +21625,25 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B111" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C111" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D111">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F111">
         <v>0</v>
       </c>
       <c r="G111">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H111" t="str">
-        <v>2026-10-07T16:25:12.924Z</v>
+        <v>2026-10-07T16:25:12.953Z</v>
       </c>
     </row>
     <row r="112">
@@ -21651,10 +21651,10 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B112" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C112" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D112">
         <v>19</v>
@@ -21669,142 +21669,220 @@
         <v>0</v>
       </c>
       <c r="H112" t="str">
-        <v>2026-10-07T16:25:12.851Z</v>
+        <v>2026-10-07T16:25:12.950Z</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>07-10-2026, 1:10:27 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B113" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>orders_export (3).csv</v>
       </c>
       <c r="C113" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D113">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E113">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F113">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G113">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="H113" t="str">
-        <v>2026-10-07T16:10:27.561Z</v>
+        <v>2026-10-07T16:25:12.939Z</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>07-10-2026, 12:20:36 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B114" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C114" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D114">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F114">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G114">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H114" t="str">
-        <v>2026-10-07T15:20:36.001Z</v>
+        <v>2026-10-07T16:25:12.924Z</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>07-10-2026, 12:20:35 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B115" t="str">
-        <v>varin_respaldo_2026-10-07.xlsx</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C115" t="str">
-        <v>Respaldo</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D115">
-        <v>322</v>
+        <v>19</v>
       </c>
       <c r="E115">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F115">
         <v>0</v>
       </c>
       <c r="G115">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H115" t="str">
-        <v>2026-10-07T15:20:35.967Z</v>
+        <v>2026-10-07T16:25:12.851Z</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>07-10-2026, 12:20:08 p. m.</v>
+        <v>07-10-2026, 1:10:27 p. m.</v>
       </c>
       <c r="B116" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C116" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D116">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E116">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="F116">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="H116" t="str">
-        <v>2026-10-07T15:20:08.547Z</v>
+        <v>2026-10-07T16:10:27.561Z</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
+        <v>07-10-2026, 12:20:36 p. m.</v>
+      </c>
+      <c r="B117" t="str">
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Ventas Mercado Libre</v>
+      </c>
+      <c r="D117">
+        <v>92</v>
+      </c>
+      <c r="E117">
+        <v>1</v>
+      </c>
+      <c r="F117">
+        <v>5</v>
+      </c>
+      <c r="G117">
+        <v>86</v>
+      </c>
+      <c r="H117" t="str">
+        <v>2026-10-07T15:20:36.001Z</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>07-10-2026, 12:20:35 p. m.</v>
+      </c>
+      <c r="B118" t="str">
+        <v>varin_respaldo_2026-10-07.xlsx</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Respaldo</v>
+      </c>
+      <c r="D118">
+        <v>322</v>
+      </c>
+      <c r="E118">
+        <v>190</v>
+      </c>
+      <c r="F118">
+        <v>0</v>
+      </c>
+      <c r="G118">
+        <v>132</v>
+      </c>
+      <c r="H118" t="str">
+        <v>2026-10-07T15:20:35.967Z</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
         <v>07-10-2026, 12:20:08 p. m.</v>
       </c>
-      <c r="B117" t="str">
+      <c r="B119" t="str">
+        <v>ventas_por_canal_y_mes.xlsx</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Ventas por canal y mes</v>
+      </c>
+      <c r="D119">
+        <v>118</v>
+      </c>
+      <c r="E119">
+        <v>118</v>
+      </c>
+      <c r="F119">
+        <v>0</v>
+      </c>
+      <c r="G119">
+        <v>0</v>
+      </c>
+      <c r="H119" t="str">
+        <v>2026-10-07T15:20:08.547Z</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>07-10-2026, 12:20:08 p. m.</v>
+      </c>
+      <c r="B120" t="str">
         <v>Varin_Movimientos_DropGO_2026-10-01_al_2026-10-06.xlsx</v>
       </c>
-      <c r="C117" t="str">
+      <c r="C120" t="str">
         <v>Movimientos DropGO</v>
       </c>
-      <c r="D117">
+      <c r="D120">
         <v>14</v>
       </c>
-      <c r="E117">
+      <c r="E120">
         <v>14</v>
       </c>
-      <c r="F117">
+      <c r="F120">
         <v>0</v>
       </c>
-      <c r="G117">
+      <c r="G120">
         <v>0</v>
       </c>
-      <c r="H117" t="str">
+      <c r="H120" t="str">
         <v>2026-10-07T15:20:08.525Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H117"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H120"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -25132,7 +25210,7 @@
         <v>Generado</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-23T13:18:00.704Z</v>
+        <v>2026-10-23T22:12:17.093Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Datos Varin 2026-10-28 10:56
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -19815,7 +19815,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H143"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -19854,7 +19854,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B2" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19875,38 +19875,38 @@
         <v>50</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-27T22:11:05.716Z</v>
+        <v>2026-10-28T10:56:06.328Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B3" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
       </c>
       <c r="C3" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D3">
-        <v>148</v>
+        <v>69</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>144</v>
+        <v>69</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-10-27T22:11:05.714Z</v>
+        <v>2026-10-28T10:56:06.326Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>27-10-2026, 7:10:39 p. m.</v>
+        <v>28-10-2026, 7:53:38 a. m.</v>
       </c>
       <c r="B4" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19927,12 +19927,12 @@
         <v>50</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-10-27T22:10:39.288Z</v>
+        <v>2026-10-28T10:53:38.820Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B5" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -19944,68 +19944,68 @@
         <v>50</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-10-27T12:40:01.215Z</v>
+        <v>2026-10-27T22:11:05.716Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B6" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
       </c>
       <c r="C6" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D6">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G6">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-10-27T12:40:01.212Z</v>
+        <v>2026-10-27T22:11:05.714Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:10:39 p. m.</v>
       </c>
       <c r="B7" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C7" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-10-27T12:40:01.116Z</v>
+        <v>2026-10-27T22:10:39.288Z</v>
       </c>
     </row>
     <row r="8">
@@ -20013,186 +20013,186 @@
         <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B8" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C8" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-10-27T12:40:01.113Z</v>
+        <v>2026-10-27T12:40:01.215Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B9" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C9" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>147</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-10-27T12:39:46.660Z</v>
+        <v>2026-10-27T12:40:01.212Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B10" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C10" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D10">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
         <v>0</v>
       </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>49</v>
-      </c>
       <c r="H10" t="str">
-        <v>2026-10-27T12:39:46.656Z</v>
+        <v>2026-10-27T12:40:01.116Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B11" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C11" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D11">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
         <v>0</v>
       </c>
-      <c r="G11">
-        <v>3</v>
-      </c>
       <c r="H11" t="str">
-        <v>2026-10-27T12:35:13.606Z</v>
+        <v>2026-10-27T12:40:01.113Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B12" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C12" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D12">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-10-27T12:35:13.605Z</v>
+        <v>2026-10-27T12:39:46.660Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B13" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C13" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D13">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="E13">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>131</v>
+        <v>49</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-10-27T12:35:13.604Z</v>
+        <v>2026-10-27T12:39:46.656Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>27-10-2026, 9:34:54 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B14" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C14" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D14">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-10-27T12:34:54.468Z</v>
+        <v>2026-10-27T12:35:13.606Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B15" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20204,177 +20204,177 @@
         <v>49</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-10-26T12:06:47.126Z</v>
+        <v>2026-10-27T12:35:13.605Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B16" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
       </c>
       <c r="C16" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-10-26T12:06:47.123Z</v>
+        <v>2026-10-27T12:35:13.604Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:34:54 a. m.</v>
       </c>
       <c r="B17" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C17" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D17">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-10-26T12:06:47.118Z</v>
+        <v>2026-10-27T12:34:54.468Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B18" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C18" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D18">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E18">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-10-26T12:05:32.699Z</v>
+        <v>2026-10-26T12:06:47.126Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B19" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C19" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D19">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
         <v>0</v>
       </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-      <c r="G19">
-        <v>48</v>
-      </c>
       <c r="H19" t="str">
-        <v>2026-10-26T12:05:32.697Z</v>
+        <v>2026-10-26T12:06:47.123Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B20" t="str">
-        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C20" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20">
         <v>0</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-10-26T12:05:32.692Z</v>
+        <v>2026-10-26T12:06:47.118Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>25-10-2026, 12:10:56 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B21" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C21" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D21">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-10-25T15:10:56.412Z</v>
+        <v>2026-10-26T12:05:32.699Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B22" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20395,38 +20395,38 @@
         <v>48</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-23T22:12:12.477Z</v>
+        <v>2026-10-26T12:05:32.697Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B23" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
+        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
       </c>
       <c r="C23" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D23">
-        <v>135</v>
+        <v>6</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
       <c r="G23">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="H23" t="str">
-        <v>2026-10-23T22:12:12.476Z</v>
+        <v>2026-10-26T12:05:32.692Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>23-10-2026, 7:11:53 p. m.</v>
+        <v>25-10-2026, 12:10:56 p. m.</v>
       </c>
       <c r="B24" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20447,12 +20447,12 @@
         <v>48</v>
       </c>
       <c r="H24" t="str">
-        <v>2026-10-23T22:11:53.140Z</v>
+        <v>2026-10-25T15:10:56.412Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B25" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20473,15 +20473,15 @@
         <v>48</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-10-23T13:17:56.047Z</v>
+        <v>2026-10-23T22:12:12.477Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B26" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C26" t="str">
         <v>Ventas Mercado Libre</v>
@@ -20499,12 +20499,12 @@
         <v>135</v>
       </c>
       <c r="H26" t="str">
-        <v>2026-10-23T13:17:56.044Z</v>
+        <v>2026-10-23T22:12:12.476Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>23-10-2026, 9:52:55 a. m.</v>
+        <v>23-10-2026, 7:11:53 p. m.</v>
       </c>
       <c r="B27" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20525,12 +20525,12 @@
         <v>48</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-10-23T12:52:55.551Z</v>
+        <v>2026-10-23T22:11:53.140Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>23-10-2026, 9:50:04 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B28" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20551,38 +20551,38 @@
         <v>48</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-10-23T12:50:04.195Z</v>
+        <v>2026-10-23T13:17:56.047Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B29" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C29" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="H29" t="str">
-        <v>2026-10-23T12:37:54.995Z</v>
+        <v>2026-10-23T13:17:56.044Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:52:55 a. m.</v>
       </c>
       <c r="B30" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20603,64 +20603,64 @@
         <v>48</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-10-23T12:37:54.994Z</v>
+        <v>2026-10-23T12:52:55.551Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:50:04 a. m.</v>
       </c>
       <c r="B31" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C31" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D31">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-10-23T12:37:54.992Z</v>
+        <v>2026-10-23T12:50:04.195Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>23-10-2026, 9:37:27 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B32" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C32" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D32">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32">
         <v>0</v>
       </c>
       <c r="G32">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H32" t="str">
-        <v>2026-10-23T12:37:27.533Z</v>
+        <v>2026-10-23T12:37:54.995Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>23-10-2026, 9:34:31 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B33" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20681,64 +20681,64 @@
         <v>48</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-10-23T12:34:31.611Z</v>
+        <v>2026-10-23T12:37:54.994Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>23-10-2026, 9:19:14 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B34" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C34" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D34">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G34">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="H34" t="str">
-        <v>2026-10-23T12:19:14.833Z</v>
+        <v>2026-10-23T12:37:54.992Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:37:27 a. m.</v>
       </c>
       <c r="B35" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C35" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E35">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
       <c r="G35">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H35" t="str">
-        <v>2026-10-22T11:51:13.535Z</v>
+        <v>2026-10-23T12:37:27.533Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:34:31 a. m.</v>
       </c>
       <c r="B36" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20759,38 +20759,38 @@
         <v>48</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-10-22T11:51:13.534Z</v>
+        <v>2026-10-23T12:34:31.611Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:19:14 a. m.</v>
       </c>
       <c r="B37" t="str">
-        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C37" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D37">
-        <v>134</v>
+        <v>48</v>
       </c>
       <c r="E37">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F37">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="H37" t="str">
-        <v>2026-10-22T11:51:13.529Z</v>
+        <v>2026-10-23T12:19:14.833Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B38" t="str">
         <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
@@ -20799,10 +20799,10 @@
         <v>Full ML · generado</v>
       </c>
       <c r="D38">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -20811,12 +20811,12 @@
         <v>2</v>
       </c>
       <c r="H38" t="str">
-        <v>2026-10-21T11:58:09.619Z</v>
+        <v>2026-10-22T11:51:13.535Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B39" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20828,42 +20828,42 @@
         <v>48</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H39" t="str">
-        <v>2026-10-21T11:58:09.618Z</v>
+        <v>2026-10-22T11:51:13.534Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B40" t="str">
-        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
+        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
       </c>
       <c r="C40" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D40">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F40">
         <v>5</v>
       </c>
       <c r="G40">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H40" t="str">
-        <v>2026-10-21T11:58:09.614Z</v>
+        <v>2026-10-22T11:51:13.529Z</v>
       </c>
     </row>
     <row r="41">
@@ -20871,25 +20871,25 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B41" t="str">
-        <v>ventas-report (11).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C41" t="str">
-        <v>DropGO · ventas</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D41">
+        <v>4</v>
+      </c>
+      <c r="E41">
         <v>2</v>
-      </c>
-      <c r="E41">
-        <v>1</v>
       </c>
       <c r="F41">
         <v>0</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" t="str">
-        <v>2026-10-21T11:58:09.533Z</v>
+        <v>2026-10-21T11:58:09.619Z</v>
       </c>
     </row>
     <row r="42">
@@ -20897,13 +20897,13 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B42" t="str">
-        <v>picking-report (11).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C42" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D42">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -20912,50 +20912,50 @@
         <v>0</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H42" t="str">
-        <v>2026-10-21T11:58:09.530Z</v>
+        <v>2026-10-21T11:58:09.618Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B43" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
       </c>
       <c r="C43" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D43">
+        <v>128</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+      <c r="F43">
         <v>5</v>
       </c>
-      <c r="E43">
-        <v>3</v>
-      </c>
-      <c r="F43">
-        <v>0</v>
-      </c>
       <c r="G43">
-        <v>2</v>
+        <v>121</v>
       </c>
       <c r="H43" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.614Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B44" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (11).xlsx</v>
       </c>
       <c r="C44" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D44">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -20964,36 +20964,36 @@
         <v>0</v>
       </c>
       <c r="G44">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="H44" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.533Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B45" t="str">
-        <v>ventas-report (10).xlsx</v>
+        <v>picking-report (11).xlsx</v>
       </c>
       <c r="C45" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D45">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E45">
         <v>1</v>
       </c>
       <c r="F45">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G45">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H45" t="str">
-        <v>2026-10-20T12:36:20.899Z</v>
+        <v>2026-10-21T11:58:09.530Z</v>
       </c>
     </row>
     <row r="46">
@@ -21001,25 +21001,25 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B46" t="str">
-        <v>picking-report (10).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C46" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D46">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="E46">
         <v>1</v>
       </c>
       <c r="F46">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G46">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="H46" t="str">
-        <v>2026-10-20T12:36:20.895Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="47">
@@ -21027,212 +21027,212 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B47" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C47" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D47">
-        <v>126</v>
+        <v>5</v>
       </c>
       <c r="E47">
         <v>3</v>
       </c>
       <c r="F47">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G47">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-10-20T12:36:20.890Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>20-10-2026, 9:34:26 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B48" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (10).xlsx</v>
       </c>
       <c r="C48" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D48">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F48">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G48">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="H48" t="str">
-        <v>2026-10-20T12:34:26.210Z</v>
+        <v>2026-10-20T12:36:20.899Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B49" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (10).xlsx</v>
       </c>
       <c r="C49" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D49">
+        <v>11</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <v>3</v>
+      </c>
+      <c r="G49">
         <v>7</v>
       </c>
-      <c r="E49">
-        <v>5</v>
-      </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-      <c r="G49">
-        <v>2</v>
-      </c>
       <c r="H49" t="str">
-        <v>2026-10-19T12:21:51.769Z</v>
+        <v>2026-10-20T12:36:20.895Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B50" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C50" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D50">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G50">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="H50" t="str">
-        <v>2026-10-19T12:21:51.768Z</v>
+        <v>2026-10-20T12:36:20.890Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:34:26 a. m.</v>
       </c>
       <c r="B51" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C51" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D51">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E51">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G51">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H51" t="str">
-        <v>2026-10-19T12:21:51.766Z</v>
+        <v>2026-10-20T12:34:26.210Z</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B52" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C52" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D52">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E52">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H52" t="str">
-        <v>2026-10-19T12:20:51.921Z</v>
+        <v>2026-10-19T12:21:51.769Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B53" t="str">
-        <v>picking-report (9).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C53" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D53">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E53">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F53">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="H53" t="str">
-        <v>2026-10-19T12:20:51.919Z</v>
+        <v>2026-10-19T12:21:51.768Z</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B54" t="str">
-        <v>ventas-report (9).xlsx</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
       </c>
       <c r="C54" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D54">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="E54">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F54">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G54">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H54" t="str">
-        <v>2026-10-19T12:20:51.913Z</v>
+        <v>2026-10-19T12:21:51.766Z</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>19-10-2026, 9:12:06 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B55" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21241,10 +21241,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D55">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F55">
         <v>0</v>
@@ -21253,229 +21253,229 @@
         <v>37</v>
       </c>
       <c r="H55" t="str">
-        <v>2026-10-19T12:12:06.575Z</v>
+        <v>2026-10-19T12:20:51.921Z</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B56" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (9).xlsx</v>
       </c>
       <c r="C56" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D56">
+        <v>14</v>
+      </c>
+      <c r="E56">
+        <v>7</v>
+      </c>
+      <c r="F56">
         <v>5</v>
-      </c>
-      <c r="E56">
-        <v>3</v>
-      </c>
-      <c r="F56">
-        <v>0</v>
       </c>
       <c r="G56">
         <v>2</v>
       </c>
       <c r="H56" t="str">
-        <v>2026-10-16T12:37:12.832Z</v>
+        <v>2026-10-19T12:20:51.919Z</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B57" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (9).xlsx</v>
       </c>
       <c r="C57" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D57">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F57">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G57">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H57" t="str">
-        <v>2026-10-16T12:37:12.831Z</v>
+        <v>2026-10-19T12:20:51.913Z</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:12:06 a. m.</v>
       </c>
       <c r="B58" t="str">
-        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C58" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D58">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F58">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G58">
         <v>37</v>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-16T12:37:12.827Z</v>
+        <v>2026-10-19T12:12:06.575Z</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B59" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C59" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D59">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E59">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F59">
         <v>0</v>
       </c>
       <c r="G59">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H59" t="str">
-        <v>2026-10-16T11:52:26.043Z</v>
+        <v>2026-10-16T12:37:12.832Z</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B60" t="str">
-        <v>picking-report (8).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C60" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D60">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E60">
         <v>0</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H60" t="str">
-        <v>2026-10-16T11:52:26.040Z</v>
+        <v>2026-10-16T12:37:12.831Z</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B61" t="str">
-        <v>ventas-report (8).xlsx</v>
+        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
       </c>
       <c r="C61" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D61">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E61">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F61">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H61" t="str">
-        <v>2026-10-16T11:52:26.034Z</v>
+        <v>2026-10-16T12:37:12.827Z</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B62" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C62" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D62">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F62">
         <v>0</v>
       </c>
       <c r="G62">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H62" t="str">
-        <v>2026-10-15T12:11:36.404Z</v>
+        <v>2026-10-16T11:52:26.043Z</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B63" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (8).xlsx</v>
       </c>
       <c r="C63" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D63">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H63" t="str">
-        <v>2026-10-15T12:11:36.403Z</v>
+        <v>2026-10-16T11:52:26.040Z</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B64" t="str">
-        <v>ventas-report (7).xlsx</v>
+        <v>ventas-report (8).xlsx</v>
       </c>
       <c r="C64" t="str">
         <v>DropGO · ventas</v>
       </c>
       <c r="D64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -21484,10 +21484,10 @@
         <v>1</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64" t="str">
-        <v>2026-10-15T12:11:36.401Z</v>
+        <v>2026-10-16T11:52:26.034Z</v>
       </c>
     </row>
     <row r="65">
@@ -21495,25 +21495,25 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B65" t="str">
-        <v>picking-report (7).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C65" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D65">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E65">
+        <v>2</v>
+      </c>
+      <c r="F65">
         <v>0</v>
-      </c>
-      <c r="F65">
-        <v>1</v>
       </c>
       <c r="G65">
         <v>2</v>
       </c>
       <c r="H65" t="str">
-        <v>2026-10-15T12:11:36.397Z</v>
+        <v>2026-10-15T12:11:36.404Z</v>
       </c>
     </row>
     <row r="66">
@@ -21521,143 +21521,143 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B66" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C66" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D66">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E66">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G66">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="H66" t="str">
-        <v>2026-10-15T12:11:36.389Z</v>
+        <v>2026-10-15T12:11:36.403Z</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>14-10-2026, 10:42:32 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B67" t="str">
-        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
+        <v>ventas-report (7).xlsx</v>
       </c>
       <c r="C67" t="str">
-        <v>Manual</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E67">
         <v>0</v>
       </c>
       <c r="F67">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G67">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H67" t="str">
-        <v>2026-10-14T13:42:32.444Z</v>
+        <v>2026-10-15T12:11:36.401Z</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B68" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (7).xlsx</v>
       </c>
       <c r="C68" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D68">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>1</v>
+      </c>
+      <c r="G68">
         <v>2</v>
       </c>
-      <c r="F68">
-        <v>0</v>
-      </c>
-      <c r="G68">
-        <v>35</v>
-      </c>
       <c r="H68" t="str">
-        <v>2026-10-14T13:41:21.926Z</v>
+        <v>2026-10-15T12:11:36.397Z</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B69" t="str">
-        <v>picking-report (6).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
       </c>
       <c r="C69" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D69">
-        <v>7</v>
+        <v>114</v>
       </c>
       <c r="E69">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F69">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G69">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="H69" t="str">
-        <v>2026-10-14T13:41:21.925Z</v>
+        <v>2026-10-15T12:11:36.389Z</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>14-10-2026, 10:42:32 a. m.</v>
       </c>
       <c r="B70" t="str">
-        <v>ventas-report (6).xlsx</v>
+        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
       </c>
       <c r="C70" t="str">
-        <v>DropGO · ventas</v>
+        <v>Manual</v>
       </c>
       <c r="D70">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E70">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F70">
         <v>0</v>
       </c>
       <c r="G70">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H70" t="str">
-        <v>2026-10-14T13:41:21.921Z</v>
+        <v>2026-10-14T13:42:32.444Z</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B71" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C71" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D71">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E71">
         <v>2</v>
@@ -21666,93 +21666,93 @@
         <v>0</v>
       </c>
       <c r="G71">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-10-14T13:40:03.191Z</v>
+        <v>2026-10-14T13:41:21.926Z</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B72" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (6).xlsx</v>
       </c>
       <c r="C72" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D72">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H72" t="str">
-        <v>2026-10-14T13:40:03.190Z</v>
+        <v>2026-10-14T13:41:21.925Z</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B73" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
+        <v>ventas-report (6).xlsx</v>
       </c>
       <c r="C73" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D73">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="E73">
         <v>3</v>
       </c>
       <c r="F73">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G73">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="H73" t="str">
-        <v>2026-10-14T13:40:03.188Z</v>
+        <v>2026-10-14T13:41:21.921Z</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>14-10-2026, 10:39:50 a. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B74" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C74" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D74">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F74">
         <v>0</v>
       </c>
       <c r="G74">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H74" t="str">
-        <v>2026-10-14T13:39:50.407Z</v>
+        <v>2026-10-14T13:40:03.191Z</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B75" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21773,38 +21773,38 @@
         <v>35</v>
       </c>
       <c r="H75" t="str">
-        <v>2026-10-13T16:19:36.490Z</v>
+        <v>2026-10-14T13:40:03.190Z</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B76" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
       </c>
       <c r="C76" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D76">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E76">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F76">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G76">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H76" t="str">
-        <v>2026-10-13T16:19:36.488Z</v>
+        <v>2026-10-14T13:40:03.188Z</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>13-10-2026, 11:56:40 a. m.</v>
+        <v>14-10-2026, 10:39:50 a. m.</v>
       </c>
       <c r="B77" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21825,12 +21825,12 @@
         <v>35</v>
       </c>
       <c r="H77" t="str">
-        <v>2026-10-13T14:56:40.589Z</v>
+        <v>2026-10-14T13:39:50.407Z</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B78" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21842,177 +21842,177 @@
         <v>35</v>
       </c>
       <c r="E78">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H78" t="str">
-        <v>2026-10-13T14:44:42.285Z</v>
+        <v>2026-10-13T16:19:36.490Z</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B79" t="str">
-        <v>picking-report (5).xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C79" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D79">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="E79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F79">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="H79" t="str">
-        <v>2026-10-13T14:44:42.284Z</v>
+        <v>2026-10-13T16:19:36.488Z</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 11:56:40 a. m.</v>
       </c>
       <c r="B80" t="str">
-        <v>ventas-report (5).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C80" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D80">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F80">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G80">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H80" t="str">
-        <v>2026-10-13T14:44:42.280Z</v>
+        <v>2026-10-13T14:56:40.589Z</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B81" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C81" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D81">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="E81">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G81">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H81" t="str">
-        <v>2026-10-13T12:49:30.632Z</v>
+        <v>2026-10-13T14:44:42.285Z</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B82" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (5).xlsx</v>
       </c>
       <c r="C82" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D82">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E82">
+        <v>2</v>
+      </c>
+      <c r="F82">
+        <v>6</v>
+      </c>
+      <c r="G82">
         <v>0</v>
       </c>
-      <c r="F82">
-        <v>0</v>
-      </c>
-      <c r="G82">
-        <v>34</v>
-      </c>
       <c r="H82" t="str">
-        <v>2026-10-13T12:49:30.631Z</v>
+        <v>2026-10-13T14:44:42.284Z</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B83" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>ventas-report (5).xlsx</v>
       </c>
       <c r="C83" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D83">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="E83">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F83">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G83">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H83" t="str">
-        <v>2026-10-13T12:49:30.629Z</v>
+        <v>2026-10-13T14:44:42.280Z</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>13-10-2026, 9:08:58 a. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B84" t="str">
-        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C84" t="str">
-        <v>Manual</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F84">
         <v>0</v>
       </c>
       <c r="G84">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H84" t="str">
-        <v>2026-10-13T12:08:58.547Z</v>
+        <v>2026-10-13T12:49:30.632Z</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B85" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22033,116 +22033,116 @@
         <v>34</v>
       </c>
       <c r="H85" t="str">
-        <v>2026-10-12T18:40:27.007Z</v>
+        <v>2026-10-13T12:49:30.631Z</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B86" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C86" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D86">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E86">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F86">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G86">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H86" t="str">
-        <v>2026-10-12T18:40:27.006Z</v>
+        <v>2026-10-13T12:49:30.629Z</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>13-10-2026, 9:08:58 a. m.</v>
       </c>
       <c r="B87" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
       </c>
       <c r="C87" t="str">
-        <v>DropGO · generado</v>
+        <v>Manual</v>
       </c>
       <c r="D87">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E87">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F87">
         <v>0</v>
       </c>
       <c r="G87">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H87" t="str">
-        <v>2026-10-12T18:39:34.326Z</v>
+        <v>2026-10-13T12:08:58.547Z</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B88" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C88" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D88">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E88">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F88">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G88">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H88" t="str">
-        <v>2026-10-12T18:39:34.325Z</v>
+        <v>2026-10-12T18:40:27.007Z</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B89" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C89" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D89">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E89">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F89">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G89">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H89" t="str">
-        <v>2026-10-12T18:39:34.319Z</v>
+        <v>2026-10-12T18:40:27.006Z</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>12-10-2026, 3:39:18 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B90" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22151,10 +22151,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D90">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E90">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F90">
         <v>0</v>
@@ -22163,116 +22163,116 @@
         <v>25</v>
       </c>
       <c r="H90" t="str">
-        <v>2026-10-12T18:39:18.385Z</v>
+        <v>2026-10-12T18:39:34.326Z</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>12-10-2026, 12:05:40 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B91" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C91" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D91">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E91">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G91">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H91" t="str">
-        <v>2026-10-12T15:05:40.188Z</v>
+        <v>2026-10-12T18:39:34.325Z</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B92" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C92" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D92">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E92">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F92">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G92">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H92" t="str">
-        <v>2026-10-12T14:26:19.514Z</v>
+        <v>2026-10-12T18:39:34.319Z</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:18 p. m.</v>
       </c>
       <c r="B93" t="str">
-        <v>orders_export (6).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C93" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D93">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E93">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F93">
         <v>0</v>
       </c>
       <c r="G93">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H93" t="str">
-        <v>2026-10-12T14:26:19.513Z</v>
+        <v>2026-10-12T18:39:18.385Z</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 12:05:40 p. m.</v>
       </c>
       <c r="B94" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C94" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D94">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E94">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F94">
         <v>0</v>
       </c>
       <c r="G94">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H94" t="str">
-        <v>2026-10-12T14:24:55.059Z</v>
+        <v>2026-10-12T15:05:40.188Z</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B95" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22293,64 +22293,64 @@
         <v>25</v>
       </c>
       <c r="H95" t="str">
-        <v>2026-10-12T14:24:55.058Z</v>
+        <v>2026-10-12T14:26:19.514Z</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B96" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>orders_export (6).csv</v>
       </c>
       <c r="C96" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D96">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E96">
         <v>4</v>
       </c>
       <c r="F96">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G96">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H96" t="str">
-        <v>2026-10-12T14:24:55.057Z</v>
+        <v>2026-10-12T14:26:19.513Z</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>12-10-2026, 11:24:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B97" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C97" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D97">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F97">
         <v>0</v>
       </c>
       <c r="G97">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H97" t="str">
-        <v>2026-10-12T14:24:00.106Z</v>
+        <v>2026-10-12T14:24:55.059Z</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B98" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22362,73 +22362,73 @@
         <v>25</v>
       </c>
       <c r="E98">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F98">
         <v>0</v>
       </c>
       <c r="G98">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H98" t="str">
-        <v>2026-10-09T14:54:00.353Z</v>
+        <v>2026-10-12T14:24:55.058Z</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B99" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C99" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D99">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E99">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F99">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G99">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H99" t="str">
-        <v>2026-10-09T14:54:00.352Z</v>
+        <v>2026-10-12T14:24:55.057Z</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:00 a. m.</v>
       </c>
       <c r="B100" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C100" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D100">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E100">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F100">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G100">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H100" t="str">
-        <v>2026-10-09T14:54:00.347Z</v>
+        <v>2026-10-12T14:24:00.106Z</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>09-10-2026, 11:50:59 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B101" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22437,10 +22437,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D101">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E101">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F101">
         <v>0</v>
@@ -22449,64 +22449,64 @@
         <v>21</v>
       </c>
       <c r="H101" t="str">
-        <v>2026-10-09T14:50:59.695Z</v>
+        <v>2026-10-09T14:54:00.353Z</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B102" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C102" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D102">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F102">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G102">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H102" t="str">
-        <v>2026-10-09T14:28:16.404Z</v>
+        <v>2026-10-09T14:54:00.352Z</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B103" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C103" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D103">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E103">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F103">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G103">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H103" t="str">
-        <v>2026-10-09T14:28:16.403Z</v>
+        <v>2026-10-09T14:54:00.347Z</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>09-10-2026, 11:28:07 a. m.</v>
+        <v>09-10-2026, 11:50:59 a. m.</v>
       </c>
       <c r="B104" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22527,12 +22527,12 @@
         <v>21</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-10-09T14:28:07.531Z</v>
+        <v>2026-10-09T14:50:59.695Z</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B105" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22553,12 +22553,12 @@
         <v>21</v>
       </c>
       <c r="H105" t="str">
-        <v>2026-10-09T14:26:45.497Z</v>
+        <v>2026-10-09T14:28:16.404Z</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B106" t="str">
         <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
@@ -22579,21 +22579,21 @@
         <v>19</v>
       </c>
       <c r="H106" t="str">
-        <v>2026-10-09T14:26:45.495Z</v>
+        <v>2026-10-09T14:28:16.403Z</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:07 a. m.</v>
       </c>
       <c r="B107" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C107" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D107">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E107">
         <v>0</v>
@@ -22602,50 +22602,50 @@
         <v>0</v>
       </c>
       <c r="G107">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H107" t="str">
-        <v>2026-10-09T14:26:45.477Z</v>
+        <v>2026-10-09T14:28:07.531Z</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B108" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C108" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D108">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E108">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-10-09T14:25:43.607Z</v>
+        <v>2026-10-09T14:26:45.497Z</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B109" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C109" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D109">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E109">
         <v>0</v>
@@ -22654,36 +22654,36 @@
         <v>0</v>
       </c>
       <c r="G109">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H109" t="str">
-        <v>2026-10-09T14:25:43.606Z</v>
+        <v>2026-10-09T14:26:45.495Z</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B110" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C110" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D110">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F110">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G110">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H110" t="str">
-        <v>2026-10-09T14:25:43.605Z</v>
+        <v>2026-10-09T14:26:45.477Z</v>
       </c>
     </row>
     <row r="111">
@@ -22691,30 +22691,30 @@
         <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B111" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C111" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D111">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E111">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F111">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G111">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H111" t="str">
-        <v>2026-10-09T14:25:43.580Z</v>
+        <v>2026-10-09T14:25:43.607Z</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>09-10-2026, 11:23:53 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B112" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22735,111 +22735,111 @@
         <v>21</v>
       </c>
       <c r="H112" t="str">
-        <v>2026-10-09T14:23:53.263Z</v>
+        <v>2026-10-09T14:25:43.606Z</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>08-10-2026, 9:14:25 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B113" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C113" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D113">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E113">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F113">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G113">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H113" t="str">
-        <v>2026-10-08T12:14:25.917Z</v>
+        <v>2026-10-09T14:25:43.605Z</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B114" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C114" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D114">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E114">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G114">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H114" t="str">
-        <v>2026-10-08T11:22:18.060Z</v>
+        <v>2026-10-09T14:25:43.580Z</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:23:53 a. m.</v>
       </c>
       <c r="B115" t="str">
-        <v>orders_export (4).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C115" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D115">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E115">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F115">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G115">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H115" t="str">
-        <v>2026-10-08T11:22:18.059Z</v>
+        <v>2026-10-09T14:23:53.263Z</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>08-10-2026, 9:14:25 a. m.</v>
       </c>
       <c r="B116" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C116" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D116">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G116">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H116" t="str">
-        <v>2026-10-08T11:22:18.042Z</v>
+        <v>2026-10-08T12:14:25.917Z</v>
       </c>
     </row>
     <row r="117">
@@ -22847,108 +22847,108 @@
         <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B117" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C117" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D117">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E117">
         <v>2</v>
       </c>
       <c r="F117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G117">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H117" t="str">
-        <v>2026-10-08T11:22:18.032Z</v>
+        <v>2026-10-08T11:22:18.060Z</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>08-10-2026, 8:18:16 a. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B118" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (4).csv</v>
       </c>
       <c r="C118" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D118">
         <v>19</v>
       </c>
       <c r="E118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F118">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G118">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H118" t="str">
-        <v>2026-10-08T11:18:16.488Z</v>
+        <v>2026-10-08T11:22:18.059Z</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B119" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C119" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D119">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E119">
+        <v>2</v>
+      </c>
+      <c r="F119">
+        <v>1</v>
+      </c>
+      <c r="G119">
         <v>0</v>
       </c>
-      <c r="F119">
-        <v>0</v>
-      </c>
-      <c r="G119">
-        <v>19</v>
-      </c>
       <c r="H119" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.042Z</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B120" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C120" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D120">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E120">
         <v>2</v>
       </c>
       <c r="F120">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G120">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H120" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.032Z</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>07-10-2026, 8:20:41 p. m.</v>
+        <v>08-10-2026, 8:18:16 a. m.</v>
       </c>
       <c r="B121" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22969,64 +22969,64 @@
         <v>19</v>
       </c>
       <c r="H121" t="str">
-        <v>2026-10-07T23:20:41.390Z</v>
+        <v>2026-10-08T11:18:16.488Z</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B122" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
       </c>
       <c r="C122" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D122">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="E122">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F122">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G122">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H122" t="str">
-        <v>2026-10-07T17:47:17.199Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B123" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C123" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D123">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="E123">
         <v>0</v>
       </c>
       <c r="F123">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G123">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="H123" t="str">
-        <v>2026-10-07T17:47:17.198Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>07-10-2026, 2:46:47 p. m.</v>
+        <v>07-10-2026, 8:20:41 p. m.</v>
       </c>
       <c r="B124" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23047,12 +23047,12 @@
         <v>19</v>
       </c>
       <c r="H124" t="str">
-        <v>2026-10-07T17:46:47.954Z</v>
+        <v>2026-10-07T23:20:41.390Z</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>07-10-2026, 2:44:00 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B125" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23073,64 +23073,64 @@
         <v>19</v>
       </c>
       <c r="H125" t="str">
-        <v>2026-10-07T17:44:00.660Z</v>
+        <v>2026-10-07T17:47:17.199Z</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>07-10-2026, 2:27:43 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B126" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
       </c>
       <c r="C126" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D126">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E126">
         <v>0</v>
       </c>
       <c r="F126">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G126">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="H126" t="str">
-        <v>2026-10-07T17:27:43.517Z</v>
+        <v>2026-10-07T17:47:17.198Z</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:46:47 p. m.</v>
       </c>
       <c r="B127" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C127" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D127">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E127">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F127">
         <v>0</v>
       </c>
       <c r="G127">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H127" t="str">
-        <v>2026-10-07T17:26:50.382Z</v>
+        <v>2026-10-07T17:46:47.954Z</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:44:00 p. m.</v>
       </c>
       <c r="B128" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23142,21 +23142,21 @@
         <v>19</v>
       </c>
       <c r="E128">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F128">
         <v>0</v>
       </c>
       <c r="G128">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H128" t="str">
-        <v>2026-10-07T17:26:50.380Z</v>
+        <v>2026-10-07T17:44:00.660Z</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:27:43 p. m.</v>
       </c>
       <c r="B129" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23165,7 +23165,7 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D129">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E129">
         <v>0</v>
@@ -23174,41 +23174,41 @@
         <v>0</v>
       </c>
       <c r="G129">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H129" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:27:43.517Z</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B130" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C130" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D130">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="E130">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F130">
         <v>0</v>
       </c>
       <c r="G130">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H130" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:26:50.382Z</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B131" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23217,71 +23217,71 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D131">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E131">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F131">
         <v>0</v>
       </c>
       <c r="G131">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H131" t="str">
-        <v>2026-10-07T16:25:12.953Z</v>
+        <v>2026-10-07T17:26:50.380Z</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B132" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>ventas_por_canal_y_mes.xlsx</v>
       </c>
       <c r="C132" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas por canal y mes</v>
       </c>
       <c r="D132">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="E132">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F132">
         <v>0</v>
       </c>
       <c r="G132">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="H132" t="str">
-        <v>2026-10-07T16:25:12.950Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B133" t="str">
-        <v>orders_export (3).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C133" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D133">
         <v>18</v>
       </c>
       <c r="E133">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F133">
         <v>0</v>
       </c>
       <c r="G133">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H133" t="str">
-        <v>2026-10-07T16:25:12.939Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="134">
@@ -23289,25 +23289,25 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B134" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C134" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D134">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E134">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F134">
         <v>0</v>
       </c>
       <c r="G134">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H134" t="str">
-        <v>2026-10-07T16:25:12.924Z</v>
+        <v>2026-10-07T16:25:12.953Z</v>
       </c>
     </row>
     <row r="135">
@@ -23315,10 +23315,10 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B135" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C135" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D135">
         <v>19</v>
@@ -23333,142 +23333,220 @@
         <v>0</v>
       </c>
       <c r="H135" t="str">
-        <v>2026-10-07T16:25:12.851Z</v>
+        <v>2026-10-07T16:25:12.950Z</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>07-10-2026, 1:10:27 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B136" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>orders_export (3).csv</v>
       </c>
       <c r="C136" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D136">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E136">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F136">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G136">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="H136" t="str">
-        <v>2026-10-07T16:10:27.561Z</v>
+        <v>2026-10-07T16:25:12.939Z</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>07-10-2026, 12:20:36 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B137" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C137" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D137">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E137">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F137">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G137">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H137" t="str">
-        <v>2026-10-07T15:20:36.001Z</v>
+        <v>2026-10-07T16:25:12.924Z</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>07-10-2026, 12:20:35 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B138" t="str">
-        <v>varin_respaldo_2026-10-07.xlsx</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C138" t="str">
-        <v>Respaldo</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D138">
-        <v>322</v>
+        <v>19</v>
       </c>
       <c r="E138">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F138">
         <v>0</v>
       </c>
       <c r="G138">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H138" t="str">
-        <v>2026-10-07T15:20:35.967Z</v>
+        <v>2026-10-07T16:25:12.851Z</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>07-10-2026, 12:20:08 p. m.</v>
+        <v>07-10-2026, 1:10:27 p. m.</v>
       </c>
       <c r="B139" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C139" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D139">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E139">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="F139">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G139">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="H139" t="str">
-        <v>2026-10-07T15:20:08.547Z</v>
+        <v>2026-10-07T16:10:27.561Z</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
+        <v>07-10-2026, 12:20:36 p. m.</v>
+      </c>
+      <c r="B140" t="str">
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+      </c>
+      <c r="C140" t="str">
+        <v>Ventas Mercado Libre</v>
+      </c>
+      <c r="D140">
+        <v>92</v>
+      </c>
+      <c r="E140">
+        <v>1</v>
+      </c>
+      <c r="F140">
+        <v>5</v>
+      </c>
+      <c r="G140">
+        <v>86</v>
+      </c>
+      <c r="H140" t="str">
+        <v>2026-10-07T15:20:36.001Z</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>07-10-2026, 12:20:35 p. m.</v>
+      </c>
+      <c r="B141" t="str">
+        <v>varin_respaldo_2026-10-07.xlsx</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Respaldo</v>
+      </c>
+      <c r="D141">
+        <v>322</v>
+      </c>
+      <c r="E141">
+        <v>190</v>
+      </c>
+      <c r="F141">
+        <v>0</v>
+      </c>
+      <c r="G141">
+        <v>132</v>
+      </c>
+      <c r="H141" t="str">
+        <v>2026-10-07T15:20:35.967Z</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
         <v>07-10-2026, 12:20:08 p. m.</v>
       </c>
-      <c r="B140" t="str">
+      <c r="B142" t="str">
+        <v>ventas_por_canal_y_mes.xlsx</v>
+      </c>
+      <c r="C142" t="str">
+        <v>Ventas por canal y mes</v>
+      </c>
+      <c r="D142">
+        <v>118</v>
+      </c>
+      <c r="E142">
+        <v>118</v>
+      </c>
+      <c r="F142">
+        <v>0</v>
+      </c>
+      <c r="G142">
+        <v>0</v>
+      </c>
+      <c r="H142" t="str">
+        <v>2026-10-07T15:20:08.547Z</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>07-10-2026, 12:20:08 p. m.</v>
+      </c>
+      <c r="B143" t="str">
         <v>Varin_Movimientos_DropGO_2026-10-01_al_2026-10-06.xlsx</v>
       </c>
-      <c r="C140" t="str">
+      <c r="C143" t="str">
         <v>Movimientos DropGO</v>
       </c>
-      <c r="D140">
+      <c r="D143">
         <v>14</v>
       </c>
-      <c r="E140">
+      <c r="E143">
         <v>14</v>
       </c>
-      <c r="F140">
+      <c r="F143">
         <v>0</v>
       </c>
-      <c r="G140">
+      <c r="G143">
         <v>0</v>
       </c>
-      <c r="H140" t="str">
+      <c r="H143" t="str">
         <v>2026-10-07T15:20:08.525Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H140"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H143"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -26918,7 +26996,7 @@
         <v>Generado</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-27T22:11:10.937Z</v>
+        <v>2026-10-28T10:56:11.261Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Datos Varin 2026-10-28 22:40
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20415,7 +20415,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H153"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -20454,42 +20454,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:21 p. m.</v>
       </c>
       <c r="B2" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C2" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D2">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-28T22:34:33.117Z</v>
+        <v>2026-10-28T22:40:21.045Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:21 p. m.</v>
       </c>
       <c r="B3" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
       </c>
       <c r="C3" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D3">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -20498,67 +20498,67 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-10-28T22:34:33.116Z</v>
+        <v>2026-10-28T22:40:21.044Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:04 p. m.</v>
       </c>
       <c r="B4" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C4" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D4">
-        <v>153</v>
+        <v>55</v>
       </c>
       <c r="E4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>147</v>
+        <v>55</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-10-28T22:34:33.114Z</v>
+        <v>2026-10-28T22:40:04.272Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>28-10-2026, 7:34:12 p. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B5" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C5" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D5">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-10-28T22:34:12.755Z</v>
+        <v>2026-10-28T22:34:33.117Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B6" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20570,73 +20570,73 @@
         <v>55</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-10-28T10:57:11.638Z</v>
+        <v>2026-10-28T22:34:33.116Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B7" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
       </c>
       <c r="C7" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="E7">
         <v>5</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>147</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-10-28T10:57:11.636Z</v>
+        <v>2026-10-28T22:34:33.114Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:12 p. m.</v>
       </c>
       <c r="B8" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C8" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D8">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-10-28T10:57:11.632Z</v>
+        <v>2026-10-28T22:34:12.755Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>28-10-2026, 7:56:06 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B9" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20645,10 +20645,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D9">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -20657,64 +20657,64 @@
         <v>50</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-10-28T10:56:06.328Z</v>
+        <v>2026-10-28T10:57:11.638Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>28-10-2026, 7:56:06 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B10" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C10" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D10">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-10-28T10:56:06.326Z</v>
+        <v>2026-10-28T10:57:11.636Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>28-10-2026, 7:53:38 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B11" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C11" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D11">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="G11">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-10-28T10:53:38.820Z</v>
+        <v>2026-10-28T10:57:11.632Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B12" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20735,38 +20735,38 @@
         <v>50</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-10-27T22:11:05.716Z</v>
+        <v>2026-10-28T10:56:06.328Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B13" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
       </c>
       <c r="C13" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D13">
-        <v>148</v>
+        <v>69</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>144</v>
+        <v>69</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-10-27T22:11:05.714Z</v>
+        <v>2026-10-28T10:56:06.326Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>27-10-2026, 7:10:39 p. m.</v>
+        <v>28-10-2026, 7:53:38 a. m.</v>
       </c>
       <c r="B14" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20787,12 +20787,12 @@
         <v>50</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-10-27T22:10:39.288Z</v>
+        <v>2026-10-28T10:53:38.820Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B15" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20804,68 +20804,68 @@
         <v>50</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15">
         <v>0</v>
       </c>
       <c r="G15">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-10-27T12:40:01.215Z</v>
+        <v>2026-10-27T22:11:05.716Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B16" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
       </c>
       <c r="C16" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D16">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G16">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-10-27T12:40:01.212Z</v>
+        <v>2026-10-27T22:11:05.714Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:10:39 p. m.</v>
       </c>
       <c r="B17" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C17" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-10-27T12:40:01.116Z</v>
+        <v>2026-10-27T22:10:39.288Z</v>
       </c>
     </row>
     <row r="18">
@@ -20873,186 +20873,186 @@
         <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B18" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C18" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E18">
         <v>1</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-10-27T12:40:01.113Z</v>
+        <v>2026-10-27T12:40:01.215Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B19" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C19" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>147</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-10-27T12:39:46.660Z</v>
+        <v>2026-10-27T12:40:01.212Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B20" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C20" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D20">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
         <v>0</v>
       </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
-        <v>49</v>
-      </c>
       <c r="H20" t="str">
-        <v>2026-10-27T12:39:46.656Z</v>
+        <v>2026-10-27T12:40:01.116Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B21" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C21" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D21">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E21">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
         <v>0</v>
       </c>
-      <c r="G21">
-        <v>3</v>
-      </c>
       <c r="H21" t="str">
-        <v>2026-10-27T12:35:13.606Z</v>
+        <v>2026-10-27T12:40:01.113Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B22" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C22" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D22">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-27T12:35:13.605Z</v>
+        <v>2026-10-27T12:39:46.660Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B23" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C23" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D23">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="E23">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F23">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>131</v>
+        <v>49</v>
       </c>
       <c r="H23" t="str">
-        <v>2026-10-27T12:35:13.604Z</v>
+        <v>2026-10-27T12:39:46.656Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>27-10-2026, 9:34:54 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B24" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C24" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D24">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H24" t="str">
-        <v>2026-10-27T12:34:54.468Z</v>
+        <v>2026-10-27T12:35:13.606Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B25" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21064,177 +21064,177 @@
         <v>49</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-10-26T12:06:47.126Z</v>
+        <v>2026-10-27T12:35:13.605Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B26" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
       </c>
       <c r="C26" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D26">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="H26" t="str">
-        <v>2026-10-26T12:06:47.123Z</v>
+        <v>2026-10-27T12:35:13.604Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:34:54 a. m.</v>
       </c>
       <c r="B27" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C27" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-10-26T12:06:47.118Z</v>
+        <v>2026-10-27T12:34:54.468Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B28" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C28" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D28">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E28">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-10-26T12:05:32.699Z</v>
+        <v>2026-10-26T12:06:47.126Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B29" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C29" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D29">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29">
         <v>0</v>
       </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-      <c r="G29">
-        <v>48</v>
-      </c>
       <c r="H29" t="str">
-        <v>2026-10-26T12:05:32.697Z</v>
+        <v>2026-10-26T12:06:47.123Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B30" t="str">
-        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C30" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D30">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E30">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30">
         <v>0</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-10-26T12:05:32.692Z</v>
+        <v>2026-10-26T12:06:47.118Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>25-10-2026, 12:10:56 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B31" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C31" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D31">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-10-25T15:10:56.412Z</v>
+        <v>2026-10-26T12:05:32.699Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B32" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21255,38 +21255,38 @@
         <v>48</v>
       </c>
       <c r="H32" t="str">
-        <v>2026-10-23T22:12:12.477Z</v>
+        <v>2026-10-26T12:05:32.697Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B33" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
+        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
       </c>
       <c r="C33" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D33">
-        <v>135</v>
+        <v>6</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-10-23T22:12:12.476Z</v>
+        <v>2026-10-26T12:05:32.692Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>23-10-2026, 7:11:53 p. m.</v>
+        <v>25-10-2026, 12:10:56 p. m.</v>
       </c>
       <c r="B34" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21307,12 +21307,12 @@
         <v>48</v>
       </c>
       <c r="H34" t="str">
-        <v>2026-10-23T22:11:53.140Z</v>
+        <v>2026-10-25T15:10:56.412Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B35" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21333,15 +21333,15 @@
         <v>48</v>
       </c>
       <c r="H35" t="str">
-        <v>2026-10-23T13:17:56.047Z</v>
+        <v>2026-10-23T22:12:12.477Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B36" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C36" t="str">
         <v>Ventas Mercado Libre</v>
@@ -21359,12 +21359,12 @@
         <v>135</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-10-23T13:17:56.044Z</v>
+        <v>2026-10-23T22:12:12.476Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>23-10-2026, 9:52:55 a. m.</v>
+        <v>23-10-2026, 7:11:53 p. m.</v>
       </c>
       <c r="B37" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21385,12 +21385,12 @@
         <v>48</v>
       </c>
       <c r="H37" t="str">
-        <v>2026-10-23T12:52:55.551Z</v>
+        <v>2026-10-23T22:11:53.140Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>23-10-2026, 9:50:04 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B38" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21411,38 +21411,38 @@
         <v>48</v>
       </c>
       <c r="H38" t="str">
-        <v>2026-10-23T12:50:04.195Z</v>
+        <v>2026-10-23T13:17:56.047Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B39" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C39" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D39">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="H39" t="str">
-        <v>2026-10-23T12:37:54.995Z</v>
+        <v>2026-10-23T13:17:56.044Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:52:55 a. m.</v>
       </c>
       <c r="B40" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21463,64 +21463,64 @@
         <v>48</v>
       </c>
       <c r="H40" t="str">
-        <v>2026-10-23T12:37:54.994Z</v>
+        <v>2026-10-23T12:52:55.551Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:50:04 a. m.</v>
       </c>
       <c r="B41" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C41" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D41">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G41">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="H41" t="str">
-        <v>2026-10-23T12:37:54.992Z</v>
+        <v>2026-10-23T12:50:04.195Z</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>23-10-2026, 9:37:27 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B42" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C42" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D42">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42">
         <v>0</v>
       </c>
       <c r="G42">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H42" t="str">
-        <v>2026-10-23T12:37:27.533Z</v>
+        <v>2026-10-23T12:37:54.995Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>23-10-2026, 9:34:31 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B43" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21541,64 +21541,64 @@
         <v>48</v>
       </c>
       <c r="H43" t="str">
-        <v>2026-10-23T12:34:31.611Z</v>
+        <v>2026-10-23T12:37:54.994Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>23-10-2026, 9:19:14 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B44" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C44" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D44">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G44">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="H44" t="str">
-        <v>2026-10-23T12:19:14.833Z</v>
+        <v>2026-10-23T12:37:54.992Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:37:27 a. m.</v>
       </c>
       <c r="B45" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C45" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D45">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E45">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H45" t="str">
-        <v>2026-10-22T11:51:13.535Z</v>
+        <v>2026-10-23T12:37:27.533Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:34:31 a. m.</v>
       </c>
       <c r="B46" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21619,38 +21619,38 @@
         <v>48</v>
       </c>
       <c r="H46" t="str">
-        <v>2026-10-22T11:51:13.534Z</v>
+        <v>2026-10-23T12:34:31.611Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:19:14 a. m.</v>
       </c>
       <c r="B47" t="str">
-        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C47" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D47">
-        <v>134</v>
+        <v>48</v>
       </c>
       <c r="E47">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G47">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-10-22T11:51:13.529Z</v>
+        <v>2026-10-23T12:19:14.833Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B48" t="str">
         <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
@@ -21659,10 +21659,10 @@
         <v>Full ML · generado</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F48">
         <v>0</v>
@@ -21671,12 +21671,12 @@
         <v>2</v>
       </c>
       <c r="H48" t="str">
-        <v>2026-10-21T11:58:09.619Z</v>
+        <v>2026-10-22T11:51:13.535Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B49" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21688,42 +21688,42 @@
         <v>48</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F49">
         <v>0</v>
       </c>
       <c r="G49">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H49" t="str">
-        <v>2026-10-21T11:58:09.618Z</v>
+        <v>2026-10-22T11:51:13.534Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B50" t="str">
-        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
+        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
       </c>
       <c r="C50" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D50">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F50">
         <v>5</v>
       </c>
       <c r="G50">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H50" t="str">
-        <v>2026-10-21T11:58:09.614Z</v>
+        <v>2026-10-22T11:51:13.529Z</v>
       </c>
     </row>
     <row r="51">
@@ -21731,25 +21731,25 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B51" t="str">
-        <v>ventas-report (11).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C51" t="str">
-        <v>DropGO · ventas</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D51">
+        <v>4</v>
+      </c>
+      <c r="E51">
         <v>2</v>
-      </c>
-      <c r="E51">
-        <v>1</v>
       </c>
       <c r="F51">
         <v>0</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H51" t="str">
-        <v>2026-10-21T11:58:09.533Z</v>
+        <v>2026-10-21T11:58:09.619Z</v>
       </c>
     </row>
     <row r="52">
@@ -21757,13 +21757,13 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B52" t="str">
-        <v>picking-report (11).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C52" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D52">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E52">
         <v>1</v>
@@ -21772,88 +21772,88 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H52" t="str">
-        <v>2026-10-21T11:58:09.530Z</v>
+        <v>2026-10-21T11:58:09.618Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B53" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
       </c>
       <c r="C53" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D53">
-        <v>47</v>
+        <v>128</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G53">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="H53" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.614Z</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B54" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>ventas-report (11).xlsx</v>
       </c>
       <c r="C54" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D54">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E54">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H54" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.533Z</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B55" t="str">
-        <v>ventas-report (10).xlsx</v>
+        <v>picking-report (11).xlsx</v>
       </c>
       <c r="C55" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D55">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E55">
         <v>1</v>
       </c>
       <c r="F55">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G55">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H55" t="str">
-        <v>2026-10-20T12:36:20.899Z</v>
+        <v>2026-10-21T11:58:09.530Z</v>
       </c>
     </row>
     <row r="56">
@@ -21861,25 +21861,25 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B56" t="str">
-        <v>picking-report (10).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C56" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D56">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="E56">
         <v>1</v>
       </c>
       <c r="F56">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G56">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="H56" t="str">
-        <v>2026-10-20T12:36:20.895Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="57">
@@ -21887,212 +21887,212 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B57" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C57" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D57">
-        <v>126</v>
+        <v>5</v>
       </c>
       <c r="E57">
         <v>3</v>
       </c>
       <c r="F57">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G57">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="H57" t="str">
-        <v>2026-10-20T12:36:20.890Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>20-10-2026, 9:34:26 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B58" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (10).xlsx</v>
       </c>
       <c r="C58" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D58">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="E58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G58">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-20T12:34:26.210Z</v>
+        <v>2026-10-20T12:36:20.899Z</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B59" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (10).xlsx</v>
       </c>
       <c r="C59" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D59">
+        <v>11</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59">
+        <v>3</v>
+      </c>
+      <c r="G59">
         <v>7</v>
       </c>
-      <c r="E59">
-        <v>5</v>
-      </c>
-      <c r="F59">
-        <v>1</v>
-      </c>
-      <c r="G59">
-        <v>2</v>
-      </c>
       <c r="H59" t="str">
-        <v>2026-10-19T12:21:51.769Z</v>
+        <v>2026-10-20T12:36:20.895Z</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B60" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C60" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D60">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E60">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F60">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G60">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="H60" t="str">
-        <v>2026-10-19T12:21:51.768Z</v>
+        <v>2026-10-20T12:36:20.890Z</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:34:26 a. m.</v>
       </c>
       <c r="B61" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C61" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D61">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E61">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F61">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G61">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H61" t="str">
-        <v>2026-10-19T12:21:51.766Z</v>
+        <v>2026-10-20T12:34:26.210Z</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B62" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C62" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D62">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E62">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G62">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H62" t="str">
-        <v>2026-10-19T12:20:51.921Z</v>
+        <v>2026-10-19T12:21:51.769Z</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B63" t="str">
-        <v>picking-report (9).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C63" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D63">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E63">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F63">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G63">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="H63" t="str">
-        <v>2026-10-19T12:20:51.919Z</v>
+        <v>2026-10-19T12:21:51.768Z</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B64" t="str">
-        <v>ventas-report (9).xlsx</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
       </c>
       <c r="C64" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D64">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="E64">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H64" t="str">
-        <v>2026-10-19T12:20:51.913Z</v>
+        <v>2026-10-19T12:21:51.766Z</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>19-10-2026, 9:12:06 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B65" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22101,10 +22101,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D65">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F65">
         <v>0</v>
@@ -22113,229 +22113,229 @@
         <v>37</v>
       </c>
       <c r="H65" t="str">
-        <v>2026-10-19T12:12:06.575Z</v>
+        <v>2026-10-19T12:20:51.921Z</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B66" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (9).xlsx</v>
       </c>
       <c r="C66" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D66">
+        <v>14</v>
+      </c>
+      <c r="E66">
+        <v>7</v>
+      </c>
+      <c r="F66">
         <v>5</v>
-      </c>
-      <c r="E66">
-        <v>3</v>
-      </c>
-      <c r="F66">
-        <v>0</v>
       </c>
       <c r="G66">
         <v>2</v>
       </c>
       <c r="H66" t="str">
-        <v>2026-10-16T12:37:12.832Z</v>
+        <v>2026-10-19T12:20:51.919Z</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B67" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (9).xlsx</v>
       </c>
       <c r="C67" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D67">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F67">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G67">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H67" t="str">
-        <v>2026-10-16T12:37:12.831Z</v>
+        <v>2026-10-19T12:20:51.913Z</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:12:06 a. m.</v>
       </c>
       <c r="B68" t="str">
-        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C68" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D68">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F68">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G68">
         <v>37</v>
       </c>
       <c r="H68" t="str">
-        <v>2026-10-16T12:37:12.827Z</v>
+        <v>2026-10-19T12:12:06.575Z</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B69" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C69" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D69">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F69">
         <v>0</v>
       </c>
       <c r="G69">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H69" t="str">
-        <v>2026-10-16T11:52:26.043Z</v>
+        <v>2026-10-16T12:37:12.832Z</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B70" t="str">
-        <v>picking-report (8).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C70" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D70">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E70">
         <v>0</v>
       </c>
       <c r="F70">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H70" t="str">
-        <v>2026-10-16T11:52:26.040Z</v>
+        <v>2026-10-16T12:37:12.831Z</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B71" t="str">
-        <v>ventas-report (8).xlsx</v>
+        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
       </c>
       <c r="C71" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D71">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F71">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G71">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-10-16T11:52:26.034Z</v>
+        <v>2026-10-16T12:37:12.827Z</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B72" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C72" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D72">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H72" t="str">
-        <v>2026-10-15T12:11:36.404Z</v>
+        <v>2026-10-16T11:52:26.043Z</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B73" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (8).xlsx</v>
       </c>
       <c r="C73" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D73">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E73">
         <v>0</v>
       </c>
       <c r="F73">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G73">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H73" t="str">
-        <v>2026-10-15T12:11:36.403Z</v>
+        <v>2026-10-16T11:52:26.040Z</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B74" t="str">
-        <v>ventas-report (7).xlsx</v>
+        <v>ventas-report (8).xlsx</v>
       </c>
       <c r="C74" t="str">
         <v>DropGO · ventas</v>
       </c>
       <c r="D74">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -22344,10 +22344,10 @@
         <v>1</v>
       </c>
       <c r="G74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H74" t="str">
-        <v>2026-10-15T12:11:36.401Z</v>
+        <v>2026-10-16T11:52:26.034Z</v>
       </c>
     </row>
     <row r="75">
@@ -22355,25 +22355,25 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B75" t="str">
-        <v>picking-report (7).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C75" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D75">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E75">
+        <v>2</v>
+      </c>
+      <c r="F75">
         <v>0</v>
-      </c>
-      <c r="F75">
-        <v>1</v>
       </c>
       <c r="G75">
         <v>2</v>
       </c>
       <c r="H75" t="str">
-        <v>2026-10-15T12:11:36.397Z</v>
+        <v>2026-10-15T12:11:36.404Z</v>
       </c>
     </row>
     <row r="76">
@@ -22381,143 +22381,143 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B76" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C76" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D76">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E76">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F76">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G76">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="H76" t="str">
-        <v>2026-10-15T12:11:36.389Z</v>
+        <v>2026-10-15T12:11:36.403Z</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>14-10-2026, 10:42:32 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B77" t="str">
-        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
+        <v>ventas-report (7).xlsx</v>
       </c>
       <c r="C77" t="str">
-        <v>Manual</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E77">
         <v>0</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H77" t="str">
-        <v>2026-10-14T13:42:32.444Z</v>
+        <v>2026-10-15T12:11:36.401Z</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B78" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (7).xlsx</v>
       </c>
       <c r="C78" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D78">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>1</v>
+      </c>
+      <c r="G78">
         <v>2</v>
       </c>
-      <c r="F78">
-        <v>0</v>
-      </c>
-      <c r="G78">
-        <v>35</v>
-      </c>
       <c r="H78" t="str">
-        <v>2026-10-14T13:41:21.926Z</v>
+        <v>2026-10-15T12:11:36.397Z</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B79" t="str">
-        <v>picking-report (6).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
       </c>
       <c r="C79" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D79">
-        <v>7</v>
+        <v>114</v>
       </c>
       <c r="E79">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G79">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="H79" t="str">
-        <v>2026-10-14T13:41:21.925Z</v>
+        <v>2026-10-15T12:11:36.389Z</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>14-10-2026, 10:42:32 a. m.</v>
       </c>
       <c r="B80" t="str">
-        <v>ventas-report (6).xlsx</v>
+        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
       </c>
       <c r="C80" t="str">
-        <v>DropGO · ventas</v>
+        <v>Manual</v>
       </c>
       <c r="D80">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E80">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F80">
         <v>0</v>
       </c>
       <c r="G80">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H80" t="str">
-        <v>2026-10-14T13:41:21.921Z</v>
+        <v>2026-10-14T13:42:32.444Z</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B81" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C81" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D81">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E81">
         <v>2</v>
@@ -22526,93 +22526,93 @@
         <v>0</v>
       </c>
       <c r="G81">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="H81" t="str">
-        <v>2026-10-14T13:40:03.191Z</v>
+        <v>2026-10-14T13:41:21.926Z</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B82" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (6).xlsx</v>
       </c>
       <c r="C82" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D82">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F82">
         <v>0</v>
       </c>
       <c r="G82">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H82" t="str">
-        <v>2026-10-14T13:40:03.190Z</v>
+        <v>2026-10-14T13:41:21.925Z</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B83" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
+        <v>ventas-report (6).xlsx</v>
       </c>
       <c r="C83" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D83">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="E83">
         <v>3</v>
       </c>
       <c r="F83">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G83">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="H83" t="str">
-        <v>2026-10-14T13:40:03.188Z</v>
+        <v>2026-10-14T13:41:21.921Z</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>14-10-2026, 10:39:50 a. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B84" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C84" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D84">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F84">
         <v>0</v>
       </c>
       <c r="G84">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H84" t="str">
-        <v>2026-10-14T13:39:50.407Z</v>
+        <v>2026-10-14T13:40:03.191Z</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B85" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22633,38 +22633,38 @@
         <v>35</v>
       </c>
       <c r="H85" t="str">
-        <v>2026-10-13T16:19:36.490Z</v>
+        <v>2026-10-14T13:40:03.190Z</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B86" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
       </c>
       <c r="C86" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D86">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E86">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F86">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G86">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H86" t="str">
-        <v>2026-10-13T16:19:36.488Z</v>
+        <v>2026-10-14T13:40:03.188Z</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>13-10-2026, 11:56:40 a. m.</v>
+        <v>14-10-2026, 10:39:50 a. m.</v>
       </c>
       <c r="B87" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22685,12 +22685,12 @@
         <v>35</v>
       </c>
       <c r="H87" t="str">
-        <v>2026-10-13T14:56:40.589Z</v>
+        <v>2026-10-14T13:39:50.407Z</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B88" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22702,177 +22702,177 @@
         <v>35</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F88">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G88">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H88" t="str">
-        <v>2026-10-13T14:44:42.285Z</v>
+        <v>2026-10-13T16:19:36.490Z</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B89" t="str">
-        <v>picking-report (5).xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C89" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D89">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="E89">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F89">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G89">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="H89" t="str">
-        <v>2026-10-13T14:44:42.284Z</v>
+        <v>2026-10-13T16:19:36.488Z</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 11:56:40 a. m.</v>
       </c>
       <c r="B90" t="str">
-        <v>ventas-report (5).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C90" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D90">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E90">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F90">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G90">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H90" t="str">
-        <v>2026-10-13T14:44:42.280Z</v>
+        <v>2026-10-13T14:56:40.589Z</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B91" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C91" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D91">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="E91">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H91" t="str">
-        <v>2026-10-13T12:49:30.632Z</v>
+        <v>2026-10-13T14:44:42.285Z</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B92" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (5).xlsx</v>
       </c>
       <c r="C92" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D92">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E92">
+        <v>2</v>
+      </c>
+      <c r="F92">
+        <v>6</v>
+      </c>
+      <c r="G92">
         <v>0</v>
       </c>
-      <c r="F92">
-        <v>0</v>
-      </c>
-      <c r="G92">
-        <v>34</v>
-      </c>
       <c r="H92" t="str">
-        <v>2026-10-13T12:49:30.631Z</v>
+        <v>2026-10-13T14:44:42.284Z</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B93" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>ventas-report (5).xlsx</v>
       </c>
       <c r="C93" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D93">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="E93">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F93">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G93">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H93" t="str">
-        <v>2026-10-13T12:49:30.629Z</v>
+        <v>2026-10-13T14:44:42.280Z</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>13-10-2026, 9:08:58 a. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B94" t="str">
-        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C94" t="str">
-        <v>Manual</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D94">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E94">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F94">
         <v>0</v>
       </c>
       <c r="G94">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H94" t="str">
-        <v>2026-10-13T12:08:58.547Z</v>
+        <v>2026-10-13T12:49:30.632Z</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B95" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22893,116 +22893,116 @@
         <v>34</v>
       </c>
       <c r="H95" t="str">
-        <v>2026-10-12T18:40:27.007Z</v>
+        <v>2026-10-13T12:49:30.631Z</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B96" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C96" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D96">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F96">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G96">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H96" t="str">
-        <v>2026-10-12T18:40:27.006Z</v>
+        <v>2026-10-13T12:49:30.629Z</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>13-10-2026, 9:08:58 a. m.</v>
       </c>
       <c r="B97" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
       </c>
       <c r="C97" t="str">
-        <v>DropGO · generado</v>
+        <v>Manual</v>
       </c>
       <c r="D97">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E97">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F97">
         <v>0</v>
       </c>
       <c r="G97">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H97" t="str">
-        <v>2026-10-12T18:39:34.326Z</v>
+        <v>2026-10-13T12:08:58.547Z</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B98" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C98" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D98">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E98">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F98">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G98">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H98" t="str">
-        <v>2026-10-12T18:39:34.325Z</v>
+        <v>2026-10-12T18:40:27.007Z</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B99" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C99" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D99">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E99">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F99">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G99">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H99" t="str">
-        <v>2026-10-12T18:39:34.319Z</v>
+        <v>2026-10-12T18:40:27.006Z</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>12-10-2026, 3:39:18 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B100" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23011,10 +23011,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D100">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E100">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F100">
         <v>0</v>
@@ -23023,116 +23023,116 @@
         <v>25</v>
       </c>
       <c r="H100" t="str">
-        <v>2026-10-12T18:39:18.385Z</v>
+        <v>2026-10-12T18:39:34.326Z</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>12-10-2026, 12:05:40 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B101" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C101" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D101">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E101">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F101">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G101">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H101" t="str">
-        <v>2026-10-12T15:05:40.188Z</v>
+        <v>2026-10-12T18:39:34.325Z</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B102" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C102" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D102">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F102">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G102">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H102" t="str">
-        <v>2026-10-12T14:26:19.514Z</v>
+        <v>2026-10-12T18:39:34.319Z</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:18 p. m.</v>
       </c>
       <c r="B103" t="str">
-        <v>orders_export (6).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C103" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D103">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E103">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F103">
         <v>0</v>
       </c>
       <c r="G103">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H103" t="str">
-        <v>2026-10-12T14:26:19.513Z</v>
+        <v>2026-10-12T18:39:18.385Z</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 12:05:40 p. m.</v>
       </c>
       <c r="B104" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C104" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D104">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E104">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F104">
         <v>0</v>
       </c>
       <c r="G104">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-10-12T14:24:55.059Z</v>
+        <v>2026-10-12T15:05:40.188Z</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B105" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23153,64 +23153,64 @@
         <v>25</v>
       </c>
       <c r="H105" t="str">
-        <v>2026-10-12T14:24:55.058Z</v>
+        <v>2026-10-12T14:26:19.514Z</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B106" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>orders_export (6).csv</v>
       </c>
       <c r="C106" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D106">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E106">
         <v>4</v>
       </c>
       <c r="F106">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G106">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H106" t="str">
-        <v>2026-10-12T14:24:55.057Z</v>
+        <v>2026-10-12T14:26:19.513Z</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>12-10-2026, 11:24:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B107" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C107" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D107">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E107">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F107">
         <v>0</v>
       </c>
       <c r="G107">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H107" t="str">
-        <v>2026-10-12T14:24:00.106Z</v>
+        <v>2026-10-12T14:24:55.059Z</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B108" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23222,73 +23222,73 @@
         <v>25</v>
       </c>
       <c r="E108">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-10-09T14:54:00.353Z</v>
+        <v>2026-10-12T14:24:55.058Z</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B109" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C109" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D109">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E109">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F109">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G109">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H109" t="str">
-        <v>2026-10-09T14:54:00.352Z</v>
+        <v>2026-10-12T14:24:55.057Z</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:00 a. m.</v>
       </c>
       <c r="B110" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C110" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D110">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E110">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F110">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G110">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H110" t="str">
-        <v>2026-10-09T14:54:00.347Z</v>
+        <v>2026-10-12T14:24:00.106Z</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>09-10-2026, 11:50:59 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B111" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23297,10 +23297,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D111">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F111">
         <v>0</v>
@@ -23309,64 +23309,64 @@
         <v>21</v>
       </c>
       <c r="H111" t="str">
-        <v>2026-10-09T14:50:59.695Z</v>
+        <v>2026-10-09T14:54:00.353Z</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B112" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C112" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D112">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E112">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F112">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G112">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H112" t="str">
-        <v>2026-10-09T14:28:16.404Z</v>
+        <v>2026-10-09T14:54:00.352Z</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B113" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C113" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D113">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E113">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H113" t="str">
-        <v>2026-10-09T14:28:16.403Z</v>
+        <v>2026-10-09T14:54:00.347Z</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>09-10-2026, 11:28:07 a. m.</v>
+        <v>09-10-2026, 11:50:59 a. m.</v>
       </c>
       <c r="B114" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23387,12 +23387,12 @@
         <v>21</v>
       </c>
       <c r="H114" t="str">
-        <v>2026-10-09T14:28:07.531Z</v>
+        <v>2026-10-09T14:50:59.695Z</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B115" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23413,12 +23413,12 @@
         <v>21</v>
       </c>
       <c r="H115" t="str">
-        <v>2026-10-09T14:26:45.497Z</v>
+        <v>2026-10-09T14:28:16.404Z</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B116" t="str">
         <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
@@ -23439,21 +23439,21 @@
         <v>19</v>
       </c>
       <c r="H116" t="str">
-        <v>2026-10-09T14:26:45.495Z</v>
+        <v>2026-10-09T14:28:16.403Z</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:07 a. m.</v>
       </c>
       <c r="B117" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C117" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D117">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E117">
         <v>0</v>
@@ -23462,50 +23462,50 @@
         <v>0</v>
       </c>
       <c r="G117">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H117" t="str">
-        <v>2026-10-09T14:26:45.477Z</v>
+        <v>2026-10-09T14:28:07.531Z</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B118" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C118" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D118">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F118">
         <v>0</v>
       </c>
       <c r="G118">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H118" t="str">
-        <v>2026-10-09T14:25:43.607Z</v>
+        <v>2026-10-09T14:26:45.497Z</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B119" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C119" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D119">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E119">
         <v>0</v>
@@ -23514,36 +23514,36 @@
         <v>0</v>
       </c>
       <c r="G119">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H119" t="str">
-        <v>2026-10-09T14:25:43.606Z</v>
+        <v>2026-10-09T14:26:45.495Z</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B120" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C120" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D120">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E120">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F120">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G120">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H120" t="str">
-        <v>2026-10-09T14:25:43.605Z</v>
+        <v>2026-10-09T14:26:45.477Z</v>
       </c>
     </row>
     <row r="121">
@@ -23551,30 +23551,30 @@
         <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B121" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C121" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D121">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G121">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H121" t="str">
-        <v>2026-10-09T14:25:43.580Z</v>
+        <v>2026-10-09T14:25:43.607Z</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>09-10-2026, 11:23:53 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B122" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23595,111 +23595,111 @@
         <v>21</v>
       </c>
       <c r="H122" t="str">
-        <v>2026-10-09T14:23:53.263Z</v>
+        <v>2026-10-09T14:25:43.606Z</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>08-10-2026, 9:14:25 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B123" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C123" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D123">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E123">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F123">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G123">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H123" t="str">
-        <v>2026-10-08T12:14:25.917Z</v>
+        <v>2026-10-09T14:25:43.605Z</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B124" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C124" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D124">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E124">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F124">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G124">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H124" t="str">
-        <v>2026-10-08T11:22:18.060Z</v>
+        <v>2026-10-09T14:25:43.580Z</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:23:53 a. m.</v>
       </c>
       <c r="B125" t="str">
-        <v>orders_export (4).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C125" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D125">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F125">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G125">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H125" t="str">
-        <v>2026-10-08T11:22:18.059Z</v>
+        <v>2026-10-09T14:23:53.263Z</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>08-10-2026, 9:14:25 a. m.</v>
       </c>
       <c r="B126" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C126" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D126">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E126">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F126">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G126">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H126" t="str">
-        <v>2026-10-08T11:22:18.042Z</v>
+        <v>2026-10-08T12:14:25.917Z</v>
       </c>
     </row>
     <row r="127">
@@ -23707,108 +23707,108 @@
         <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B127" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C127" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D127">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E127">
         <v>2</v>
       </c>
       <c r="F127">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G127">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H127" t="str">
-        <v>2026-10-08T11:22:18.032Z</v>
+        <v>2026-10-08T11:22:18.060Z</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>08-10-2026, 8:18:16 a. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B128" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (4).csv</v>
       </c>
       <c r="C128" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D128">
         <v>19</v>
       </c>
       <c r="E128">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F128">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G128">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H128" t="str">
-        <v>2026-10-08T11:18:16.488Z</v>
+        <v>2026-10-08T11:22:18.059Z</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B129" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C129" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D129">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E129">
         <v>2</v>
       </c>
       <c r="F129">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G129">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H129" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.042Z</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B130" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C130" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D130">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E130">
+        <v>2</v>
+      </c>
+      <c r="F130">
+        <v>1</v>
+      </c>
+      <c r="G130">
         <v>0</v>
       </c>
-      <c r="F130">
-        <v>0</v>
-      </c>
-      <c r="G130">
-        <v>19</v>
-      </c>
       <c r="H130" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.032Z</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>07-10-2026, 8:20:41 p. m.</v>
+        <v>08-10-2026, 8:18:16 a. m.</v>
       </c>
       <c r="B131" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23829,64 +23829,64 @@
         <v>19</v>
       </c>
       <c r="H131" t="str">
-        <v>2026-10-07T23:20:41.390Z</v>
+        <v>2026-10-08T11:18:16.488Z</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B132" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
       </c>
       <c r="C132" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D132">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="E132">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F132">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G132">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H132" t="str">
-        <v>2026-10-07T17:47:17.199Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B133" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C133" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D133">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="E133">
         <v>0</v>
       </c>
       <c r="F133">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G133">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="H133" t="str">
-        <v>2026-10-07T17:47:17.198Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>07-10-2026, 2:46:47 p. m.</v>
+        <v>07-10-2026, 8:20:41 p. m.</v>
       </c>
       <c r="B134" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23907,12 +23907,12 @@
         <v>19</v>
       </c>
       <c r="H134" t="str">
-        <v>2026-10-07T17:46:47.954Z</v>
+        <v>2026-10-07T23:20:41.390Z</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>07-10-2026, 2:44:00 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B135" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23933,64 +23933,64 @@
         <v>19</v>
       </c>
       <c r="H135" t="str">
-        <v>2026-10-07T17:44:00.660Z</v>
+        <v>2026-10-07T17:47:17.199Z</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>07-10-2026, 2:27:43 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B136" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
       </c>
       <c r="C136" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D136">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E136">
         <v>0</v>
       </c>
       <c r="F136">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G136">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="H136" t="str">
-        <v>2026-10-07T17:27:43.517Z</v>
+        <v>2026-10-07T17:47:17.198Z</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:46:47 p. m.</v>
       </c>
       <c r="B137" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C137" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D137">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E137">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F137">
         <v>0</v>
       </c>
       <c r="G137">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H137" t="str">
-        <v>2026-10-07T17:26:50.382Z</v>
+        <v>2026-10-07T17:46:47.954Z</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:44:00 p. m.</v>
       </c>
       <c r="B138" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24002,30 +24002,30 @@
         <v>19</v>
       </c>
       <c r="E138">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F138">
         <v>0</v>
       </c>
       <c r="G138">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H138" t="str">
-        <v>2026-10-07T17:26:50.380Z</v>
+        <v>2026-10-07T17:44:00.660Z</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:27:43 p. m.</v>
       </c>
       <c r="B139" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C139" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D139">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="E139">
         <v>0</v>
@@ -24034,41 +24034,41 @@
         <v>0</v>
       </c>
       <c r="G139">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="H139" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:27:43.517Z</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B140" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C140" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D140">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E140">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F140">
         <v>0</v>
       </c>
       <c r="G140">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H140" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:26:50.382Z</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B141" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24077,71 +24077,71 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D141">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E141">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F141">
         <v>0</v>
       </c>
       <c r="G141">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H141" t="str">
-        <v>2026-10-07T16:25:12.953Z</v>
+        <v>2026-10-07T17:26:50.380Z</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B142" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>ventas_por_canal_y_mes.xlsx</v>
       </c>
       <c r="C142" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas por canal y mes</v>
       </c>
       <c r="D142">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="E142">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F142">
         <v>0</v>
       </c>
       <c r="G142">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="H142" t="str">
-        <v>2026-10-07T16:25:12.950Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B143" t="str">
-        <v>orders_export (3).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C143" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D143">
         <v>18</v>
       </c>
       <c r="E143">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F143">
         <v>0</v>
       </c>
       <c r="G143">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H143" t="str">
-        <v>2026-10-07T16:25:12.939Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="144">
@@ -24149,25 +24149,25 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B144" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C144" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D144">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E144">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F144">
         <v>0</v>
       </c>
       <c r="G144">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H144" t="str">
-        <v>2026-10-07T16:25:12.924Z</v>
+        <v>2026-10-07T16:25:12.953Z</v>
       </c>
     </row>
     <row r="145">
@@ -24175,10 +24175,10 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B145" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C145" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D145">
         <v>19</v>
@@ -24193,142 +24193,220 @@
         <v>0</v>
       </c>
       <c r="H145" t="str">
-        <v>2026-10-07T16:25:12.851Z</v>
+        <v>2026-10-07T16:25:12.950Z</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>07-10-2026, 1:10:27 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B146" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>orders_export (3).csv</v>
       </c>
       <c r="C146" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D146">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E146">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F146">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G146">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="H146" t="str">
-        <v>2026-10-07T16:10:27.561Z</v>
+        <v>2026-10-07T16:25:12.939Z</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>07-10-2026, 12:20:36 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B147" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C147" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D147">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E147">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F147">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G147">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H147" t="str">
-        <v>2026-10-07T15:20:36.001Z</v>
+        <v>2026-10-07T16:25:12.924Z</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>07-10-2026, 12:20:35 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B148" t="str">
-        <v>varin_respaldo_2026-10-07.xlsx</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C148" t="str">
-        <v>Respaldo</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D148">
-        <v>322</v>
+        <v>19</v>
       </c>
       <c r="E148">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F148">
         <v>0</v>
       </c>
       <c r="G148">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H148" t="str">
-        <v>2026-10-07T15:20:35.967Z</v>
+        <v>2026-10-07T16:25:12.851Z</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>07-10-2026, 12:20:08 p. m.</v>
+        <v>07-10-2026, 1:10:27 p. m.</v>
       </c>
       <c r="B149" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C149" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D149">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E149">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="F149">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G149">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="H149" t="str">
-        <v>2026-10-07T15:20:08.547Z</v>
+        <v>2026-10-07T16:10:27.561Z</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
+        <v>07-10-2026, 12:20:36 p. m.</v>
+      </c>
+      <c r="B150" t="str">
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Ventas Mercado Libre</v>
+      </c>
+      <c r="D150">
+        <v>92</v>
+      </c>
+      <c r="E150">
+        <v>1</v>
+      </c>
+      <c r="F150">
+        <v>5</v>
+      </c>
+      <c r="G150">
+        <v>86</v>
+      </c>
+      <c r="H150" t="str">
+        <v>2026-10-07T15:20:36.001Z</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>07-10-2026, 12:20:35 p. m.</v>
+      </c>
+      <c r="B151" t="str">
+        <v>varin_respaldo_2026-10-07.xlsx</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Respaldo</v>
+      </c>
+      <c r="D151">
+        <v>322</v>
+      </c>
+      <c r="E151">
+        <v>190</v>
+      </c>
+      <c r="F151">
+        <v>0</v>
+      </c>
+      <c r="G151">
+        <v>132</v>
+      </c>
+      <c r="H151" t="str">
+        <v>2026-10-07T15:20:35.967Z</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
         <v>07-10-2026, 12:20:08 p. m.</v>
       </c>
-      <c r="B150" t="str">
+      <c r="B152" t="str">
+        <v>ventas_por_canal_y_mes.xlsx</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Ventas por canal y mes</v>
+      </c>
+      <c r="D152">
+        <v>118</v>
+      </c>
+      <c r="E152">
+        <v>118</v>
+      </c>
+      <c r="F152">
+        <v>0</v>
+      </c>
+      <c r="G152">
+        <v>0</v>
+      </c>
+      <c r="H152" t="str">
+        <v>2026-10-07T15:20:08.547Z</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>07-10-2026, 12:20:08 p. m.</v>
+      </c>
+      <c r="B153" t="str">
         <v>Varin_Movimientos_DropGO_2026-10-01_al_2026-10-06.xlsx</v>
       </c>
-      <c r="C150" t="str">
+      <c r="C153" t="str">
         <v>Movimientos DropGO</v>
       </c>
-      <c r="D150">
+      <c r="D153">
         <v>14</v>
       </c>
-      <c r="E150">
+      <c r="E153">
         <v>14</v>
       </c>
-      <c r="F150">
+      <c r="F153">
         <v>0</v>
       </c>
-      <c r="G150">
+      <c r="G153">
         <v>0</v>
       </c>
-      <c r="H150" t="str">
+      <c r="H153" t="str">
         <v>2026-10-07T15:20:08.525Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H150"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H153"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -28121,7 +28199,7 @@
         <v>Generado</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-28T22:34:38.094Z</v>
+        <v>2026-10-28T22:40:25.898Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Datos Varin 2026-10-28 22:43
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20415,7 +20415,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H156"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -20454,7 +20454,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>28-10-2026, 7:40:21 p. m.</v>
+        <v>28-10-2026, 7:43:14 p. m.</v>
       </c>
       <c r="B2" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20475,99 +20475,99 @@
         <v>55</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-28T22:40:21.045Z</v>
+        <v>2026-10-28T22:43:14.280Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>28-10-2026, 7:40:21 p. m.</v>
+        <v>28-10-2026, 7:43:14 p. m.</v>
       </c>
       <c r="B3" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C3" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D3">
-        <v>153</v>
+        <v>5</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>153</v>
+        <v>1</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-10-28T22:40:21.044Z</v>
+        <v>2026-10-28T22:43:14.278Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>28-10-2026, 7:40:04 p. m.</v>
+        <v>28-10-2026, 7:43:14 p. m.</v>
       </c>
       <c r="B4" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C4" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D4">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-10-28T22:40:04.272Z</v>
+        <v>2026-10-28T22:43:14.269Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:21 p. m.</v>
       </c>
       <c r="B5" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C5" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-10-28T22:34:33.117Z</v>
+        <v>2026-10-28T22:40:21.045Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:21 p. m.</v>
       </c>
       <c r="B6" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
       </c>
       <c r="C6" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -20576,67 +20576,67 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-10-28T22:34:33.116Z</v>
+        <v>2026-10-28T22:40:21.044Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:04 p. m.</v>
       </c>
       <c r="B7" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C7" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D7">
-        <v>153</v>
+        <v>55</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>147</v>
+        <v>55</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-10-28T22:34:33.114Z</v>
+        <v>2026-10-28T22:40:04.272Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>28-10-2026, 7:34:12 p. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B8" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C8" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D8">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-10-28T22:34:12.755Z</v>
+        <v>2026-10-28T22:34:33.117Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B9" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20648,73 +20648,73 @@
         <v>55</v>
       </c>
       <c r="E9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-10-28T10:57:11.638Z</v>
+        <v>2026-10-28T22:34:33.116Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B10" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
       </c>
       <c r="C10" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D10">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>147</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-10-28T10:57:11.636Z</v>
+        <v>2026-10-28T22:34:33.114Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:12 p. m.</v>
       </c>
       <c r="B11" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C11" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="E11">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-10-28T10:57:11.632Z</v>
+        <v>2026-10-28T22:34:12.755Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>28-10-2026, 7:56:06 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B12" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20723,10 +20723,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -20735,64 +20735,64 @@
         <v>50</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-10-28T10:56:06.328Z</v>
+        <v>2026-10-28T10:57:11.638Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>28-10-2026, 7:56:06 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B13" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C13" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D13">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
       <c r="G13">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-10-28T10:56:06.326Z</v>
+        <v>2026-10-28T10:57:11.636Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>28-10-2026, 7:53:38 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B14" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C14" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D14">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-10-28T10:53:38.820Z</v>
+        <v>2026-10-28T10:57:11.632Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B15" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20813,38 +20813,38 @@
         <v>50</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-10-27T22:11:05.716Z</v>
+        <v>2026-10-28T10:56:06.328Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B16" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
       </c>
       <c r="C16" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D16">
-        <v>148</v>
+        <v>69</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>144</v>
+        <v>69</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-10-27T22:11:05.714Z</v>
+        <v>2026-10-28T10:56:06.326Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>27-10-2026, 7:10:39 p. m.</v>
+        <v>28-10-2026, 7:53:38 a. m.</v>
       </c>
       <c r="B17" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20865,12 +20865,12 @@
         <v>50</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-10-27T22:10:39.288Z</v>
+        <v>2026-10-28T10:53:38.820Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B18" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -20882,68 +20882,68 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-10-27T12:40:01.215Z</v>
+        <v>2026-10-27T22:11:05.716Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B19" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
       </c>
       <c r="C19" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D19">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G19">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-10-27T12:40:01.212Z</v>
+        <v>2026-10-27T22:11:05.714Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:10:39 p. m.</v>
       </c>
       <c r="B20" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C20" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-10-27T12:40:01.116Z</v>
+        <v>2026-10-27T22:10:39.288Z</v>
       </c>
     </row>
     <row r="21">
@@ -20951,186 +20951,186 @@
         <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B21" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C21" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-10-27T12:40:01.113Z</v>
+        <v>2026-10-27T12:40:01.215Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B22" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C22" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D22">
-        <v>4</v>
+        <v>147</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-27T12:39:46.660Z</v>
+        <v>2026-10-27T12:40:01.212Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B23" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C23" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D23">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
         <v>0</v>
       </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
-        <v>49</v>
-      </c>
       <c r="H23" t="str">
-        <v>2026-10-27T12:39:46.656Z</v>
+        <v>2026-10-27T12:40:01.116Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B24" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C24" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D24">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E24">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
         <v>0</v>
       </c>
-      <c r="G24">
-        <v>3</v>
-      </c>
       <c r="H24" t="str">
-        <v>2026-10-27T12:35:13.606Z</v>
+        <v>2026-10-27T12:40:01.113Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B25" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C25" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D25">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-10-27T12:35:13.605Z</v>
+        <v>2026-10-27T12:39:46.660Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B26" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C26" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D26">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="E26">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>131</v>
+        <v>49</v>
       </c>
       <c r="H26" t="str">
-        <v>2026-10-27T12:35:13.604Z</v>
+        <v>2026-10-27T12:39:46.656Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>27-10-2026, 9:34:54 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B27" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C27" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D27">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
       <c r="G27">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-10-27T12:34:54.468Z</v>
+        <v>2026-10-27T12:35:13.606Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B28" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21142,177 +21142,177 @@
         <v>49</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
       <c r="G28">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-10-26T12:06:47.126Z</v>
+        <v>2026-10-27T12:35:13.605Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B29" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
       </c>
       <c r="C29" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F29">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="H29" t="str">
-        <v>2026-10-26T12:06:47.123Z</v>
+        <v>2026-10-27T12:35:13.604Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:34:54 a. m.</v>
       </c>
       <c r="B30" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C30" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-10-26T12:06:47.118Z</v>
+        <v>2026-10-27T12:34:54.468Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B31" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C31" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D31">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E31">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-10-26T12:05:32.699Z</v>
+        <v>2026-10-26T12:06:47.126Z</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B32" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C32" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D32">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>2</v>
+      </c>
+      <c r="G32">
         <v>0</v>
       </c>
-      <c r="F32">
-        <v>0</v>
-      </c>
-      <c r="G32">
-        <v>48</v>
-      </c>
       <c r="H32" t="str">
-        <v>2026-10-26T12:05:32.697Z</v>
+        <v>2026-10-26T12:06:47.123Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B33" t="str">
-        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C33" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D33">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E33">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33">
         <v>0</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-10-26T12:05:32.692Z</v>
+        <v>2026-10-26T12:06:47.118Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>25-10-2026, 12:10:56 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B34" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C34" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D34">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F34">
         <v>0</v>
       </c>
       <c r="G34">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H34" t="str">
-        <v>2026-10-25T15:10:56.412Z</v>
+        <v>2026-10-26T12:05:32.699Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B35" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21333,38 +21333,38 @@
         <v>48</v>
       </c>
       <c r="H35" t="str">
-        <v>2026-10-23T22:12:12.477Z</v>
+        <v>2026-10-26T12:05:32.697Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B36" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
+        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
       </c>
       <c r="C36" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D36">
-        <v>135</v>
+        <v>6</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-10-23T22:12:12.476Z</v>
+        <v>2026-10-26T12:05:32.692Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>23-10-2026, 7:11:53 p. m.</v>
+        <v>25-10-2026, 12:10:56 p. m.</v>
       </c>
       <c r="B37" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21385,12 +21385,12 @@
         <v>48</v>
       </c>
       <c r="H37" t="str">
-        <v>2026-10-23T22:11:53.140Z</v>
+        <v>2026-10-25T15:10:56.412Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B38" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21411,15 +21411,15 @@
         <v>48</v>
       </c>
       <c r="H38" t="str">
-        <v>2026-10-23T13:17:56.047Z</v>
+        <v>2026-10-23T22:12:12.477Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B39" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C39" t="str">
         <v>Ventas Mercado Libre</v>
@@ -21437,12 +21437,12 @@
         <v>135</v>
       </c>
       <c r="H39" t="str">
-        <v>2026-10-23T13:17:56.044Z</v>
+        <v>2026-10-23T22:12:12.476Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>23-10-2026, 9:52:55 a. m.</v>
+        <v>23-10-2026, 7:11:53 p. m.</v>
       </c>
       <c r="B40" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21463,12 +21463,12 @@
         <v>48</v>
       </c>
       <c r="H40" t="str">
-        <v>2026-10-23T12:52:55.551Z</v>
+        <v>2026-10-23T22:11:53.140Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>23-10-2026, 9:50:04 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B41" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21489,38 +21489,38 @@
         <v>48</v>
       </c>
       <c r="H41" t="str">
-        <v>2026-10-23T12:50:04.195Z</v>
+        <v>2026-10-23T13:17:56.047Z</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B42" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C42" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D42">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42">
         <v>0</v>
       </c>
       <c r="G42">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="H42" t="str">
-        <v>2026-10-23T12:37:54.995Z</v>
+        <v>2026-10-23T13:17:56.044Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:52:55 a. m.</v>
       </c>
       <c r="B43" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21541,64 +21541,64 @@
         <v>48</v>
       </c>
       <c r="H43" t="str">
-        <v>2026-10-23T12:37:54.994Z</v>
+        <v>2026-10-23T12:52:55.551Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:50:04 a. m.</v>
       </c>
       <c r="B44" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C44" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D44">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G44">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="H44" t="str">
-        <v>2026-10-23T12:37:54.992Z</v>
+        <v>2026-10-23T12:50:04.195Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>23-10-2026, 9:37:27 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B45" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C45" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D45">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
       <c r="G45">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H45" t="str">
-        <v>2026-10-23T12:37:27.533Z</v>
+        <v>2026-10-23T12:37:54.995Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>23-10-2026, 9:34:31 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B46" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21619,64 +21619,64 @@
         <v>48</v>
       </c>
       <c r="H46" t="str">
-        <v>2026-10-23T12:34:31.611Z</v>
+        <v>2026-10-23T12:37:54.994Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>23-10-2026, 9:19:14 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B47" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C47" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D47">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G47">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-10-23T12:19:14.833Z</v>
+        <v>2026-10-23T12:37:54.992Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:37:27 a. m.</v>
       </c>
       <c r="B48" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C48" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D48">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E48">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F48">
         <v>0</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H48" t="str">
-        <v>2026-10-22T11:51:13.535Z</v>
+        <v>2026-10-23T12:37:27.533Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:34:31 a. m.</v>
       </c>
       <c r="B49" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21697,38 +21697,38 @@
         <v>48</v>
       </c>
       <c r="H49" t="str">
-        <v>2026-10-22T11:51:13.534Z</v>
+        <v>2026-10-23T12:34:31.611Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:19:14 a. m.</v>
       </c>
       <c r="B50" t="str">
-        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C50" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D50">
-        <v>134</v>
+        <v>48</v>
       </c>
       <c r="E50">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F50">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G50">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="H50" t="str">
-        <v>2026-10-22T11:51:13.529Z</v>
+        <v>2026-10-23T12:19:14.833Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B51" t="str">
         <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
@@ -21737,10 +21737,10 @@
         <v>Full ML · generado</v>
       </c>
       <c r="D51">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F51">
         <v>0</v>
@@ -21749,12 +21749,12 @@
         <v>2</v>
       </c>
       <c r="H51" t="str">
-        <v>2026-10-21T11:58:09.619Z</v>
+        <v>2026-10-22T11:51:13.535Z</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B52" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21766,42 +21766,42 @@
         <v>48</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52">
         <v>0</v>
       </c>
       <c r="G52">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H52" t="str">
-        <v>2026-10-21T11:58:09.618Z</v>
+        <v>2026-10-22T11:51:13.534Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B53" t="str">
-        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
+        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
       </c>
       <c r="C53" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D53">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F53">
         <v>5</v>
       </c>
       <c r="G53">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H53" t="str">
-        <v>2026-10-21T11:58:09.614Z</v>
+        <v>2026-10-22T11:51:13.529Z</v>
       </c>
     </row>
     <row r="54">
@@ -21809,25 +21809,25 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B54" t="str">
-        <v>ventas-report (11).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C54" t="str">
-        <v>DropGO · ventas</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D54">
+        <v>4</v>
+      </c>
+      <c r="E54">
         <v>2</v>
-      </c>
-      <c r="E54">
-        <v>1</v>
       </c>
       <c r="F54">
         <v>0</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H54" t="str">
-        <v>2026-10-21T11:58:09.533Z</v>
+        <v>2026-10-21T11:58:09.619Z</v>
       </c>
     </row>
     <row r="55">
@@ -21835,13 +21835,13 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B55" t="str">
-        <v>picking-report (11).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C55" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D55">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -21850,88 +21850,88 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H55" t="str">
-        <v>2026-10-21T11:58:09.530Z</v>
+        <v>2026-10-21T11:58:09.618Z</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B56" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
       </c>
       <c r="C56" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D56">
-        <v>47</v>
+        <v>128</v>
       </c>
       <c r="E56">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G56">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="H56" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.614Z</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B57" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>ventas-report (11).xlsx</v>
       </c>
       <c r="C57" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D57">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57">
         <v>0</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H57" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.533Z</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B58" t="str">
-        <v>ventas-report (10).xlsx</v>
+        <v>picking-report (11).xlsx</v>
       </c>
       <c r="C58" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D58">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E58">
         <v>1</v>
       </c>
       <c r="F58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G58">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-20T12:36:20.899Z</v>
+        <v>2026-10-21T11:58:09.530Z</v>
       </c>
     </row>
     <row r="59">
@@ -21939,25 +21939,25 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B59" t="str">
-        <v>picking-report (10).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C59" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D59">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="E59">
         <v>1</v>
       </c>
       <c r="F59">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="H59" t="str">
-        <v>2026-10-20T12:36:20.895Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="60">
@@ -21965,212 +21965,212 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B60" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C60" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D60">
-        <v>126</v>
+        <v>5</v>
       </c>
       <c r="E60">
         <v>3</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G60">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="H60" t="str">
-        <v>2026-10-20T12:36:20.890Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>20-10-2026, 9:34:26 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B61" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (10).xlsx</v>
       </c>
       <c r="C61" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D61">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="E61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G61">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="H61" t="str">
-        <v>2026-10-20T12:34:26.210Z</v>
+        <v>2026-10-20T12:36:20.899Z</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B62" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (10).xlsx</v>
       </c>
       <c r="C62" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D62">
+        <v>11</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62">
+        <v>3</v>
+      </c>
+      <c r="G62">
         <v>7</v>
       </c>
-      <c r="E62">
-        <v>5</v>
-      </c>
-      <c r="F62">
-        <v>1</v>
-      </c>
-      <c r="G62">
-        <v>2</v>
-      </c>
       <c r="H62" t="str">
-        <v>2026-10-19T12:21:51.769Z</v>
+        <v>2026-10-20T12:36:20.895Z</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B63" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C63" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D63">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E63">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F63">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G63">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="H63" t="str">
-        <v>2026-10-19T12:21:51.768Z</v>
+        <v>2026-10-20T12:36:20.890Z</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:34:26 a. m.</v>
       </c>
       <c r="B64" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C64" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D64">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E64">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F64">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G64">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H64" t="str">
-        <v>2026-10-19T12:21:51.766Z</v>
+        <v>2026-10-20T12:34:26.210Z</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B65" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C65" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D65">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E65">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H65" t="str">
-        <v>2026-10-19T12:20:51.921Z</v>
+        <v>2026-10-19T12:21:51.769Z</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B66" t="str">
-        <v>picking-report (9).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C66" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D66">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E66">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="H66" t="str">
-        <v>2026-10-19T12:20:51.919Z</v>
+        <v>2026-10-19T12:21:51.768Z</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B67" t="str">
-        <v>ventas-report (9).xlsx</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
       </c>
       <c r="C67" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D67">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="E67">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F67">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G67">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H67" t="str">
-        <v>2026-10-19T12:20:51.913Z</v>
+        <v>2026-10-19T12:21:51.766Z</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>19-10-2026, 9:12:06 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B68" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22179,10 +22179,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D68">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F68">
         <v>0</v>
@@ -22191,229 +22191,229 @@
         <v>37</v>
       </c>
       <c r="H68" t="str">
-        <v>2026-10-19T12:12:06.575Z</v>
+        <v>2026-10-19T12:20:51.921Z</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B69" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (9).xlsx</v>
       </c>
       <c r="C69" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D69">
+        <v>14</v>
+      </c>
+      <c r="E69">
+        <v>7</v>
+      </c>
+      <c r="F69">
         <v>5</v>
-      </c>
-      <c r="E69">
-        <v>3</v>
-      </c>
-      <c r="F69">
-        <v>0</v>
       </c>
       <c r="G69">
         <v>2</v>
       </c>
       <c r="H69" t="str">
-        <v>2026-10-16T12:37:12.832Z</v>
+        <v>2026-10-19T12:20:51.919Z</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B70" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (9).xlsx</v>
       </c>
       <c r="C70" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D70">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F70">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G70">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H70" t="str">
-        <v>2026-10-16T12:37:12.831Z</v>
+        <v>2026-10-19T12:20:51.913Z</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:12:06 a. m.</v>
       </c>
       <c r="B71" t="str">
-        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C71" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D71">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E71">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F71">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G71">
         <v>37</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-10-16T12:37:12.827Z</v>
+        <v>2026-10-19T12:12:06.575Z</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B72" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C72" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D72">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F72">
         <v>0</v>
       </c>
       <c r="G72">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H72" t="str">
-        <v>2026-10-16T11:52:26.043Z</v>
+        <v>2026-10-16T12:37:12.832Z</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B73" t="str">
-        <v>picking-report (8).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C73" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D73">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E73">
         <v>0</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G73">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H73" t="str">
-        <v>2026-10-16T11:52:26.040Z</v>
+        <v>2026-10-16T12:37:12.831Z</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B74" t="str">
-        <v>ventas-report (8).xlsx</v>
+        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
       </c>
       <c r="C74" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D74">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F74">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G74">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H74" t="str">
-        <v>2026-10-16T11:52:26.034Z</v>
+        <v>2026-10-16T12:37:12.827Z</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B75" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C75" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D75">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F75">
         <v>0</v>
       </c>
       <c r="G75">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H75" t="str">
-        <v>2026-10-15T12:11:36.404Z</v>
+        <v>2026-10-16T11:52:26.043Z</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B76" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (8).xlsx</v>
       </c>
       <c r="C76" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D76">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E76">
         <v>0</v>
       </c>
       <c r="F76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G76">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H76" t="str">
-        <v>2026-10-15T12:11:36.403Z</v>
+        <v>2026-10-16T11:52:26.040Z</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B77" t="str">
-        <v>ventas-report (7).xlsx</v>
+        <v>ventas-report (8).xlsx</v>
       </c>
       <c r="C77" t="str">
         <v>DropGO · ventas</v>
       </c>
       <c r="D77">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -22422,10 +22422,10 @@
         <v>1</v>
       </c>
       <c r="G77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H77" t="str">
-        <v>2026-10-15T12:11:36.401Z</v>
+        <v>2026-10-16T11:52:26.034Z</v>
       </c>
     </row>
     <row r="78">
@@ -22433,25 +22433,25 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B78" t="str">
-        <v>picking-report (7).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C78" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D78">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E78">
+        <v>2</v>
+      </c>
+      <c r="F78">
         <v>0</v>
-      </c>
-      <c r="F78">
-        <v>1</v>
       </c>
       <c r="G78">
         <v>2</v>
       </c>
       <c r="H78" t="str">
-        <v>2026-10-15T12:11:36.397Z</v>
+        <v>2026-10-15T12:11:36.404Z</v>
       </c>
     </row>
     <row r="79">
@@ -22459,143 +22459,143 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B79" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C79" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D79">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F79">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="H79" t="str">
-        <v>2026-10-15T12:11:36.389Z</v>
+        <v>2026-10-15T12:11:36.403Z</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>14-10-2026, 10:42:32 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B80" t="str">
-        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
+        <v>ventas-report (7).xlsx</v>
       </c>
       <c r="C80" t="str">
-        <v>Manual</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E80">
         <v>0</v>
       </c>
       <c r="F80">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G80">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H80" t="str">
-        <v>2026-10-14T13:42:32.444Z</v>
+        <v>2026-10-15T12:11:36.401Z</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B81" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (7).xlsx</v>
       </c>
       <c r="C81" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D81">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>1</v>
+      </c>
+      <c r="G81">
         <v>2</v>
       </c>
-      <c r="F81">
-        <v>0</v>
-      </c>
-      <c r="G81">
-        <v>35</v>
-      </c>
       <c r="H81" t="str">
-        <v>2026-10-14T13:41:21.926Z</v>
+        <v>2026-10-15T12:11:36.397Z</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B82" t="str">
-        <v>picking-report (6).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
       </c>
       <c r="C82" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D82">
-        <v>7</v>
+        <v>114</v>
       </c>
       <c r="E82">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F82">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G82">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="H82" t="str">
-        <v>2026-10-14T13:41:21.925Z</v>
+        <v>2026-10-15T12:11:36.389Z</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>14-10-2026, 10:42:32 a. m.</v>
       </c>
       <c r="B83" t="str">
-        <v>ventas-report (6).xlsx</v>
+        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
       </c>
       <c r="C83" t="str">
-        <v>DropGO · ventas</v>
+        <v>Manual</v>
       </c>
       <c r="D83">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E83">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F83">
         <v>0</v>
       </c>
       <c r="G83">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H83" t="str">
-        <v>2026-10-14T13:41:21.921Z</v>
+        <v>2026-10-14T13:42:32.444Z</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B84" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C84" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D84">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E84">
         <v>2</v>
@@ -22604,93 +22604,93 @@
         <v>0</v>
       </c>
       <c r="G84">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="H84" t="str">
-        <v>2026-10-14T13:40:03.191Z</v>
+        <v>2026-10-14T13:41:21.926Z</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B85" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (6).xlsx</v>
       </c>
       <c r="C85" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D85">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F85">
         <v>0</v>
       </c>
       <c r="G85">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H85" t="str">
-        <v>2026-10-14T13:40:03.190Z</v>
+        <v>2026-10-14T13:41:21.925Z</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B86" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
+        <v>ventas-report (6).xlsx</v>
       </c>
       <c r="C86" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D86">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="E86">
         <v>3</v>
       </c>
       <c r="F86">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G86">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="H86" t="str">
-        <v>2026-10-14T13:40:03.188Z</v>
+        <v>2026-10-14T13:41:21.921Z</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>14-10-2026, 10:39:50 a. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B87" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C87" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D87">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E87">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F87">
         <v>0</v>
       </c>
       <c r="G87">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H87" t="str">
-        <v>2026-10-14T13:39:50.407Z</v>
+        <v>2026-10-14T13:40:03.191Z</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B88" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22711,38 +22711,38 @@
         <v>35</v>
       </c>
       <c r="H88" t="str">
-        <v>2026-10-13T16:19:36.490Z</v>
+        <v>2026-10-14T13:40:03.190Z</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B89" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
       </c>
       <c r="C89" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D89">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E89">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F89">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G89">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H89" t="str">
-        <v>2026-10-13T16:19:36.488Z</v>
+        <v>2026-10-14T13:40:03.188Z</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>13-10-2026, 11:56:40 a. m.</v>
+        <v>14-10-2026, 10:39:50 a. m.</v>
       </c>
       <c r="B90" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22763,12 +22763,12 @@
         <v>35</v>
       </c>
       <c r="H90" t="str">
-        <v>2026-10-13T14:56:40.589Z</v>
+        <v>2026-10-14T13:39:50.407Z</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B91" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22780,177 +22780,177 @@
         <v>35</v>
       </c>
       <c r="E91">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F91">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G91">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H91" t="str">
-        <v>2026-10-13T14:44:42.285Z</v>
+        <v>2026-10-13T16:19:36.490Z</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B92" t="str">
-        <v>picking-report (5).xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C92" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D92">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="E92">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F92">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G92">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="H92" t="str">
-        <v>2026-10-13T14:44:42.284Z</v>
+        <v>2026-10-13T16:19:36.488Z</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 11:56:40 a. m.</v>
       </c>
       <c r="B93" t="str">
-        <v>ventas-report (5).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C93" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D93">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E93">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F93">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G93">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H93" t="str">
-        <v>2026-10-13T14:44:42.280Z</v>
+        <v>2026-10-13T14:56:40.589Z</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B94" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C94" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D94">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="E94">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F94">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H94" t="str">
-        <v>2026-10-13T12:49:30.632Z</v>
+        <v>2026-10-13T14:44:42.285Z</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B95" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (5).xlsx</v>
       </c>
       <c r="C95" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D95">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E95">
+        <v>2</v>
+      </c>
+      <c r="F95">
+        <v>6</v>
+      </c>
+      <c r="G95">
         <v>0</v>
       </c>
-      <c r="F95">
-        <v>0</v>
-      </c>
-      <c r="G95">
-        <v>34</v>
-      </c>
       <c r="H95" t="str">
-        <v>2026-10-13T12:49:30.631Z</v>
+        <v>2026-10-13T14:44:42.284Z</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B96" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>ventas-report (5).xlsx</v>
       </c>
       <c r="C96" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D96">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="E96">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F96">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G96">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H96" t="str">
-        <v>2026-10-13T12:49:30.629Z</v>
+        <v>2026-10-13T14:44:42.280Z</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>13-10-2026, 9:08:58 a. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B97" t="str">
-        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C97" t="str">
-        <v>Manual</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D97">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F97">
         <v>0</v>
       </c>
       <c r="G97">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H97" t="str">
-        <v>2026-10-13T12:08:58.547Z</v>
+        <v>2026-10-13T12:49:30.632Z</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B98" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22971,116 +22971,116 @@
         <v>34</v>
       </c>
       <c r="H98" t="str">
-        <v>2026-10-12T18:40:27.007Z</v>
+        <v>2026-10-13T12:49:30.631Z</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B99" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C99" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D99">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E99">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F99">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G99">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H99" t="str">
-        <v>2026-10-12T18:40:27.006Z</v>
+        <v>2026-10-13T12:49:30.629Z</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>13-10-2026, 9:08:58 a. m.</v>
       </c>
       <c r="B100" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
       </c>
       <c r="C100" t="str">
-        <v>DropGO · generado</v>
+        <v>Manual</v>
       </c>
       <c r="D100">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E100">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F100">
         <v>0</v>
       </c>
       <c r="G100">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H100" t="str">
-        <v>2026-10-12T18:39:34.326Z</v>
+        <v>2026-10-13T12:08:58.547Z</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B101" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C101" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D101">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E101">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F101">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G101">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H101" t="str">
-        <v>2026-10-12T18:39:34.325Z</v>
+        <v>2026-10-12T18:40:27.007Z</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B102" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C102" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D102">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E102">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F102">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G102">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H102" t="str">
-        <v>2026-10-12T18:39:34.319Z</v>
+        <v>2026-10-12T18:40:27.006Z</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>12-10-2026, 3:39:18 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B103" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23089,10 +23089,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D103">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E103">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F103">
         <v>0</v>
@@ -23101,116 +23101,116 @@
         <v>25</v>
       </c>
       <c r="H103" t="str">
-        <v>2026-10-12T18:39:18.385Z</v>
+        <v>2026-10-12T18:39:34.326Z</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>12-10-2026, 12:05:40 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B104" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C104" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D104">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E104">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F104">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G104">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-10-12T15:05:40.188Z</v>
+        <v>2026-10-12T18:39:34.325Z</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B105" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C105" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D105">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E105">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F105">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G105">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H105" t="str">
-        <v>2026-10-12T14:26:19.514Z</v>
+        <v>2026-10-12T18:39:34.319Z</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:18 p. m.</v>
       </c>
       <c r="B106" t="str">
-        <v>orders_export (6).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C106" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D106">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E106">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F106">
         <v>0</v>
       </c>
       <c r="G106">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H106" t="str">
-        <v>2026-10-12T14:26:19.513Z</v>
+        <v>2026-10-12T18:39:18.385Z</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 12:05:40 p. m.</v>
       </c>
       <c r="B107" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C107" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D107">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E107">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F107">
         <v>0</v>
       </c>
       <c r="G107">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H107" t="str">
-        <v>2026-10-12T14:24:55.059Z</v>
+        <v>2026-10-12T15:05:40.188Z</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B108" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23231,64 +23231,64 @@
         <v>25</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-10-12T14:24:55.058Z</v>
+        <v>2026-10-12T14:26:19.514Z</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B109" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>orders_export (6).csv</v>
       </c>
       <c r="C109" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D109">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E109">
         <v>4</v>
       </c>
       <c r="F109">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G109">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H109" t="str">
-        <v>2026-10-12T14:24:55.057Z</v>
+        <v>2026-10-12T14:26:19.513Z</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>12-10-2026, 11:24:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B110" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C110" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D110">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F110">
         <v>0</v>
       </c>
       <c r="G110">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H110" t="str">
-        <v>2026-10-12T14:24:00.106Z</v>
+        <v>2026-10-12T14:24:55.059Z</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B111" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23300,73 +23300,73 @@
         <v>25</v>
       </c>
       <c r="E111">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F111">
         <v>0</v>
       </c>
       <c r="G111">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H111" t="str">
-        <v>2026-10-09T14:54:00.353Z</v>
+        <v>2026-10-12T14:24:55.058Z</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B112" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C112" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D112">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E112">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F112">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G112">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H112" t="str">
-        <v>2026-10-09T14:54:00.352Z</v>
+        <v>2026-10-12T14:24:55.057Z</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:00 a. m.</v>
       </c>
       <c r="B113" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C113" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D113">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E113">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G113">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H113" t="str">
-        <v>2026-10-09T14:54:00.347Z</v>
+        <v>2026-10-12T14:24:00.106Z</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>09-10-2026, 11:50:59 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B114" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23375,10 +23375,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D114">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E114">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F114">
         <v>0</v>
@@ -23387,64 +23387,64 @@
         <v>21</v>
       </c>
       <c r="H114" t="str">
-        <v>2026-10-09T14:50:59.695Z</v>
+        <v>2026-10-09T14:54:00.353Z</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B115" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C115" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D115">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E115">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G115">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H115" t="str">
-        <v>2026-10-09T14:28:16.404Z</v>
+        <v>2026-10-09T14:54:00.352Z</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B116" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C116" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D116">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E116">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G116">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H116" t="str">
-        <v>2026-10-09T14:28:16.403Z</v>
+        <v>2026-10-09T14:54:00.347Z</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>09-10-2026, 11:28:07 a. m.</v>
+        <v>09-10-2026, 11:50:59 a. m.</v>
       </c>
       <c r="B117" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23465,12 +23465,12 @@
         <v>21</v>
       </c>
       <c r="H117" t="str">
-        <v>2026-10-09T14:28:07.531Z</v>
+        <v>2026-10-09T14:50:59.695Z</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B118" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23491,12 +23491,12 @@
         <v>21</v>
       </c>
       <c r="H118" t="str">
-        <v>2026-10-09T14:26:45.497Z</v>
+        <v>2026-10-09T14:28:16.404Z</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B119" t="str">
         <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
@@ -23517,21 +23517,21 @@
         <v>19</v>
       </c>
       <c r="H119" t="str">
-        <v>2026-10-09T14:26:45.495Z</v>
+        <v>2026-10-09T14:28:16.403Z</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:07 a. m.</v>
       </c>
       <c r="B120" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C120" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D120">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E120">
         <v>0</v>
@@ -23540,50 +23540,50 @@
         <v>0</v>
       </c>
       <c r="G120">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H120" t="str">
-        <v>2026-10-09T14:26:45.477Z</v>
+        <v>2026-10-09T14:28:07.531Z</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B121" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C121" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D121">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E121">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F121">
         <v>0</v>
       </c>
       <c r="G121">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H121" t="str">
-        <v>2026-10-09T14:25:43.607Z</v>
+        <v>2026-10-09T14:26:45.497Z</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B122" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C122" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D122">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E122">
         <v>0</v>
@@ -23592,36 +23592,36 @@
         <v>0</v>
       </c>
       <c r="G122">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H122" t="str">
-        <v>2026-10-09T14:25:43.606Z</v>
+        <v>2026-10-09T14:26:45.495Z</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B123" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C123" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D123">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E123">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F123">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G123">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H123" t="str">
-        <v>2026-10-09T14:25:43.605Z</v>
+        <v>2026-10-09T14:26:45.477Z</v>
       </c>
     </row>
     <row r="124">
@@ -23629,30 +23629,30 @@
         <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B124" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C124" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D124">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E124">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F124">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G124">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H124" t="str">
-        <v>2026-10-09T14:25:43.580Z</v>
+        <v>2026-10-09T14:25:43.607Z</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>09-10-2026, 11:23:53 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B125" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23673,111 +23673,111 @@
         <v>21</v>
       </c>
       <c r="H125" t="str">
-        <v>2026-10-09T14:23:53.263Z</v>
+        <v>2026-10-09T14:25:43.606Z</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>08-10-2026, 9:14:25 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B126" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C126" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D126">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E126">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F126">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G126">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H126" t="str">
-        <v>2026-10-08T12:14:25.917Z</v>
+        <v>2026-10-09T14:25:43.605Z</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B127" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C127" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D127">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E127">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G127">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H127" t="str">
-        <v>2026-10-08T11:22:18.060Z</v>
+        <v>2026-10-09T14:25:43.580Z</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:23:53 a. m.</v>
       </c>
       <c r="B128" t="str">
-        <v>orders_export (4).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C128" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D128">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E128">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F128">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G128">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H128" t="str">
-        <v>2026-10-08T11:22:18.059Z</v>
+        <v>2026-10-09T14:23:53.263Z</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>08-10-2026, 9:14:25 a. m.</v>
       </c>
       <c r="B129" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C129" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D129">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E129">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F129">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G129">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H129" t="str">
-        <v>2026-10-08T11:22:18.042Z</v>
+        <v>2026-10-08T12:14:25.917Z</v>
       </c>
     </row>
     <row r="130">
@@ -23785,108 +23785,108 @@
         <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B130" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C130" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D130">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E130">
         <v>2</v>
       </c>
       <c r="F130">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G130">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H130" t="str">
-        <v>2026-10-08T11:22:18.032Z</v>
+        <v>2026-10-08T11:22:18.060Z</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>08-10-2026, 8:18:16 a. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B131" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (4).csv</v>
       </c>
       <c r="C131" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D131">
         <v>19</v>
       </c>
       <c r="E131">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F131">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G131">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H131" t="str">
-        <v>2026-10-08T11:18:16.488Z</v>
+        <v>2026-10-08T11:22:18.059Z</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B132" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C132" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D132">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E132">
         <v>2</v>
       </c>
       <c r="F132">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G132">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H132" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.042Z</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B133" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C133" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D133">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E133">
+        <v>2</v>
+      </c>
+      <c r="F133">
+        <v>1</v>
+      </c>
+      <c r="G133">
         <v>0</v>
       </c>
-      <c r="F133">
-        <v>0</v>
-      </c>
-      <c r="G133">
-        <v>19</v>
-      </c>
       <c r="H133" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.032Z</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>07-10-2026, 8:20:41 p. m.</v>
+        <v>08-10-2026, 8:18:16 a. m.</v>
       </c>
       <c r="B134" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23907,64 +23907,64 @@
         <v>19</v>
       </c>
       <c r="H134" t="str">
-        <v>2026-10-07T23:20:41.390Z</v>
+        <v>2026-10-08T11:18:16.488Z</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B135" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
       </c>
       <c r="C135" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D135">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="E135">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F135">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G135">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="H135" t="str">
-        <v>2026-10-07T17:47:17.199Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B136" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C136" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D136">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="E136">
         <v>0</v>
       </c>
       <c r="F136">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G136">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="H136" t="str">
-        <v>2026-10-07T17:47:17.198Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>07-10-2026, 2:46:47 p. m.</v>
+        <v>07-10-2026, 8:20:41 p. m.</v>
       </c>
       <c r="B137" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23985,12 +23985,12 @@
         <v>19</v>
       </c>
       <c r="H137" t="str">
-        <v>2026-10-07T17:46:47.954Z</v>
+        <v>2026-10-07T23:20:41.390Z</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>07-10-2026, 2:44:00 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B138" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24011,64 +24011,64 @@
         <v>19</v>
       </c>
       <c r="H138" t="str">
-        <v>2026-10-07T17:44:00.660Z</v>
+        <v>2026-10-07T17:47:17.199Z</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>07-10-2026, 2:27:43 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B139" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
       </c>
       <c r="C139" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D139">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E139">
         <v>0</v>
       </c>
       <c r="F139">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G139">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="H139" t="str">
-        <v>2026-10-07T17:27:43.517Z</v>
+        <v>2026-10-07T17:47:17.198Z</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:46:47 p. m.</v>
       </c>
       <c r="B140" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C140" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D140">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E140">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F140">
         <v>0</v>
       </c>
       <c r="G140">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H140" t="str">
-        <v>2026-10-07T17:26:50.382Z</v>
+        <v>2026-10-07T17:46:47.954Z</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:44:00 p. m.</v>
       </c>
       <c r="B141" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24080,30 +24080,30 @@
         <v>19</v>
       </c>
       <c r="E141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F141">
         <v>0</v>
       </c>
       <c r="G141">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H141" t="str">
-        <v>2026-10-07T17:26:50.380Z</v>
+        <v>2026-10-07T17:44:00.660Z</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:27:43 p. m.</v>
       </c>
       <c r="B142" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C142" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D142">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="E142">
         <v>0</v>
@@ -24112,41 +24112,41 @@
         <v>0</v>
       </c>
       <c r="G142">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="H142" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:27:43.517Z</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B143" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C143" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D143">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E143">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F143">
         <v>0</v>
       </c>
       <c r="G143">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H143" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:26:50.382Z</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B144" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24155,71 +24155,71 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D144">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E144">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F144">
         <v>0</v>
       </c>
       <c r="G144">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H144" t="str">
-        <v>2026-10-07T16:25:12.953Z</v>
+        <v>2026-10-07T17:26:50.380Z</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B145" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>ventas_por_canal_y_mes.xlsx</v>
       </c>
       <c r="C145" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas por canal y mes</v>
       </c>
       <c r="D145">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="E145">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F145">
         <v>0</v>
       </c>
       <c r="G145">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="H145" t="str">
-        <v>2026-10-07T16:25:12.950Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B146" t="str">
-        <v>orders_export (3).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C146" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D146">
         <v>18</v>
       </c>
       <c r="E146">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F146">
         <v>0</v>
       </c>
       <c r="G146">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H146" t="str">
-        <v>2026-10-07T16:25:12.939Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="147">
@@ -24227,25 +24227,25 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B147" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C147" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D147">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E147">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F147">
         <v>0</v>
       </c>
       <c r="G147">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H147" t="str">
-        <v>2026-10-07T16:25:12.924Z</v>
+        <v>2026-10-07T16:25:12.953Z</v>
       </c>
     </row>
     <row r="148">
@@ -24253,10 +24253,10 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B148" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C148" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D148">
         <v>19</v>
@@ -24271,142 +24271,220 @@
         <v>0</v>
       </c>
       <c r="H148" t="str">
-        <v>2026-10-07T16:25:12.851Z</v>
+        <v>2026-10-07T16:25:12.950Z</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>07-10-2026, 1:10:27 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B149" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>orders_export (3).csv</v>
       </c>
       <c r="C149" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D149">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E149">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F149">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G149">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="H149" t="str">
-        <v>2026-10-07T16:10:27.561Z</v>
+        <v>2026-10-07T16:25:12.939Z</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>07-10-2026, 12:20:36 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B150" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C150" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D150">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E150">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F150">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G150">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H150" t="str">
-        <v>2026-10-07T15:20:36.001Z</v>
+        <v>2026-10-07T16:25:12.924Z</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>07-10-2026, 12:20:35 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B151" t="str">
-        <v>varin_respaldo_2026-10-07.xlsx</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C151" t="str">
-        <v>Respaldo</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D151">
-        <v>322</v>
+        <v>19</v>
       </c>
       <c r="E151">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F151">
         <v>0</v>
       </c>
       <c r="G151">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H151" t="str">
-        <v>2026-10-07T15:20:35.967Z</v>
+        <v>2026-10-07T16:25:12.851Z</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>07-10-2026, 12:20:08 p. m.</v>
+        <v>07-10-2026, 1:10:27 p. m.</v>
       </c>
       <c r="B152" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C152" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D152">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E152">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="F152">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G152">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="H152" t="str">
-        <v>2026-10-07T15:20:08.547Z</v>
+        <v>2026-10-07T16:10:27.561Z</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
+        <v>07-10-2026, 12:20:36 p. m.</v>
+      </c>
+      <c r="B153" t="str">
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Ventas Mercado Libre</v>
+      </c>
+      <c r="D153">
+        <v>92</v>
+      </c>
+      <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153">
+        <v>5</v>
+      </c>
+      <c r="G153">
+        <v>86</v>
+      </c>
+      <c r="H153" t="str">
+        <v>2026-10-07T15:20:36.001Z</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>07-10-2026, 12:20:35 p. m.</v>
+      </c>
+      <c r="B154" t="str">
+        <v>varin_respaldo_2026-10-07.xlsx</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Respaldo</v>
+      </c>
+      <c r="D154">
+        <v>322</v>
+      </c>
+      <c r="E154">
+        <v>190</v>
+      </c>
+      <c r="F154">
+        <v>0</v>
+      </c>
+      <c r="G154">
+        <v>132</v>
+      </c>
+      <c r="H154" t="str">
+        <v>2026-10-07T15:20:35.967Z</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
         <v>07-10-2026, 12:20:08 p. m.</v>
       </c>
-      <c r="B153" t="str">
+      <c r="B155" t="str">
+        <v>ventas_por_canal_y_mes.xlsx</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Ventas por canal y mes</v>
+      </c>
+      <c r="D155">
+        <v>118</v>
+      </c>
+      <c r="E155">
+        <v>118</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155" t="str">
+        <v>2026-10-07T15:20:08.547Z</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>07-10-2026, 12:20:08 p. m.</v>
+      </c>
+      <c r="B156" t="str">
         <v>Varin_Movimientos_DropGO_2026-10-01_al_2026-10-06.xlsx</v>
       </c>
-      <c r="C153" t="str">
+      <c r="C156" t="str">
         <v>Movimientos DropGO</v>
       </c>
-      <c r="D153">
+      <c r="D156">
         <v>14</v>
       </c>
-      <c r="E153">
+      <c r="E156">
         <v>14</v>
       </c>
-      <c r="F153">
+      <c r="F156">
         <v>0</v>
       </c>
-      <c r="G153">
+      <c r="G156">
         <v>0</v>
       </c>
-      <c r="H153" t="str">
+      <c r="H156" t="str">
         <v>2026-10-07T15:20:08.525Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H156"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -25660,7 +25738,7 @@
         <v>2026-10-27 10:28</v>
       </c>
       <c r="B53" t="str">
-        <v>LISTO PARA ENVIO</v>
+        <v>ENTREGADO</v>
       </c>
       <c r="C53" t="str">
         <v>AB68-48359366999</v>
@@ -25706,7 +25784,7 @@
         <v>2026-10-27 17:43</v>
       </c>
       <c r="B55" t="str">
-        <v>PREPARACION</v>
+        <v>ENTREGADO</v>
       </c>
       <c r="C55" t="str">
         <v>AB59-1040</v>
@@ -25729,7 +25807,7 @@
         <v>2026-10-27 21:47</v>
       </c>
       <c r="B56" t="str">
-        <v>PREPARACION</v>
+        <v>EN CAMINO</v>
       </c>
       <c r="C56" t="str">
         <v>AB59-1041</v>
@@ -25752,7 +25830,7 @@
         <v>2026-10-28 00:10</v>
       </c>
       <c r="B57" t="str">
-        <v>PREPARACION</v>
+        <v>EN CAMINO</v>
       </c>
       <c r="C57" t="str">
         <v>AB59-1042</v>
@@ -27952,7 +28030,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="B58" t="str">
-        <v>LISTO PARA ENVIO</v>
+        <v>ENTREGADO</v>
       </c>
       <c r="C58" t="str">
         <v>AB68-48359366999</v>
@@ -27990,7 +28068,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="B59" t="str">
-        <v>LISTO PARA ENVIO</v>
+        <v>ENTREGADO</v>
       </c>
       <c r="C59" t="str">
         <v>AB68-48359366999</v>
@@ -28066,7 +28144,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="B61" t="str">
-        <v>PREPARACION</v>
+        <v>ENTREGADO</v>
       </c>
       <c r="C61" t="str">
         <v>AB59-1040</v>
@@ -28078,7 +28156,7 @@
         <v>219800</v>
       </c>
       <c r="F61" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="G61" t="str">
         <v>Ventilador de Techo Inteligente - WiFi Negro Nogal S/L</v>
@@ -28093,7 +28171,7 @@
         <v>0</v>
       </c>
       <c r="K61" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="L61" t="str">
         <v>SI</v>
@@ -28104,7 +28182,7 @@
         <v>2026-10-27</v>
       </c>
       <c r="B62" t="str">
-        <v>PREPARACION</v>
+        <v>EN CAMINO</v>
       </c>
       <c r="C62" t="str">
         <v>AB59-1041</v>
@@ -28116,7 +28194,7 @@
         <v>130000</v>
       </c>
       <c r="F62" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="G62" t="str">
         <v>Ventilador de Techo Inteligente - WiFi Luz Blanco Blanco</v>
@@ -28131,7 +28209,7 @@
         <v>0</v>
       </c>
       <c r="K62" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="L62" t="str">
         <v>SI</v>
@@ -28142,7 +28220,7 @@
         <v>2026-10-28</v>
       </c>
       <c r="B63" t="str">
-        <v>PREPARACION</v>
+        <v>EN CAMINO</v>
       </c>
       <c r="C63" t="str">
         <v>AB59-1042</v>
@@ -28154,7 +28232,7 @@
         <v>123800</v>
       </c>
       <c r="F63" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="G63" t="str">
         <v>Estufa Calefactor Panel Radiador Eléctrico Wifi Varin® 2000w</v>
@@ -28169,7 +28247,7 @@
         <v>0</v>
       </c>
       <c r="K63" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="L63" t="str">
         <v>SI</v>
@@ -28199,7 +28277,7 @@
         <v>Generado</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-28T22:40:25.898Z</v>
+        <v>2026-10-28T22:43:18.854Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Datos Varin 2026-10-30 11:40
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20875,7 +20875,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H164"/>
+  <dimension ref="A1:H167"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -20914,42 +20914,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>30-10-2026, 8:31:15 a. m.</v>
+        <v>30-10-2026, 8:40:12 a. m.</v>
       </c>
       <c r="B2" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C2" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D2">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-30T11:31:15.714Z</v>
+        <v>2026-10-30T11:40:12.326Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>30-10-2026, 8:31:15 a. m.</v>
+        <v>30-10-2026, 8:40:12 a. m.</v>
       </c>
       <c r="B3" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261030_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-30_07-29hs_2967682966.xlsx</v>
       </c>
       <c r="C3" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D3">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -20958,67 +20958,67 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-10-30T11:31:15.713Z</v>
+        <v>2026-10-30T11:40:12.320Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>30-10-2026, 8:31:15 a. m.</v>
+        <v>30-10-2026, 8:38:08 a. m.</v>
       </c>
       <c r="B4" t="str">
-        <v>20261030_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-30_07-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C4" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D4">
-        <v>160</v>
+        <v>55</v>
       </c>
       <c r="E4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>149</v>
+        <v>55</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-10-30T11:31:15.712Z</v>
+        <v>2026-10-30T11:38:08.555Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>30-10-2026, 8:30:42 a. m.</v>
+        <v>30-10-2026, 8:31:15 a. m.</v>
       </c>
       <c r="B5" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C5" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D5">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-10-30T11:30:42.940Z</v>
+        <v>2026-10-30T11:31:15.714Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>29-10-2026, 9:16:55 a. m.</v>
+        <v>30-10-2026, 8:31:15 a. m.</v>
       </c>
       <c r="B6" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21039,38 +21039,38 @@
         <v>55</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-10-29T12:16:55.755Z</v>
+        <v>2026-10-30T11:31:15.713Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>29-10-2026, 8:44:17 a. m.</v>
+        <v>30-10-2026, 8:31:15 a. m.</v>
       </c>
       <c r="B7" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261030_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-30_07-29hs_2967682966.xlsx</v>
       </c>
       <c r="C7" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D7">
+        <v>160</v>
+      </c>
+      <c r="E7">
         <v>5</v>
       </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
       <c r="F7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7">
-        <v>4</v>
+        <v>149</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-10-29T11:44:17.403Z</v>
+        <v>2026-10-30T11:31:15.712Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>29-10-2026, 8:44:17 a. m.</v>
+        <v>30-10-2026, 8:30:42 a. m.</v>
       </c>
       <c r="B8" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21091,116 +21091,116 @@
         <v>55</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-10-29T11:44:17.401Z</v>
+        <v>2026-10-30T11:30:42.940Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>29-10-2026, 8:44:17 a. m.</v>
+        <v>29-10-2026, 9:16:55 a. m.</v>
       </c>
       <c r="B9" t="str">
-        <v>20261029_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-29_07-36hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C9" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D9">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-10-29T11:44:17.400Z</v>
+        <v>2026-10-29T12:16:55.755Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>28-10-2026, 7:43:14 p. m.</v>
+        <v>29-10-2026, 8:44:17 a. m.</v>
       </c>
       <c r="B10" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C10" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D10">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-10-28T22:43:14.280Z</v>
+        <v>2026-10-29T11:44:17.403Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>28-10-2026, 7:43:14 p. m.</v>
+        <v>29-10-2026, 8:44:17 a. m.</v>
       </c>
       <c r="B11" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C11" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-10-28T22:43:14.278Z</v>
+        <v>2026-10-29T11:44:17.401Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>28-10-2026, 7:43:14 p. m.</v>
+        <v>29-10-2026, 8:44:17 a. m.</v>
       </c>
       <c r="B12" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261029_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-29_07-36hs_2967682966.xlsx</v>
       </c>
       <c r="C12" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D12">
-        <v>5</v>
+        <v>76</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12">
         <v>4</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-10-28T22:43:14.269Z</v>
+        <v>2026-10-29T11:44:17.400Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>28-10-2026, 7:40:21 p. m.</v>
+        <v>28-10-2026, 7:43:14 p. m.</v>
       </c>
       <c r="B13" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21221,99 +21221,99 @@
         <v>55</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-10-28T22:40:21.045Z</v>
+        <v>2026-10-28T22:43:14.280Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>28-10-2026, 7:40:21 p. m.</v>
+        <v>28-10-2026, 7:43:14 p. m.</v>
       </c>
       <c r="B14" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C14" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D14">
-        <v>153</v>
+        <v>5</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G14">
-        <v>153</v>
+        <v>1</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-10-28T22:40:21.044Z</v>
+        <v>2026-10-28T22:43:14.278Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>28-10-2026, 7:40:04 p. m.</v>
+        <v>28-10-2026, 7:43:14 p. m.</v>
       </c>
       <c r="B15" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C15" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D15">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G15">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-10-28T22:40:04.272Z</v>
+        <v>2026-10-28T22:43:14.269Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:21 p. m.</v>
       </c>
       <c r="B16" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C16" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D16">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E16">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-10-28T22:34:33.117Z</v>
+        <v>2026-10-28T22:40:21.045Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:21 p. m.</v>
       </c>
       <c r="B17" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
       </c>
       <c r="C17" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D17">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -21322,67 +21322,67 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-10-28T22:34:33.116Z</v>
+        <v>2026-10-28T22:40:21.044Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>28-10-2026, 7:34:33 p. m.</v>
+        <v>28-10-2026, 7:40:04 p. m.</v>
       </c>
       <c r="B18" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C18" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D18">
-        <v>153</v>
+        <v>55</v>
       </c>
       <c r="E18">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>147</v>
+        <v>55</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-10-28T22:34:33.114Z</v>
+        <v>2026-10-28T22:40:04.272Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>28-10-2026, 7:34:12 p. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B19" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C19" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D19">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-10-28T22:34:12.755Z</v>
+        <v>2026-10-28T22:34:33.117Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B20" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21394,73 +21394,73 @@
         <v>55</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-10-28T10:57:11.638Z</v>
+        <v>2026-10-28T22:34:33.116Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:33 p. m.</v>
       </c>
       <c r="B21" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_18-32hs_2967682966.xlsx</v>
       </c>
       <c r="C21" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D21">
-        <v>6</v>
+        <v>153</v>
       </c>
       <c r="E21">
         <v>5</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>147</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-10-28T10:57:11.636Z</v>
+        <v>2026-10-28T22:34:33.114Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>28-10-2026, 7:57:11 a. m.</v>
+        <v>28-10-2026, 7:34:12 p. m.</v>
       </c>
       <c r="B22" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C22" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D22">
-        <v>6</v>
+        <v>55</v>
       </c>
       <c r="E22">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-10-28T10:57:11.632Z</v>
+        <v>2026-10-28T22:34:12.755Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>28-10-2026, 7:56:06 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B23" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21469,10 +21469,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D23">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -21481,64 +21481,64 @@
         <v>50</v>
       </c>
       <c r="H23" t="str">
-        <v>2026-10-28T10:56:06.328Z</v>
+        <v>2026-10-28T10:57:11.638Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>28-10-2026, 7:56:06 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B24" t="str">
-        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C24" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D24">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="H24" t="str">
-        <v>2026-10-28T10:56:06.326Z</v>
+        <v>2026-10-28T10:57:11.636Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>28-10-2026, 7:53:38 a. m.</v>
+        <v>28-10-2026, 7:57:11 a. m.</v>
       </c>
       <c r="B25" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C25" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D25">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-10-28T10:53:38.820Z</v>
+        <v>2026-10-28T10:57:11.632Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B26" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21559,38 +21559,38 @@
         <v>50</v>
       </c>
       <c r="H26" t="str">
-        <v>2026-10-27T22:11:05.716Z</v>
+        <v>2026-10-28T10:56:06.328Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>27-10-2026, 7:11:05 p. m.</v>
+        <v>28-10-2026, 7:56:06 a. m.</v>
       </c>
       <c r="B27" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
+        <v>20261028_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-28_06-54hs_2967682966.xlsx</v>
       </c>
       <c r="C27" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D27">
-        <v>148</v>
+        <v>69</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>144</v>
+        <v>69</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-10-27T22:11:05.714Z</v>
+        <v>2026-10-28T10:56:06.326Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>27-10-2026, 7:10:39 p. m.</v>
+        <v>28-10-2026, 7:53:38 a. m.</v>
       </c>
       <c r="B28" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21611,12 +21611,12 @@
         <v>50</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-10-27T22:10:39.288Z</v>
+        <v>2026-10-28T10:53:38.820Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B29" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21628,68 +21628,68 @@
         <v>50</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H29" t="str">
-        <v>2026-10-27T12:40:01.215Z</v>
+        <v>2026-10-27T22:11:05.716Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:11:05 p. m.</v>
       </c>
       <c r="B30" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_18-09hs_2967682966.xlsx</v>
       </c>
       <c r="C30" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D30">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G30">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-10-27T12:40:01.212Z</v>
+        <v>2026-10-27T22:11:05.714Z</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>27-10-2026, 9:40:01 a. m.</v>
+        <v>27-10-2026, 7:10:39 p. m.</v>
       </c>
       <c r="B31" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C31" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-10-27T12:40:01.116Z</v>
+        <v>2026-10-27T22:10:39.288Z</v>
       </c>
     </row>
     <row r="32">
@@ -21697,186 +21697,186 @@
         <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B32" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C32" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H32" t="str">
-        <v>2026-10-27T12:40:01.113Z</v>
+        <v>2026-10-27T12:40:01.215Z</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B33" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C33" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D33">
-        <v>4</v>
+        <v>147</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-10-27T12:39:46.660Z</v>
+        <v>2026-10-27T12:40:01.212Z</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>27-10-2026, 9:39:46 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B34" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C34" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D34">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34">
         <v>0</v>
       </c>
-      <c r="F34">
-        <v>0</v>
-      </c>
-      <c r="G34">
-        <v>49</v>
-      </c>
       <c r="H34" t="str">
-        <v>2026-10-27T12:39:46.656Z</v>
+        <v>2026-10-27T12:40:01.116Z</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:40:01 a. m.</v>
       </c>
       <c r="B35" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C35" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E35">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35">
         <v>0</v>
       </c>
-      <c r="G35">
-        <v>3</v>
-      </c>
       <c r="H35" t="str">
-        <v>2026-10-27T12:35:13.606Z</v>
+        <v>2026-10-27T12:40:01.113Z</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B36" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C36" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D36">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="G36">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-10-27T12:35:13.605Z</v>
+        <v>2026-10-27T12:39:46.660Z</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>27-10-2026, 9:35:13 a. m.</v>
+        <v>27-10-2026, 9:39:46 a. m.</v>
       </c>
       <c r="B37" t="str">
-        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C37" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D37">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="E37">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>131</v>
+        <v>49</v>
       </c>
       <c r="H37" t="str">
-        <v>2026-10-27T12:35:13.604Z</v>
+        <v>2026-10-27T12:39:46.656Z</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>27-10-2026, 9:34:54 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B38" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C38" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D38">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F38">
         <v>0</v>
       </c>
       <c r="G38">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="H38" t="str">
-        <v>2026-10-27T12:34:54.468Z</v>
+        <v>2026-10-27T12:35:13.606Z</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B39" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -21888,177 +21888,177 @@
         <v>49</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39">
         <v>0</v>
       </c>
       <c r="G39">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H39" t="str">
-        <v>2026-10-26T12:06:47.126Z</v>
+        <v>2026-10-27T12:35:13.605Z</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:35:13 a. m.</v>
       </c>
       <c r="B40" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>20261027_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-27_08-33hs_2967682966.xlsx</v>
       </c>
       <c r="C40" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D40">
-        <v>3</v>
+        <v>147</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G40">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="H40" t="str">
-        <v>2026-10-26T12:06:47.123Z</v>
+        <v>2026-10-27T12:35:13.604Z</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>26-10-2026, 9:06:47 a. m.</v>
+        <v>27-10-2026, 9:34:54 a. m.</v>
       </c>
       <c r="B41" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C41" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="H41" t="str">
-        <v>2026-10-26T12:06:47.118Z</v>
+        <v>2026-10-27T12:34:54.468Z</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B42" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C42" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D42">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E42">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F42">
         <v>0</v>
       </c>
       <c r="G42">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H42" t="str">
-        <v>2026-10-26T12:05:32.699Z</v>
+        <v>2026-10-26T12:06:47.126Z</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B43" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C43" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D43">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>2</v>
+      </c>
+      <c r="G43">
         <v>0</v>
       </c>
-      <c r="F43">
-        <v>0</v>
-      </c>
-      <c r="G43">
-        <v>48</v>
-      </c>
       <c r="H43" t="str">
-        <v>2026-10-26T12:05:32.697Z</v>
+        <v>2026-10-26T12:06:47.123Z</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>26-10-2026, 9:05:32 a. m.</v>
+        <v>26-10-2026, 9:06:47 a. m.</v>
       </c>
       <c r="B44" t="str">
-        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C44" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D44">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E44">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G44">
         <v>0</v>
       </c>
       <c r="H44" t="str">
-        <v>2026-10-26T12:05:32.692Z</v>
+        <v>2026-10-26T12:06:47.118Z</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>25-10-2026, 12:10:56 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B45" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C45" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D45">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
       <c r="G45">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H45" t="str">
-        <v>2026-10-25T15:10:56.412Z</v>
+        <v>2026-10-26T12:05:32.699Z</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B46" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22079,38 +22079,38 @@
         <v>48</v>
       </c>
       <c r="H46" t="str">
-        <v>2026-10-23T22:12:12.477Z</v>
+        <v>2026-10-26T12:05:32.697Z</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>23-10-2026, 7:12:12 p. m.</v>
+        <v>26-10-2026, 9:05:32 a. m.</v>
       </c>
       <c r="B47" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
+        <v>20261026_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-26_08-00hs_2967682966.xlsx</v>
       </c>
       <c r="C47" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D47">
-        <v>135</v>
+        <v>6</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F47">
         <v>0</v>
       </c>
       <c r="G47">
-        <v>135</v>
+        <v>0</v>
       </c>
       <c r="H47" t="str">
-        <v>2026-10-23T22:12:12.476Z</v>
+        <v>2026-10-26T12:05:32.692Z</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>23-10-2026, 7:11:53 p. m.</v>
+        <v>25-10-2026, 12:10:56 p. m.</v>
       </c>
       <c r="B48" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22131,12 +22131,12 @@
         <v>48</v>
       </c>
       <c r="H48" t="str">
-        <v>2026-10-23T22:11:53.140Z</v>
+        <v>2026-10-25T15:10:56.412Z</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B49" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22157,15 +22157,15 @@
         <v>48</v>
       </c>
       <c r="H49" t="str">
-        <v>2026-10-23T13:17:56.047Z</v>
+        <v>2026-10-23T22:12:12.477Z</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>23-10-2026, 10:17:56 a. m.</v>
+        <v>23-10-2026, 7:12:12 p. m.</v>
       </c>
       <c r="B50" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C50" t="str">
         <v>Ventas Mercado Libre</v>
@@ -22183,12 +22183,12 @@
         <v>135</v>
       </c>
       <c r="H50" t="str">
-        <v>2026-10-23T13:17:56.044Z</v>
+        <v>2026-10-23T22:12:12.476Z</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>23-10-2026, 9:52:55 a. m.</v>
+        <v>23-10-2026, 7:11:53 p. m.</v>
       </c>
       <c r="B51" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22209,12 +22209,12 @@
         <v>48</v>
       </c>
       <c r="H51" t="str">
-        <v>2026-10-23T12:52:55.551Z</v>
+        <v>2026-10-23T22:11:53.140Z</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>23-10-2026, 9:50:04 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B52" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22235,38 +22235,38 @@
         <v>48</v>
       </c>
       <c r="H52" t="str">
-        <v>2026-10-23T12:50:04.195Z</v>
+        <v>2026-10-23T13:17:56.047Z</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 10:17:56 a. m.</v>
       </c>
       <c r="B53" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C53" t="str">
-        <v>Full ML · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D53">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53">
         <v>0</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="H53" t="str">
-        <v>2026-10-23T12:37:54.995Z</v>
+        <v>2026-10-23T13:17:56.044Z</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:52:55 a. m.</v>
       </c>
       <c r="B54" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22287,64 +22287,64 @@
         <v>48</v>
       </c>
       <c r="H54" t="str">
-        <v>2026-10-23T12:37:54.994Z</v>
+        <v>2026-10-23T12:52:55.551Z</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>23-10-2026, 9:37:54 a. m.</v>
+        <v>23-10-2026, 9:50:04 a. m.</v>
       </c>
       <c r="B55" t="str">
-        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C55" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D55">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G55">
-        <v>126</v>
+        <v>48</v>
       </c>
       <c r="H55" t="str">
-        <v>2026-10-23T12:37:54.992Z</v>
+        <v>2026-10-23T12:50:04.195Z</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>23-10-2026, 9:37:27 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B56" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C56" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D56">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56">
         <v>0</v>
       </c>
       <c r="G56">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="H56" t="str">
-        <v>2026-10-23T12:37:27.533Z</v>
+        <v>2026-10-23T12:37:54.995Z</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>23-10-2026, 9:34:31 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B57" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22365,64 +22365,64 @@
         <v>48</v>
       </c>
       <c r="H57" t="str">
-        <v>2026-10-23T12:34:31.611Z</v>
+        <v>2026-10-23T12:37:54.994Z</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>23-10-2026, 9:19:14 a. m.</v>
+        <v>23-10-2026, 9:37:54 a. m.</v>
       </c>
       <c r="B58" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261023_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-23_08-35hs_2967682966.xlsx</v>
       </c>
       <c r="C58" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D58">
-        <v>48</v>
+        <v>135</v>
       </c>
       <c r="E58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F58">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G58">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="H58" t="str">
-        <v>2026-10-23T12:19:14.833Z</v>
+        <v>2026-10-23T12:37:54.992Z</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:37:27 a. m.</v>
       </c>
       <c r="B59" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C59" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D59">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="E59">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F59">
         <v>0</v>
       </c>
       <c r="G59">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="H59" t="str">
-        <v>2026-10-22T11:51:13.535Z</v>
+        <v>2026-10-23T12:37:27.533Z</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:34:31 a. m.</v>
       </c>
       <c r="B60" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22443,38 +22443,38 @@
         <v>48</v>
       </c>
       <c r="H60" t="str">
-        <v>2026-10-22T11:51:13.534Z</v>
+        <v>2026-10-23T12:34:31.611Z</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>22-10-2026, 8:51:13 a. m.</v>
+        <v>23-10-2026, 9:19:14 a. m.</v>
       </c>
       <c r="B61" t="str">
-        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C61" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D61">
-        <v>134</v>
+        <v>48</v>
       </c>
       <c r="E61">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G61">
-        <v>123</v>
+        <v>48</v>
       </c>
       <c r="H61" t="str">
-        <v>2026-10-22T11:51:13.529Z</v>
+        <v>2026-10-23T12:19:14.833Z</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B62" t="str">
         <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
@@ -22483,10 +22483,10 @@
         <v>Full ML · generado</v>
       </c>
       <c r="D62">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -22495,12 +22495,12 @@
         <v>2</v>
       </c>
       <c r="H62" t="str">
-        <v>2026-10-21T11:58:09.619Z</v>
+        <v>2026-10-22T11:51:13.535Z</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B63" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22512,42 +22512,42 @@
         <v>48</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F63">
         <v>0</v>
       </c>
       <c r="G63">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H63" t="str">
-        <v>2026-10-21T11:58:09.618Z</v>
+        <v>2026-10-22T11:51:13.534Z</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>21-10-2026, 8:58:09 a. m.</v>
+        <v>22-10-2026, 8:51:13 a. m.</v>
       </c>
       <c r="B64" t="str">
-        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
+        <v>20261022_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-22_07-48hs_2967682966.xlsx</v>
       </c>
       <c r="C64" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D64">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F64">
         <v>5</v>
       </c>
       <c r="G64">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H64" t="str">
-        <v>2026-10-21T11:58:09.614Z</v>
+        <v>2026-10-22T11:51:13.529Z</v>
       </c>
     </row>
     <row r="65">
@@ -22555,25 +22555,25 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B65" t="str">
-        <v>ventas-report (11).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C65" t="str">
-        <v>DropGO · ventas</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D65">
+        <v>4</v>
+      </c>
+      <c r="E65">
         <v>2</v>
-      </c>
-      <c r="E65">
-        <v>1</v>
       </c>
       <c r="F65">
         <v>0</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H65" t="str">
-        <v>2026-10-21T11:58:09.533Z</v>
+        <v>2026-10-21T11:58:09.619Z</v>
       </c>
     </row>
     <row r="66">
@@ -22581,13 +22581,13 @@
         <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B66" t="str">
-        <v>picking-report (11).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C66" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D66">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E66">
         <v>1</v>
@@ -22596,88 +22596,88 @@
         <v>0</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="H66" t="str">
-        <v>2026-10-21T11:58:09.530Z</v>
+        <v>2026-10-21T11:58:09.618Z</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B67" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261021_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-21_09-44hs_2967682966.xlsx</v>
       </c>
       <c r="C67" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D67">
-        <v>47</v>
+        <v>128</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F67">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G67">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="H67" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.614Z</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B68" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>ventas-report (11).xlsx</v>
       </c>
       <c r="C68" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F68">
         <v>0</v>
       </c>
       <c r="G68">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H68" t="str">
-        <v>2026-10-20T12:36:20.901Z</v>
+        <v>2026-10-21T11:58:09.533Z</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>20-10-2026, 9:36:20 a. m.</v>
+        <v>21-10-2026, 8:58:09 a. m.</v>
       </c>
       <c r="B69" t="str">
-        <v>ventas-report (10).xlsx</v>
+        <v>picking-report (11).xlsx</v>
       </c>
       <c r="C69" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D69">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E69">
         <v>1</v>
       </c>
       <c r="F69">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G69">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H69" t="str">
-        <v>2026-10-20T12:36:20.899Z</v>
+        <v>2026-10-21T11:58:09.530Z</v>
       </c>
     </row>
     <row r="70">
@@ -22685,25 +22685,25 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B70" t="str">
-        <v>picking-report (10).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C70" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D70">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G70">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H70" t="str">
-        <v>2026-10-20T12:36:20.895Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="71">
@@ -22711,212 +22711,212 @@
         <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B71" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C71" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D71">
-        <v>126</v>
+        <v>47</v>
       </c>
       <c r="E71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F71">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G71">
-        <v>119</v>
+        <v>46</v>
       </c>
       <c r="H71" t="str">
-        <v>2026-10-20T12:36:20.890Z</v>
+        <v>2026-10-20T12:36:20.901Z</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>20-10-2026, 9:34:26 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B72" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (10).xlsx</v>
       </c>
       <c r="C72" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D72">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F72">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G72">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="H72" t="str">
-        <v>2026-10-20T12:34:26.210Z</v>
+        <v>2026-10-20T12:36:20.899Z</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B73" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (10).xlsx</v>
       </c>
       <c r="C73" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D73">
+        <v>11</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+      <c r="F73">
+        <v>3</v>
+      </c>
+      <c r="G73">
         <v>7</v>
       </c>
-      <c r="E73">
-        <v>5</v>
-      </c>
-      <c r="F73">
-        <v>1</v>
-      </c>
-      <c r="G73">
-        <v>2</v>
-      </c>
       <c r="H73" t="str">
-        <v>2026-10-19T12:21:51.769Z</v>
+        <v>2026-10-20T12:36:20.895Z</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:36:20 a. m.</v>
       </c>
       <c r="B74" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_18-09hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C74" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D74">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F74">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G74">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="H74" t="str">
-        <v>2026-10-19T12:21:51.768Z</v>
+        <v>2026-10-20T12:36:20.890Z</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>19-10-2026, 9:21:51 a. m.</v>
+        <v>20-10-2026, 9:34:26 a. m.</v>
       </c>
       <c r="B75" t="str">
-        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C75" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D75">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E75">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F75">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G75">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H75" t="str">
-        <v>2026-10-19T12:21:51.766Z</v>
+        <v>2026-10-20T12:34:26.210Z</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B76" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C76" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D76">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="E76">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G76">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H76" t="str">
-        <v>2026-10-19T12:20:51.921Z</v>
+        <v>2026-10-19T12:21:51.769Z</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B77" t="str">
-        <v>picking-report (9).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C77" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D77">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E77">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F77">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G77">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="H77" t="str">
-        <v>2026-10-19T12:20:51.919Z</v>
+        <v>2026-10-19T12:21:51.768Z</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>19-10-2026, 9:20:51 a. m.</v>
+        <v>19-10-2026, 9:21:51 a. m.</v>
       </c>
       <c r="B78" t="str">
-        <v>ventas-report (9).xlsx</v>
+        <v>20261019_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-19_08-21hs_2967682966.xlsx</v>
       </c>
       <c r="C78" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D78">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="E78">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G78">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="H78" t="str">
-        <v>2026-10-19T12:20:51.913Z</v>
+        <v>2026-10-19T12:21:51.766Z</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>19-10-2026, 9:12:06 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B79" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -22925,10 +22925,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D79">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F79">
         <v>0</v>
@@ -22937,229 +22937,229 @@
         <v>37</v>
       </c>
       <c r="H79" t="str">
-        <v>2026-10-19T12:12:06.575Z</v>
+        <v>2026-10-19T12:20:51.921Z</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B80" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>picking-report (9).xlsx</v>
       </c>
       <c r="C80" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D80">
+        <v>14</v>
+      </c>
+      <c r="E80">
+        <v>7</v>
+      </c>
+      <c r="F80">
         <v>5</v>
-      </c>
-      <c r="E80">
-        <v>3</v>
-      </c>
-      <c r="F80">
-        <v>0</v>
       </c>
       <c r="G80">
         <v>2</v>
       </c>
       <c r="H80" t="str">
-        <v>2026-10-16T12:37:12.832Z</v>
+        <v>2026-10-19T12:20:51.919Z</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:20:51 a. m.</v>
       </c>
       <c r="B81" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (9).xlsx</v>
       </c>
       <c r="C81" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D81">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E81">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F81">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G81">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H81" t="str">
-        <v>2026-10-16T12:37:12.831Z</v>
+        <v>2026-10-19T12:20:51.913Z</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>16-10-2026, 9:37:12 a. m.</v>
+        <v>19-10-2026, 9:12:06 a. m.</v>
       </c>
       <c r="B82" t="str">
-        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C82" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D82">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E82">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F82">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G82">
         <v>37</v>
       </c>
       <c r="H82" t="str">
-        <v>2026-10-16T12:37:12.827Z</v>
+        <v>2026-10-19T12:12:06.575Z</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B83" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C83" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D83">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F83">
         <v>0</v>
       </c>
       <c r="G83">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="H83" t="str">
-        <v>2026-10-16T11:52:26.043Z</v>
+        <v>2026-10-16T12:37:12.832Z</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B84" t="str">
-        <v>picking-report (8).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C84" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D84">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E84">
         <v>0</v>
       </c>
       <c r="F84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G84">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H84" t="str">
-        <v>2026-10-16T11:52:26.040Z</v>
+        <v>2026-10-16T12:37:12.831Z</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>16-10-2026, 8:52:26 a. m.</v>
+        <v>16-10-2026, 9:37:12 a. m.</v>
       </c>
       <c r="B85" t="str">
-        <v>ventas-report (8).xlsx</v>
+        <v>20261016_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-16_08-29hs_2967682966.xlsx</v>
       </c>
       <c r="C85" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D85">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F85">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G85">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="H85" t="str">
-        <v>2026-10-16T11:52:26.034Z</v>
+        <v>2026-10-16T12:37:12.827Z</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B86" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C86" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D86">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F86">
         <v>0</v>
       </c>
       <c r="G86">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H86" t="str">
-        <v>2026-10-15T12:11:36.404Z</v>
+        <v>2026-10-16T11:52:26.043Z</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B87" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (8).xlsx</v>
       </c>
       <c r="C87" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D87">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E87">
         <v>0</v>
       </c>
       <c r="F87">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G87">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="H87" t="str">
-        <v>2026-10-15T12:11:36.403Z</v>
+        <v>2026-10-16T11:52:26.040Z</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>15-10-2026, 9:11:36 a. m.</v>
+        <v>16-10-2026, 8:52:26 a. m.</v>
       </c>
       <c r="B88" t="str">
-        <v>ventas-report (7).xlsx</v>
+        <v>ventas-report (8).xlsx</v>
       </c>
       <c r="C88" t="str">
         <v>DropGO · ventas</v>
       </c>
       <c r="D88">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E88">
         <v>0</v>
@@ -23168,10 +23168,10 @@
         <v>1</v>
       </c>
       <c r="G88">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H88" t="str">
-        <v>2026-10-15T12:11:36.401Z</v>
+        <v>2026-10-16T11:52:26.034Z</v>
       </c>
     </row>
     <row r="89">
@@ -23179,25 +23179,25 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B89" t="str">
-        <v>picking-report (7).xlsx</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C89" t="str">
-        <v>DropGO · picking</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D89">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E89">
+        <v>2</v>
+      </c>
+      <c r="F89">
         <v>0</v>
-      </c>
-      <c r="F89">
-        <v>1</v>
       </c>
       <c r="G89">
         <v>2</v>
       </c>
       <c r="H89" t="str">
-        <v>2026-10-15T12:11:36.397Z</v>
+        <v>2026-10-15T12:11:36.404Z</v>
       </c>
     </row>
     <row r="90">
@@ -23205,143 +23205,143 @@
         <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B90" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C90" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D90">
-        <v>114</v>
+        <v>37</v>
       </c>
       <c r="E90">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F90">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G90">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="H90" t="str">
-        <v>2026-10-15T12:11:36.389Z</v>
+        <v>2026-10-15T12:11:36.403Z</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>14-10-2026, 10:42:32 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B91" t="str">
-        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
+        <v>ventas-report (7).xlsx</v>
       </c>
       <c r="C91" t="str">
-        <v>Manual</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D91">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E91">
         <v>0</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H91" t="str">
-        <v>2026-10-14T13:42:32.444Z</v>
+        <v>2026-10-15T12:11:36.401Z</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B92" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (7).xlsx</v>
       </c>
       <c r="C92" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D92">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+      <c r="G92">
         <v>2</v>
       </c>
-      <c r="F92">
-        <v>0</v>
-      </c>
-      <c r="G92">
-        <v>35</v>
-      </c>
       <c r="H92" t="str">
-        <v>2026-10-14T13:41:21.926Z</v>
+        <v>2026-10-15T12:11:36.397Z</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>15-10-2026, 9:11:36 a. m.</v>
       </c>
       <c r="B93" t="str">
-        <v>picking-report (6).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_18-02hs_2967682966.xlsx</v>
       </c>
       <c r="C93" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D93">
-        <v>7</v>
+        <v>114</v>
       </c>
       <c r="E93">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F93">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G93">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="H93" t="str">
-        <v>2026-10-14T13:41:21.925Z</v>
+        <v>2026-10-15T12:11:36.389Z</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>14-10-2026, 10:41:21 a. m.</v>
+        <v>14-10-2026, 10:42:32 a. m.</v>
       </c>
       <c r="B94" t="str">
-        <v>ventas-report (6).xlsx</v>
+        <v>Agregado: VA-F001 -1 en Office (2026-10-14)</v>
       </c>
       <c r="C94" t="str">
-        <v>DropGO · ventas</v>
+        <v>Manual</v>
       </c>
       <c r="D94">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E94">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F94">
         <v>0</v>
       </c>
       <c r="G94">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H94" t="str">
-        <v>2026-10-14T13:41:21.921Z</v>
+        <v>2026-10-14T13:42:32.444Z</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B95" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C95" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D95">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="E95">
         <v>2</v>
@@ -23350,93 +23350,93 @@
         <v>0</v>
       </c>
       <c r="G95">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="H95" t="str">
-        <v>2026-10-14T13:40:03.191Z</v>
+        <v>2026-10-14T13:41:21.926Z</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B96" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (6).xlsx</v>
       </c>
       <c r="C96" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D96">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F96">
         <v>0</v>
       </c>
       <c r="G96">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H96" t="str">
-        <v>2026-10-14T13:40:03.190Z</v>
+        <v>2026-10-14T13:41:21.925Z</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>14-10-2026, 10:40:03 a. m.</v>
+        <v>14-10-2026, 10:41:21 a. m.</v>
       </c>
       <c r="B97" t="str">
-        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
+        <v>ventas-report (6).xlsx</v>
       </c>
       <c r="C97" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D97">
-        <v>112</v>
+        <v>7</v>
       </c>
       <c r="E97">
         <v>3</v>
       </c>
       <c r="F97">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G97">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="H97" t="str">
-        <v>2026-10-14T13:40:03.188Z</v>
+        <v>2026-10-14T13:41:21.921Z</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>14-10-2026, 10:39:50 a. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B98" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C98" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D98">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="E98">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F98">
         <v>0</v>
       </c>
       <c r="G98">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="H98" t="str">
-        <v>2026-10-14T13:39:50.407Z</v>
+        <v>2026-10-14T13:40:03.191Z</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B99" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23457,38 +23457,38 @@
         <v>35</v>
       </c>
       <c r="H99" t="str">
-        <v>2026-10-13T16:19:36.490Z</v>
+        <v>2026-10-14T13:40:03.190Z</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>13-10-2026, 1:19:36 p. m.</v>
+        <v>14-10-2026, 10:40:03 a. m.</v>
       </c>
       <c r="B100" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>20261014_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-14_09-36hs_2967682966.xlsx</v>
       </c>
       <c r="C100" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D100">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E100">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F100">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G100">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H100" t="str">
-        <v>2026-10-13T16:19:36.488Z</v>
+        <v>2026-10-14T13:40:03.188Z</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>13-10-2026, 11:56:40 a. m.</v>
+        <v>14-10-2026, 10:39:50 a. m.</v>
       </c>
       <c r="B101" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23509,12 +23509,12 @@
         <v>35</v>
       </c>
       <c r="H101" t="str">
-        <v>2026-10-13T14:56:40.589Z</v>
+        <v>2026-10-14T13:39:50.407Z</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B102" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23526,177 +23526,177 @@
         <v>35</v>
       </c>
       <c r="E102">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F102">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G102">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H102" t="str">
-        <v>2026-10-13T14:44:42.285Z</v>
+        <v>2026-10-13T16:19:36.490Z</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 1:19:36 p. m.</v>
       </c>
       <c r="B103" t="str">
-        <v>picking-report (5).xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C103" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D103">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="E103">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F103">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G103">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="H103" t="str">
-        <v>2026-10-13T14:44:42.284Z</v>
+        <v>2026-10-13T16:19:36.488Z</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>13-10-2026, 11:44:42 a. m.</v>
+        <v>13-10-2026, 11:56:40 a. m.</v>
       </c>
       <c r="B104" t="str">
-        <v>ventas-report (5).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C104" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D104">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="E104">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F104">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G104">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H104" t="str">
-        <v>2026-10-13T14:44:42.280Z</v>
+        <v>2026-10-13T14:56:40.589Z</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B105" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C105" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D105">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="E105">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F105">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G105">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H105" t="str">
-        <v>2026-10-13T12:49:30.632Z</v>
+        <v>2026-10-13T14:44:42.285Z</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B106" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (5).xlsx</v>
       </c>
       <c r="C106" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D106">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E106">
+        <v>2</v>
+      </c>
+      <c r="F106">
+        <v>6</v>
+      </c>
+      <c r="G106">
         <v>0</v>
       </c>
-      <c r="F106">
-        <v>0</v>
-      </c>
-      <c r="G106">
-        <v>34</v>
-      </c>
       <c r="H106" t="str">
-        <v>2026-10-13T12:49:30.631Z</v>
+        <v>2026-10-13T14:44:42.284Z</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>13-10-2026, 9:49:30 a. m.</v>
+        <v>13-10-2026, 11:44:42 a. m.</v>
       </c>
       <c r="B107" t="str">
-        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
+        <v>ventas-report (5).xlsx</v>
       </c>
       <c r="C107" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D107">
-        <v>109</v>
+        <v>8</v>
       </c>
       <c r="E107">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F107">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G107">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H107" t="str">
-        <v>2026-10-13T12:49:30.629Z</v>
+        <v>2026-10-13T14:44:42.280Z</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>13-10-2026, 9:08:58 a. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B108" t="str">
-        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C108" t="str">
-        <v>Manual</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D108">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F108">
         <v>0</v>
       </c>
       <c r="G108">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H108" t="str">
-        <v>2026-10-13T12:08:58.547Z</v>
+        <v>2026-10-13T12:49:30.632Z</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B109" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23717,116 +23717,116 @@
         <v>34</v>
       </c>
       <c r="H109" t="str">
-        <v>2026-10-12T18:40:27.007Z</v>
+        <v>2026-10-13T12:49:30.631Z</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>12-10-2026, 3:40:27 p. m.</v>
+        <v>13-10-2026, 9:49:30 a. m.</v>
       </c>
       <c r="B110" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>20261013_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-13_08-03hs_2967682966 (1).xlsx</v>
       </c>
       <c r="C110" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D110">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F110">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G110">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H110" t="str">
-        <v>2026-10-12T18:40:27.006Z</v>
+        <v>2026-10-13T12:49:30.629Z</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>13-10-2026, 9:08:58 a. m.</v>
       </c>
       <c r="B111" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Agregado: VA-F001 -2 en Office (2026-10-13)</v>
       </c>
       <c r="C111" t="str">
-        <v>DropGO · generado</v>
+        <v>Manual</v>
       </c>
       <c r="D111">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E111">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F111">
         <v>0</v>
       </c>
       <c r="G111">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H111" t="str">
-        <v>2026-10-12T18:39:34.326Z</v>
+        <v>2026-10-13T12:08:58.547Z</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B112" t="str">
-        <v>picking-report (4).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C112" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D112">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="E112">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F112">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G112">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H112" t="str">
-        <v>2026-10-12T18:39:34.325Z</v>
+        <v>2026-10-12T18:40:27.007Z</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>12-10-2026, 3:39:34 p. m.</v>
+        <v>12-10-2026, 3:40:27 p. m.</v>
       </c>
       <c r="B113" t="str">
-        <v>ventas-report (4).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C113" t="str">
-        <v>DropGO · ventas</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D113">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E113">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F113">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G113">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H113" t="str">
-        <v>2026-10-12T18:39:34.319Z</v>
+        <v>2026-10-12T18:40:27.006Z</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>12-10-2026, 3:39:18 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B114" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23835,10 +23835,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D114">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E114">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F114">
         <v>0</v>
@@ -23847,116 +23847,116 @@
         <v>25</v>
       </c>
       <c r="H114" t="str">
-        <v>2026-10-12T18:39:18.385Z</v>
+        <v>2026-10-12T18:39:34.326Z</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>12-10-2026, 12:05:40 p. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B115" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (4).xlsx</v>
       </c>
       <c r="C115" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D115">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E115">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F115">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G115">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H115" t="str">
-        <v>2026-10-12T15:05:40.188Z</v>
+        <v>2026-10-12T18:39:34.325Z</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:34 p. m.</v>
       </c>
       <c r="B116" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>ventas-report (4).xlsx</v>
       </c>
       <c r="C116" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D116">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E116">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F116">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G116">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H116" t="str">
-        <v>2026-10-12T14:26:19.514Z</v>
+        <v>2026-10-12T18:39:34.319Z</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>12-10-2026, 11:26:19 a. m.</v>
+        <v>12-10-2026, 3:39:18 p. m.</v>
       </c>
       <c r="B117" t="str">
-        <v>orders_export (6).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C117" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D117">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F117">
         <v>0</v>
       </c>
       <c r="G117">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H117" t="str">
-        <v>2026-10-12T14:26:19.513Z</v>
+        <v>2026-10-12T18:39:18.385Z</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 12:05:40 p. m.</v>
       </c>
       <c r="B118" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C118" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D118">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E118">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F118">
         <v>0</v>
       </c>
       <c r="G118">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H118" t="str">
-        <v>2026-10-12T14:24:55.059Z</v>
+        <v>2026-10-12T15:05:40.188Z</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B119" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -23977,64 +23977,64 @@
         <v>25</v>
       </c>
       <c r="H119" t="str">
-        <v>2026-10-12T14:24:55.058Z</v>
+        <v>2026-10-12T14:26:19.514Z</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>12-10-2026, 11:24:55 a. m.</v>
+        <v>12-10-2026, 11:26:19 a. m.</v>
       </c>
       <c r="B120" t="str">
-        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
+        <v>orders_export (6).csv</v>
       </c>
       <c r="C120" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D120">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E120">
         <v>4</v>
       </c>
       <c r="F120">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G120">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H120" t="str">
-        <v>2026-10-12T14:24:55.057Z</v>
+        <v>2026-10-12T14:26:19.513Z</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>12-10-2026, 11:24:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B121" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C121" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D121">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E121">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F121">
         <v>0</v>
       </c>
       <c r="G121">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="H121" t="str">
-        <v>2026-10-12T14:24:00.106Z</v>
+        <v>2026-10-12T14:24:55.059Z</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B122" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24046,73 +24046,73 @@
         <v>25</v>
       </c>
       <c r="E122">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F122">
         <v>0</v>
       </c>
       <c r="G122">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H122" t="str">
-        <v>2026-10-09T14:54:00.353Z</v>
+        <v>2026-10-12T14:24:55.058Z</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:55 a. m.</v>
       </c>
       <c r="B123" t="str">
-        <v>picking-report (3).xlsx</v>
+        <v>20261012_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-12_10-24hs_2967682966.xlsx</v>
       </c>
       <c r="C123" t="str">
-        <v>DropGO · picking</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D123">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E123">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F123">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G123">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H123" t="str">
-        <v>2026-10-09T14:54:00.352Z</v>
+        <v>2026-10-12T14:24:55.057Z</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>09-10-2026, 11:54:00 a. m.</v>
+        <v>12-10-2026, 11:24:00 a. m.</v>
       </c>
       <c r="B124" t="str">
-        <v>ventas-report (3).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C124" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D124">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E124">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F124">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G124">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H124" t="str">
-        <v>2026-10-09T14:54:00.347Z</v>
+        <v>2026-10-12T14:24:00.106Z</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>09-10-2026, 11:50:59 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B125" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24121,10 +24121,10 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D125">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E125">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F125">
         <v>0</v>
@@ -24133,64 +24133,64 @@
         <v>21</v>
       </c>
       <c r="H125" t="str">
-        <v>2026-10-09T14:50:59.695Z</v>
+        <v>2026-10-09T14:54:00.353Z</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B126" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (3).xlsx</v>
       </c>
       <c r="C126" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D126">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E126">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F126">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G126">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H126" t="str">
-        <v>2026-10-09T14:28:16.404Z</v>
+        <v>2026-10-09T14:54:00.352Z</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>09-10-2026, 11:28:16 a. m.</v>
+        <v>09-10-2026, 11:54:00 a. m.</v>
       </c>
       <c r="B127" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>ventas-report (3).xlsx</v>
       </c>
       <c r="C127" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D127">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E127">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G127">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H127" t="str">
-        <v>2026-10-09T14:28:16.403Z</v>
+        <v>2026-10-09T14:54:00.347Z</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>09-10-2026, 11:28:07 a. m.</v>
+        <v>09-10-2026, 11:50:59 a. m.</v>
       </c>
       <c r="B128" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24211,12 +24211,12 @@
         <v>21</v>
       </c>
       <c r="H128" t="str">
-        <v>2026-10-09T14:28:07.531Z</v>
+        <v>2026-10-09T14:50:59.695Z</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B129" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24237,12 +24237,12 @@
         <v>21</v>
       </c>
       <c r="H129" t="str">
-        <v>2026-10-09T14:26:45.497Z</v>
+        <v>2026-10-09T14:28:16.404Z</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:16 a. m.</v>
       </c>
       <c r="B130" t="str">
         <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
@@ -24263,21 +24263,21 @@
         <v>19</v>
       </c>
       <c r="H130" t="str">
-        <v>2026-10-09T14:26:45.495Z</v>
+        <v>2026-10-09T14:28:16.403Z</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>09-10-2026, 11:26:45 a. m.</v>
+        <v>09-10-2026, 11:28:07 a. m.</v>
       </c>
       <c r="B131" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C131" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D131">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E131">
         <v>0</v>
@@ -24286,50 +24286,50 @@
         <v>0</v>
       </c>
       <c r="G131">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H131" t="str">
-        <v>2026-10-09T14:26:45.477Z</v>
+        <v>2026-10-09T14:28:07.531Z</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B132" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C132" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D132">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E132">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F132">
         <v>0</v>
       </c>
       <c r="G132">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H132" t="str">
-        <v>2026-10-09T14:25:43.607Z</v>
+        <v>2026-10-09T14:26:45.497Z</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B133" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C133" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D133">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E133">
         <v>0</v>
@@ -24338,36 +24338,36 @@
         <v>0</v>
       </c>
       <c r="G133">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H133" t="str">
-        <v>2026-10-09T14:25:43.606Z</v>
+        <v>2026-10-09T14:26:45.495Z</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>09-10-2026, 11:25:43 a. m.</v>
+        <v>09-10-2026, 11:26:45 a. m.</v>
       </c>
       <c r="B134" t="str">
-        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C134" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D134">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E134">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F134">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G134">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H134" t="str">
-        <v>2026-10-09T14:25:43.605Z</v>
+        <v>2026-10-09T14:26:45.477Z</v>
       </c>
     </row>
     <row r="135">
@@ -24375,30 +24375,30 @@
         <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B135" t="str">
-        <v>orders_export (5).csv</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C135" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D135">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="E135">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F135">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G135">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="H135" t="str">
-        <v>2026-10-09T14:25:43.580Z</v>
+        <v>2026-10-09T14:25:43.607Z</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>09-10-2026, 11:23:53 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B136" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24419,111 +24419,111 @@
         <v>21</v>
       </c>
       <c r="H136" t="str">
-        <v>2026-10-09T14:23:53.263Z</v>
+        <v>2026-10-09T14:25:43.606Z</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>08-10-2026, 9:14:25 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B137" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261009_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-09_12-25hs_2967682966.xlsx</v>
       </c>
       <c r="C137" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D137">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E137">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F137">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G137">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H137" t="str">
-        <v>2026-10-08T12:14:25.917Z</v>
+        <v>2026-10-09T14:25:43.605Z</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:25:43 a. m.</v>
       </c>
       <c r="B138" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (5).csv</v>
       </c>
       <c r="C138" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D138">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E138">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F138">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G138">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H138" t="str">
-        <v>2026-10-08T11:22:18.060Z</v>
+        <v>2026-10-09T14:25:43.580Z</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>09-10-2026, 11:23:53 a. m.</v>
       </c>
       <c r="B139" t="str">
-        <v>orders_export (4).csv</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C139" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D139">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E139">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F139">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G139">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H139" t="str">
-        <v>2026-10-08T11:22:18.059Z</v>
+        <v>2026-10-09T14:23:53.263Z</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>08-10-2026, 8:22:18 a. m.</v>
+        <v>08-10-2026, 9:14:25 a. m.</v>
       </c>
       <c r="B140" t="str">
-        <v>ventas-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C140" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D140">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E140">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F140">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G140">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H140" t="str">
-        <v>2026-10-08T11:22:18.042Z</v>
+        <v>2026-10-08T12:14:25.917Z</v>
       </c>
     </row>
     <row r="141">
@@ -24531,108 +24531,108 @@
         <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B141" t="str">
-        <v>picking-report (2).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C141" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D141">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E141">
         <v>2</v>
       </c>
       <c r="F141">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G141">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H141" t="str">
-        <v>2026-10-08T11:22:18.032Z</v>
+        <v>2026-10-08T11:22:18.060Z</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>08-10-2026, 8:18:16 a. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B142" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>orders_export (4).csv</v>
       </c>
       <c r="C142" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D142">
         <v>19</v>
       </c>
       <c r="E142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F142">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G142">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H142" t="str">
-        <v>2026-10-08T11:18:16.488Z</v>
+        <v>2026-10-08T11:22:18.059Z</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B143" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
+        <v>ventas-report (2).xlsx</v>
       </c>
       <c r="C143" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D143">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="E143">
         <v>2</v>
       </c>
       <c r="F143">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G143">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H143" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.042Z</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>07-10-2026, 8:20:51 p. m.</v>
+        <v>08-10-2026, 8:22:18 a. m.</v>
       </c>
       <c r="B144" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>picking-report (2).xlsx</v>
       </c>
       <c r="C144" t="str">
-        <v>DropGO · generado</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D144">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E144">
+        <v>2</v>
+      </c>
+      <c r="F144">
+        <v>1</v>
+      </c>
+      <c r="G144">
         <v>0</v>
       </c>
-      <c r="F144">
-        <v>0</v>
-      </c>
-      <c r="G144">
-        <v>19</v>
-      </c>
       <c r="H144" t="str">
-        <v>2026-10-07T23:20:51.545Z</v>
+        <v>2026-10-08T11:22:18.032Z</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>07-10-2026, 8:20:41 p. m.</v>
+        <v>08-10-2026, 8:18:16 a. m.</v>
       </c>
       <c r="B145" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24653,12 +24653,12 @@
         <v>19</v>
       </c>
       <c r="H145" t="str">
-        <v>2026-10-07T23:20:41.390Z</v>
+        <v>2026-10-08T11:18:16.488Z</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B146" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24679,38 +24679,38 @@
         <v>19</v>
       </c>
       <c r="H146" t="str">
-        <v>2026-10-07T17:47:17.199Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>07-10-2026, 2:47:17 p. m.</v>
+        <v>07-10-2026, 8:20:51 p. m.</v>
       </c>
       <c r="B147" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_18-03hs_2967682966.xlsx</v>
       </c>
       <c r="C147" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D147">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E147">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F147">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G147">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H147" t="str">
-        <v>2026-10-07T17:47:17.198Z</v>
+        <v>2026-10-07T23:20:51.545Z</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>07-10-2026, 2:46:47 p. m.</v>
+        <v>07-10-2026, 8:20:41 p. m.</v>
       </c>
       <c r="B148" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24731,12 +24731,12 @@
         <v>19</v>
       </c>
       <c r="H148" t="str">
-        <v>2026-10-07T17:46:47.954Z</v>
+        <v>2026-10-07T23:20:41.390Z</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>07-10-2026, 2:44:00 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B149" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24757,64 +24757,64 @@
         <v>19</v>
       </c>
       <c r="H149" t="str">
-        <v>2026-10-07T17:44:00.660Z</v>
+        <v>2026-10-07T17:47:17.199Z</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>07-10-2026, 2:27:43 p. m.</v>
+        <v>07-10-2026, 2:47:17 p. m.</v>
       </c>
       <c r="B150" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
       </c>
       <c r="C150" t="str">
-        <v>DropGO · generado</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D150">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E150">
         <v>0</v>
       </c>
       <c r="F150">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G150">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="H150" t="str">
-        <v>2026-10-07T17:27:43.517Z</v>
+        <v>2026-10-07T17:47:17.198Z</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:46:47 p. m.</v>
       </c>
       <c r="B151" t="str">
-        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C151" t="str">
-        <v>Full ML · generado</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D151">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E151">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F151">
         <v>0</v>
       </c>
       <c r="G151">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H151" t="str">
-        <v>2026-10-07T17:26:50.382Z</v>
+        <v>2026-10-07T17:46:47.954Z</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>07-10-2026, 2:26:50 p. m.</v>
+        <v>07-10-2026, 2:44:00 p. m.</v>
       </c>
       <c r="B152" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24826,30 +24826,30 @@
         <v>19</v>
       </c>
       <c r="E152">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F152">
         <v>0</v>
       </c>
       <c r="G152">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H152" t="str">
-        <v>2026-10-07T17:26:50.380Z</v>
+        <v>2026-10-07T17:44:00.660Z</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:27:43 p. m.</v>
       </c>
       <c r="B153" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C153" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D153">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="E153">
         <v>0</v>
@@ -24858,41 +24858,41 @@
         <v>0</v>
       </c>
       <c r="G153">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="H153" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:27:43.517Z</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>07-10-2026, 1:25:42 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B154" t="str">
-        <v>Movimientos DropGO (desde ventas + picking)</v>
+        <v>Salidas Full ML (desde ventas FULL de Mercado Libre)</v>
       </c>
       <c r="C154" t="str">
-        <v>DropGO · generado</v>
+        <v>Full ML · generado</v>
       </c>
       <c r="D154">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E154">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F154">
         <v>0</v>
       </c>
       <c r="G154">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H154" t="str">
-        <v>2026-10-07T16:25:42.540Z</v>
+        <v>2026-10-07T17:26:50.382Z</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 2:26:50 p. m.</v>
       </c>
       <c r="B155" t="str">
         <v>Movimientos DropGO (desde ventas + picking)</v>
@@ -24901,71 +24901,71 @@
         <v>DropGO · generado</v>
       </c>
       <c r="D155">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E155">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F155">
         <v>0</v>
       </c>
       <c r="G155">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H155" t="str">
-        <v>2026-10-07T16:25:12.953Z</v>
+        <v>2026-10-07T17:26:50.380Z</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B156" t="str">
-        <v>picking-report (1).xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C156" t="str">
-        <v>DropGO · picking</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D156">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E156">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F156">
         <v>0</v>
       </c>
       <c r="G156">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H156" t="str">
-        <v>2026-10-07T16:25:12.950Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>07-10-2026, 1:25:12 p. m.</v>
+        <v>07-10-2026, 1:25:42 p. m.</v>
       </c>
       <c r="B157" t="str">
-        <v>orders_export (3).csv</v>
+        <v>ventas_por_canal_y_mes.xlsx</v>
       </c>
       <c r="C157" t="str">
-        <v>Ventas Shopify (Varin)</v>
+        <v>Ventas por canal y mes</v>
       </c>
       <c r="D157">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="E157">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F157">
         <v>0</v>
       </c>
       <c r="G157">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="H157" t="str">
-        <v>2026-10-07T16:25:12.939Z</v>
+        <v>2026-10-07T16:25:42.540Z</v>
       </c>
     </row>
     <row r="158">
@@ -24973,25 +24973,25 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B158" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>Movimientos DropGO (desde ventas + picking)</v>
       </c>
       <c r="C158" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>DropGO · generado</v>
       </c>
       <c r="D158">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E158">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F158">
         <v>0</v>
       </c>
       <c r="G158">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H158" t="str">
-        <v>2026-10-07T16:25:12.924Z</v>
+        <v>2026-10-07T16:25:12.953Z</v>
       </c>
     </row>
     <row r="159">
@@ -24999,10 +24999,10 @@
         <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B159" t="str">
-        <v>ventas-report (1).xlsx</v>
+        <v>picking-report (1).xlsx</v>
       </c>
       <c r="C159" t="str">
-        <v>DropGO · ventas</v>
+        <v>DropGO · picking</v>
       </c>
       <c r="D159">
         <v>19</v>
@@ -25017,142 +25017,220 @@
         <v>0</v>
       </c>
       <c r="H159" t="str">
-        <v>2026-10-07T16:25:12.851Z</v>
+        <v>2026-10-07T16:25:12.950Z</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>07-10-2026, 1:10:27 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B160" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
+        <v>orders_export (3).csv</v>
       </c>
       <c r="C160" t="str">
-        <v>Ventas Mercado Libre</v>
+        <v>Ventas Shopify (Varin)</v>
       </c>
       <c r="D160">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="E160">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F160">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G160">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="H160" t="str">
-        <v>2026-10-07T16:10:27.561Z</v>
+        <v>2026-10-07T16:25:12.939Z</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>07-10-2026, 12:20:36 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B161" t="str">
-        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C161" t="str">
         <v>Ventas Mercado Libre</v>
       </c>
       <c r="D161">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E161">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F161">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G161">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H161" t="str">
-        <v>2026-10-07T15:20:36.001Z</v>
+        <v>2026-10-07T16:25:12.924Z</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>07-10-2026, 12:20:35 p. m.</v>
+        <v>07-10-2026, 1:25:12 p. m.</v>
       </c>
       <c r="B162" t="str">
-        <v>varin_respaldo_2026-10-07.xlsx</v>
+        <v>ventas-report (1).xlsx</v>
       </c>
       <c r="C162" t="str">
-        <v>Respaldo</v>
+        <v>DropGO · ventas</v>
       </c>
       <c r="D162">
-        <v>322</v>
+        <v>19</v>
       </c>
       <c r="E162">
-        <v>190</v>
+        <v>19</v>
       </c>
       <c r="F162">
         <v>0</v>
       </c>
       <c r="G162">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="H162" t="str">
-        <v>2026-10-07T15:20:35.967Z</v>
+        <v>2026-10-07T16:25:12.851Z</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>07-10-2026, 12:20:08 p. m.</v>
+        <v>07-10-2026, 1:10:27 p. m.</v>
       </c>
       <c r="B163" t="str">
-        <v>ventas_por_canal_y_mes.xlsx</v>
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_12-03hs_2967682966.xlsx</v>
       </c>
       <c r="C163" t="str">
-        <v>Ventas por canal y mes</v>
+        <v>Ventas Mercado Libre</v>
       </c>
       <c r="D163">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="E163">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="F163">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G163">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="H163" t="str">
-        <v>2026-10-07T15:20:08.547Z</v>
+        <v>2026-10-07T16:10:27.561Z</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
+        <v>07-10-2026, 12:20:36 p. m.</v>
+      </c>
+      <c r="B164" t="str">
+        <v>20261007_Ventas_CL_Mercado_Libre_y_Mercado_Shops_2026-10-07_07-59hs_2967682966.xlsx</v>
+      </c>
+      <c r="C164" t="str">
+        <v>Ventas Mercado Libre</v>
+      </c>
+      <c r="D164">
+        <v>92</v>
+      </c>
+      <c r="E164">
+        <v>1</v>
+      </c>
+      <c r="F164">
+        <v>5</v>
+      </c>
+      <c r="G164">
+        <v>86</v>
+      </c>
+      <c r="H164" t="str">
+        <v>2026-10-07T15:20:36.001Z</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>07-10-2026, 12:20:35 p. m.</v>
+      </c>
+      <c r="B165" t="str">
+        <v>varin_respaldo_2026-10-07.xlsx</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Respaldo</v>
+      </c>
+      <c r="D165">
+        <v>322</v>
+      </c>
+      <c r="E165">
+        <v>190</v>
+      </c>
+      <c r="F165">
+        <v>0</v>
+      </c>
+      <c r="G165">
+        <v>132</v>
+      </c>
+      <c r="H165" t="str">
+        <v>2026-10-07T15:20:35.967Z</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
         <v>07-10-2026, 12:20:08 p. m.</v>
       </c>
-      <c r="B164" t="str">
+      <c r="B166" t="str">
+        <v>ventas_por_canal_y_mes.xlsx</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Ventas por canal y mes</v>
+      </c>
+      <c r="D166">
+        <v>118</v>
+      </c>
+      <c r="E166">
+        <v>118</v>
+      </c>
+      <c r="F166">
+        <v>0</v>
+      </c>
+      <c r="G166">
+        <v>0</v>
+      </c>
+      <c r="H166" t="str">
+        <v>2026-10-07T15:20:08.547Z</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>07-10-2026, 12:20:08 p. m.</v>
+      </c>
+      <c r="B167" t="str">
         <v>Varin_Movimientos_DropGO_2026-10-01_al_2026-10-06.xlsx</v>
       </c>
-      <c r="C164" t="str">
+      <c r="C167" t="str">
         <v>Movimientos DropGO</v>
       </c>
-      <c r="D164">
+      <c r="D167">
         <v>14</v>
       </c>
-      <c r="E164">
+      <c r="E167">
         <v>14</v>
       </c>
-      <c r="F164">
+      <c r="F167">
         <v>0</v>
       </c>
-      <c r="G164">
+      <c r="G167">
         <v>0</v>
       </c>
-      <c r="H164" t="str">
+      <c r="H167" t="str">
         <v>2026-10-07T15:20:08.525Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H164"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H167"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -28945,7 +29023,7 @@
         <v>Generado</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-30T11:31:20.673Z</v>
+        <v>2026-10-30T11:40:17.598Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>